<commit_message>
Update ALLW XLSX 2026-10-12
</commit_message>
<xml_diff>
--- a/latest/allw-latest.xlsx
+++ b/latest/allw-latest.xlsx
@@ -192,7 +192,7 @@
     <t>ALLW</t>
   </si>
   <si>
-    <t>As of 08-Oct-2026</t>
+    <t>As of 09-Oct-2026</t>
   </si>
   <si>
     <t>Name</t>
@@ -414,6 +414,24 @@
     <t>ADI3917X6</t>
   </si>
   <si>
+    <t>AUST 10Y BOND FUT DEC26</t>
+  </si>
+  <si>
+    <t>XMZ6</t>
+  </si>
+  <si>
+    <t>ADI3BDHZ1</t>
+  </si>
+  <si>
+    <t>SPI 200 FUTURES   DEC26</t>
+  </si>
+  <si>
+    <t>XPZ6</t>
+  </si>
+  <si>
+    <t>ADI391SG0</t>
+  </si>
+  <si>
     <t>CANADIAN DOLLAR</t>
   </si>
   <si>
@@ -432,24 +450,6 @@
     <t>999JPYZ94</t>
   </si>
   <si>
-    <t>AUST 10Y BOND FUT DEC26</t>
-  </si>
-  <si>
-    <t>XMZ6</t>
-  </si>
-  <si>
-    <t>ADI3BDHZ1</t>
-  </si>
-  <si>
-    <t>SPI 200 FUTURES   DEC26</t>
-  </si>
-  <si>
-    <t>XPZ6</t>
-  </si>
-  <si>
-    <t>ADI391SG0</t>
-  </si>
-  <si>
     <t>FTSE 100 IDX FUT  DEC26</t>
   </si>
   <si>
@@ -459,6 +459,15 @@
     <t>ADI38QPG9</t>
   </si>
   <si>
+    <t>EURO STOXX 50     DEC26</t>
+  </si>
+  <si>
+    <t>VGZ6</t>
+  </si>
+  <si>
+    <t>ADI2VHXS0</t>
+  </si>
+  <si>
     <t>EURO-BUND FUTURE  DEC26</t>
   </si>
   <si>
@@ -466,15 +475,6 @@
   </si>
   <si>
     <t>ADI39K4N9</t>
-  </si>
-  <si>
-    <t>EURO STOXX 50     DEC26</t>
-  </si>
-  <si>
-    <t>VGZ6</t>
-  </si>
-  <si>
-    <t>ADI2VHXS0</t>
   </si>
   <si>
     <t>LONG GILT FUTURE  DEC26</t>
@@ -960,43 +960,43 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
@@ -1479,16 +1479,16 @@
         <v>22</v>
       </c>
       <c r="D6" t="n" s="19">
-        <v>33.855801</v>
+        <v>33.794871</v>
       </c>
       <c r="E6" t="n" s="20">
-        <v>6.1125512293E8</v>
+        <v>6.1390035639E8</v>
       </c>
       <c r="F6" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G6" t="n" s="21">
-        <v>6.1125512293E8</v>
+        <v>6.1390035639E8</v>
       </c>
     </row>
     <row r="7">
@@ -1502,10 +1502,10 @@
         <v>25</v>
       </c>
       <c r="D7" t="n" s="22">
-        <v>13.769748</v>
+        <v>13.771398</v>
       </c>
       <c r="E7" t="n" s="23">
-        <v>2.4860816806E8</v>
+        <v>2.5016418712E8</v>
       </c>
       <c r="F7" t="s" s="18">
         <v>21</v>
@@ -1525,16 +1525,16 @@
         <v>27</v>
       </c>
       <c r="D8" t="n" s="25">
-        <v>5.17863</v>
+        <v>5.001418</v>
       </c>
       <c r="E8" t="n" s="26">
-        <v>9.349842935E7</v>
+        <v>9.085319589E7</v>
       </c>
       <c r="F8" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G8" t="n" s="27">
-        <v>9.349842935E7</v>
+        <v>9.085319589E7</v>
       </c>
     </row>
     <row r="9">
@@ -1548,10 +1548,10 @@
         <v>29</v>
       </c>
       <c r="D9" t="n" s="28">
-        <v>5.003381</v>
+        <v>4.97475</v>
       </c>
       <c r="E9" t="n" s="29">
-        <v>9.033437242E7</v>
+        <v>9.036876634E7</v>
       </c>
       <c r="F9" t="s" s="18">
         <v>21</v>
@@ -1571,10 +1571,10 @@
         <v>32</v>
       </c>
       <c r="D10" t="n" s="31">
-        <v>4.317412</v>
+        <v>4.347698</v>
       </c>
       <c r="E10" t="n" s="32">
-        <v>7.7949431E7</v>
+        <v>7.8978067E7</v>
       </c>
       <c r="F10" t="s" s="18">
         <v>21</v>
@@ -1594,16 +1594,16 @@
         <v>34</v>
       </c>
       <c r="D11" t="n" s="34">
-        <v>4.294966</v>
+        <v>4.260765</v>
       </c>
       <c r="E11" t="n" s="35">
-        <v>7.754417464E7</v>
+        <v>7.739888344E7</v>
       </c>
       <c r="F11" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G11" t="n" s="36">
-        <v>8.3591497E7</v>
+        <v>8.360033E7</v>
       </c>
     </row>
     <row r="12">
@@ -1617,16 +1617,16 @@
         <v>36</v>
       </c>
       <c r="D12" t="n" s="37">
-        <v>4.2014</v>
+        <v>4.167787</v>
       </c>
       <c r="E12" t="n" s="38">
-        <v>7.585487099E7</v>
+        <v>7.570988719E7</v>
       </c>
       <c r="F12" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G12" t="n" s="39">
-        <v>8.250174E7</v>
+        <v>8.2510562E7</v>
       </c>
     </row>
     <row r="13">
@@ -1640,16 +1640,16 @@
         <v>38</v>
       </c>
       <c r="D13" t="n" s="40">
-        <v>4.017985</v>
+        <v>3.986661</v>
       </c>
       <c r="E13" t="n" s="41">
-        <v>7.254337486E7</v>
+        <v>7.241964088E7</v>
       </c>
       <c r="F13" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G13" t="n" s="42">
-        <v>7.6366157E7</v>
+        <v>7.6374088E7</v>
       </c>
     </row>
     <row r="14">
@@ -1663,16 +1663,16 @@
         <v>40</v>
       </c>
       <c r="D14" t="n" s="43">
-        <v>3.707237</v>
+        <v>3.679182</v>
       </c>
       <c r="E14" t="n" s="44">
-        <v>6.693291437E7</v>
+        <v>6.683414795E7</v>
       </c>
       <c r="F14" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G14" t="n" s="45">
-        <v>7.11859995E7</v>
+        <v>7.119335025E7</v>
       </c>
     </row>
     <row r="15">
@@ -1686,16 +1686,16 @@
         <v>42</v>
       </c>
       <c r="D15" t="n" s="46">
-        <v>3.5342</v>
+        <v>3.506829</v>
       </c>
       <c r="E15" t="n" s="47">
-        <v>6.380878581E7</v>
+        <v>6.370327265E7</v>
       </c>
       <c r="F15" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G15" t="n" s="48">
-        <v>6.824041455E7</v>
+        <v>6.82473176E7</v>
       </c>
     </row>
     <row r="16">
@@ -1709,10 +1709,10 @@
         <v>45</v>
       </c>
       <c r="D16" t="n" s="49">
-        <v>3.300669</v>
+        <v>3.343982</v>
       </c>
       <c r="E16" t="n" s="50">
-        <v>5.959246552E7</v>
+        <v>6.074506861E7</v>
       </c>
       <c r="F16" t="s" s="18">
         <v>21</v>
@@ -1732,16 +1732,16 @@
         <v>47</v>
       </c>
       <c r="D17" t="n" s="52">
-        <v>2.538909</v>
+        <v>2.518836</v>
       </c>
       <c r="E17" t="n" s="53">
-        <v>4.583915393E7</v>
+        <v>4.575589081E7</v>
       </c>
       <c r="F17" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G17" t="n" s="54">
-        <v>4.7841586E7</v>
+        <v>4.7846366E7</v>
       </c>
     </row>
     <row r="18">
@@ -1755,16 +1755,16 @@
         <v>49</v>
       </c>
       <c r="D18" t="n" s="55">
-        <v>1.476568</v>
+        <v>1.467713</v>
       </c>
       <c r="E18" t="n" s="56">
-        <v>2.665894037E7</v>
+        <v>2.666172852E7</v>
       </c>
       <c r="F18" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G18" t="n" s="57">
-        <v>3.55832463E7</v>
+        <v>3.55869678E7</v>
       </c>
     </row>
     <row r="19">
@@ -1778,16 +1778,16 @@
         <v>51</v>
       </c>
       <c r="D19" t="n" s="58">
-        <v>1.303053</v>
+        <v>1.296206</v>
       </c>
       <c r="E19" t="n" s="59">
-        <v>2.352619315E7</v>
+        <v>2.354621363E7</v>
       </c>
       <c r="F19" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G19" t="n" s="60">
-        <v>3.62464218E7</v>
+        <v>3.62499967E7</v>
       </c>
     </row>
     <row r="20">
@@ -1801,16 +1801,16 @@
         <v>53</v>
       </c>
       <c r="D20" t="n" s="61">
-        <v>1.221116</v>
+        <v>1.214687</v>
       </c>
       <c r="E20" t="n" s="62">
-        <v>2.204684211E7</v>
+        <v>2.20653792E7</v>
       </c>
       <c r="F20" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G20" t="n" s="63">
-        <v>2.6832069E7</v>
+        <v>2.68348553E7</v>
       </c>
     </row>
     <row r="21">
@@ -1824,16 +1824,16 @@
         <v>55</v>
       </c>
       <c r="D21" t="n" s="64">
-        <v>1.149993</v>
+        <v>1.143693</v>
       </c>
       <c r="E21" t="n" s="65">
-        <v>2.076274005E7</v>
+        <v>2.077574931E7</v>
       </c>
       <c r="F21" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G21" t="n" s="66">
-        <v>2.66022445E7</v>
+        <v>2.660493125E7</v>
       </c>
     </row>
     <row r="22">
@@ -1847,16 +1847,16 @@
         <v>57</v>
       </c>
       <c r="D22" t="n" s="67">
-        <v>1.125819</v>
+        <v>1.119644</v>
       </c>
       <c r="E22" t="n" s="68">
-        <v>2.032627949E7</v>
+        <v>2.033888755E7</v>
       </c>
       <c r="F22" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G22" t="n" s="69">
-        <v>2.475336E7</v>
+        <v>2.475576E7</v>
       </c>
     </row>
     <row r="23">
@@ -1870,16 +1870,16 @@
         <v>59</v>
       </c>
       <c r="D23" t="n" s="70">
-        <v>1.097088</v>
+        <v>1.09084</v>
       </c>
       <c r="E23" t="n" s="71">
-        <v>1.98075624E7</v>
+        <v>1.981563561E7</v>
       </c>
       <c r="F23" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G23" t="n" s="72">
-        <v>2.82248532E7</v>
+        <v>2.82277152E7</v>
       </c>
     </row>
     <row r="24">
@@ -1893,16 +1893,16 @@
         <v>61</v>
       </c>
       <c r="D24" t="n" s="73">
-        <v>0.940844</v>
+        <v>0.93577</v>
       </c>
       <c r="E24" t="n" s="74">
-        <v>1.698662711E7</v>
+        <v>1.699872616E7</v>
       </c>
       <c r="F24" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G24" t="n" s="75">
-        <v>2.5076127E7</v>
+        <v>2.5078803E7</v>
       </c>
     </row>
     <row r="25">
@@ -1916,16 +1916,16 @@
         <v>63</v>
       </c>
       <c r="D25" t="n" s="76">
-        <v>0.92555</v>
+        <v>0.920132</v>
       </c>
       <c r="E25" t="n" s="77">
-        <v>1.67104881E7</v>
+        <v>1.671465315E7</v>
       </c>
       <c r="F25" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G25" t="n" s="78">
-        <v>2.49920253E7</v>
+        <v>2.49946038E7</v>
       </c>
     </row>
     <row r="26">
@@ -1939,16 +1939,16 @@
         <v>65</v>
       </c>
       <c r="D26" t="n" s="79">
-        <v>0.877857</v>
+        <v>0.873151</v>
       </c>
       <c r="E26" t="n" s="80">
-        <v>1.584940776E7</v>
+        <v>1.586120604E7</v>
       </c>
       <c r="F26" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G26" t="n" s="81">
-        <v>2.4855724E7</v>
+        <v>2.4858237E7</v>
       </c>
     </row>
     <row r="27">
@@ -1962,16 +1962,16 @@
         <v>67</v>
       </c>
       <c r="D27" t="n" s="82">
-        <v>0.726692</v>
+        <v>0.722883</v>
       </c>
       <c r="E27" t="n" s="83">
-        <v>1.312018595E7</v>
+        <v>1.313152551E7</v>
       </c>
       <c r="F27" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G27" t="n" s="84">
-        <v>1.95806548E7</v>
+        <v>1.95827368E7</v>
       </c>
     </row>
     <row r="28">
@@ -1985,16 +1985,16 @@
         <v>69</v>
       </c>
       <c r="D28" t="n" s="85">
-        <v>0.712467</v>
+        <v>0.709079</v>
       </c>
       <c r="E28" t="n" s="86">
-        <v>1.286335495E7</v>
+        <v>1.288076099E7</v>
       </c>
       <c r="F28" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G28" t="n" s="87">
-        <v>2.8458012E7</v>
+        <v>2.8460856E7</v>
       </c>
     </row>
     <row r="29">
@@ -2008,16 +2008,16 @@
         <v>71</v>
       </c>
       <c r="D29" t="n" s="88">
-        <v>0.706058</v>
+        <v>0.702621</v>
       </c>
       <c r="E29" t="n" s="89">
-        <v>1.274763638E7</v>
+        <v>1.276345534E7</v>
       </c>
       <c r="F29" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G29" t="n" s="90">
-        <v>2.55022461E7</v>
+        <v>2.55049922E7</v>
       </c>
     </row>
     <row r="30">
@@ -2031,16 +2031,16 @@
         <v>73</v>
       </c>
       <c r="D30" t="n" s="91">
-        <v>0.595577</v>
+        <v>0.592872</v>
       </c>
       <c r="E30" t="n" s="92">
-        <v>1.075294915E7</v>
+        <v>1.076981087E7</v>
       </c>
       <c r="F30" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G30" t="n" s="93">
-        <v>2.30713236E7</v>
+        <v>2.30736597E7</v>
       </c>
     </row>
     <row r="31">
@@ -2054,16 +2054,16 @@
         <v>75</v>
       </c>
       <c r="D31" t="n" s="94">
-        <v>0.5652</v>
+        <v>0.562215</v>
       </c>
       <c r="E31" t="n" s="95">
-        <v>1.020450052E7</v>
+        <v>1.021291397E7</v>
       </c>
       <c r="F31" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G31" t="n" s="96">
-        <v>1.585935E7</v>
+        <v>1.5860871E7</v>
       </c>
     </row>
     <row r="32">
@@ -2077,16 +2077,16 @@
         <v>77</v>
       </c>
       <c r="D32" t="n" s="97">
-        <v>0.552779</v>
+        <v>0.549956</v>
       </c>
       <c r="E32" t="n" s="98">
-        <v>9980234.68</v>
+        <v>9990222.12</v>
       </c>
       <c r="F32" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G32" t="n" s="99">
-        <v>1.577415625E7</v>
+        <v>1.577581875E7</v>
       </c>
     </row>
     <row r="33">
@@ -2100,10 +2100,10 @@
         <v>21</v>
       </c>
       <c r="D33" t="n" s="100">
-        <v>0.319683</v>
+        <v>0.367568</v>
       </c>
       <c r="E33" t="n" s="101">
-        <v>5771768.83</v>
+        <v>6677053.59</v>
       </c>
       <c r="F33" t="n" s="102">
         <v>4.1426456199E8</v>
@@ -2123,10 +2123,10 @@
         <v>80</v>
       </c>
       <c r="D34" t="n" s="104">
-        <v>0.26988</v>
+        <v>0.267947</v>
       </c>
       <c r="E34" t="n" s="105">
-        <v>4872600.58</v>
+        <v>4867385.25</v>
       </c>
       <c r="F34" t="s" s="18">
         <v>21</v>
@@ -2146,10 +2146,10 @@
         <v>82</v>
       </c>
       <c r="D35" t="n" s="107">
-        <v>0.14896</v>
+        <v>0.14804</v>
       </c>
       <c r="E35" t="n" s="108">
-        <v>2689425.28</v>
+        <v>2689222.54</v>
       </c>
       <c r="F35" t="s" s="18">
         <v>21</v>
@@ -2169,13 +2169,13 @@
         <v>85</v>
       </c>
       <c r="D36" t="n" s="110">
-        <v>0.076431</v>
+        <v>0.112867</v>
       </c>
       <c r="E36" t="n" s="111">
-        <v>8.739740227E7</v>
+        <v>8.795915791E7</v>
       </c>
       <c r="F36" t="n" s="112">
-        <v>8.739740227E7</v>
+        <v>8.795915791E7</v>
       </c>
       <c r="G36" t="n" s="113">
         <v>3380000.0</v>
@@ -2186,114 +2186,114 @@
         <v>86</v>
       </c>
       <c r="B37" t="s" s="18">
-        <v>21</v>
+        <v>87</v>
       </c>
       <c r="C37" t="s" s="18">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D37" t="n" s="114">
-        <v>0.0</v>
+        <v>0.03417</v>
       </c>
       <c r="E37" t="n" s="115">
-        <v>7.44</v>
-      </c>
-      <c r="F37" t="s" s="18">
-        <v>21</v>
-      </c>
-      <c r="G37" t="n" s="116">
-        <v>10.58</v>
+        <v>1.7062590858E8</v>
+      </c>
+      <c r="F37" t="n" s="116">
+        <v>1.7062590858E8</v>
+      </c>
+      <c r="G37" t="n" s="117">
+        <v>2.331E8</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s" s="18">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B38" t="s" s="18">
-        <v>21</v>
+        <v>90</v>
       </c>
       <c r="C38" t="s" s="18">
-        <v>89</v>
-      </c>
-      <c r="D38" t="n" s="117">
-        <v>-0.006863</v>
-      </c>
-      <c r="E38" t="n" s="118">
-        <v>-123915.92</v>
-      </c>
-      <c r="F38" t="s" s="18">
-        <v>21</v>
-      </c>
-      <c r="G38" t="n" s="119">
-        <v>-177976.22</v>
+        <v>91</v>
+      </c>
+      <c r="D38" t="n" s="118">
+        <v>0.002619</v>
+      </c>
+      <c r="E38" t="n" s="119">
+        <v>6.727925175E7</v>
+      </c>
+      <c r="F38" t="n" s="120">
+        <v>6.727925175E7</v>
+      </c>
+      <c r="G38" t="n" s="121">
+        <v>11025.0</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s" s="18">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B39" t="s" s="18">
         <v>21</v>
       </c>
       <c r="C39" t="s" s="18">
-        <v>91</v>
-      </c>
-      <c r="D39" t="n" s="120">
-        <v>-0.007848</v>
-      </c>
-      <c r="E39" t="n" s="121">
-        <v>-141695.2</v>
+        <v>93</v>
+      </c>
+      <c r="D39" t="n" s="122">
+        <v>0.0</v>
+      </c>
+      <c r="E39" t="n" s="123">
+        <v>7.41</v>
       </c>
       <c r="F39" t="s" s="18">
         <v>21</v>
       </c>
-      <c r="G39" t="n" s="122">
-        <v>-2.2418306E7</v>
+      <c r="G39" t="n" s="124">
+        <v>10.58</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s" s="18">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B40" t="s" s="18">
-        <v>93</v>
+        <v>21</v>
       </c>
       <c r="C40" t="s" s="18">
-        <v>94</v>
-      </c>
-      <c r="D40" t="n" s="123">
-        <v>-0.008158</v>
-      </c>
-      <c r="E40" t="n" s="124">
-        <v>1.6955324154E8</v>
-      </c>
-      <c r="F40" t="n" s="125">
-        <v>1.6955324154E8</v>
-      </c>
-      <c r="G40" t="n" s="126">
-        <v>2.331E8</v>
+        <v>95</v>
+      </c>
+      <c r="D40" t="n" s="125">
+        <v>-0.006834</v>
+      </c>
+      <c r="E40" t="n" s="126">
+        <v>-124138.39</v>
+      </c>
+      <c r="F40" t="s" s="18">
+        <v>21</v>
+      </c>
+      <c r="G40" t="n" s="127">
+        <v>-177976.22</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s" s="18">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B41" t="s" s="18">
-        <v>96</v>
+        <v>21</v>
       </c>
       <c r="C41" t="s" s="18">
         <v>97</v>
       </c>
-      <c r="D41" t="n" s="127">
-        <v>-0.019904</v>
-      </c>
-      <c r="E41" t="n" s="128">
-        <v>6.675184123E7</v>
-      </c>
-      <c r="F41" t="n" s="129">
-        <v>6.675184123E7</v>
+      <c r="D41" t="n" s="128">
+        <v>-0.00779</v>
+      </c>
+      <c r="E41" t="n" s="129">
+        <v>-141516.31</v>
+      </c>
+      <c r="F41" t="s" s="18">
+        <v>21</v>
       </c>
       <c r="G41" t="n" s="130">
-        <v>11025.0</v>
+        <v>-2.2418306E7</v>
       </c>
     </row>
     <row r="42">
@@ -2307,13 +2307,13 @@
         <v>100</v>
       </c>
       <c r="D42" t="n" s="131">
-        <v>-0.107989</v>
+        <v>-0.064588</v>
       </c>
       <c r="E42" t="n" s="132">
-        <v>7.01820363E7</v>
+        <v>7.095302963E7</v>
       </c>
       <c r="F42" t="n" s="133">
-        <v>7.01820363E7</v>
+        <v>7.095302963E7</v>
       </c>
       <c r="G42" t="n" s="134">
         <v>5060.0</v>
@@ -2330,16 +2330,16 @@
         <v>103</v>
       </c>
       <c r="D43" t="n" s="135">
-        <v>-0.155067</v>
+        <v>-0.104507</v>
       </c>
       <c r="E43" t="n" s="136">
-        <v>3.2580981148E8</v>
+        <v>1.6562984227E8</v>
       </c>
       <c r="F43" t="n" s="137">
-        <v>3.2580981148E8</v>
+        <v>1.6562984227E8</v>
       </c>
       <c r="G43" t="n" s="138">
-        <v>2.409E8</v>
+        <v>23880.0</v>
       </c>
     </row>
     <row r="44">
@@ -2353,16 +2353,16 @@
         <v>106</v>
       </c>
       <c r="D44" t="n" s="139">
-        <v>-0.171971</v>
+        <v>-0.128715</v>
       </c>
       <c r="E44" t="n" s="140">
-        <v>1.6460290063E8</v>
+        <v>3.2591959479E8</v>
       </c>
       <c r="F44" t="n" s="141">
-        <v>1.6460290063E8</v>
+        <v>3.2591959479E8</v>
       </c>
       <c r="G44" t="n" s="142">
-        <v>23880.0</v>
+        <v>2.409E8</v>
       </c>
     </row>
     <row r="45">
@@ -2376,13 +2376,13 @@
         <v>109</v>
       </c>
       <c r="D45" t="n" s="143">
-        <v>-0.21032</v>
+        <v>-0.184768</v>
       </c>
       <c r="E45" t="n" s="144">
-        <v>1.1476282243E8</v>
+        <v>1.151947389E8</v>
       </c>
       <c r="F45" t="n" s="145">
-        <v>1.1476282243E8</v>
+        <v>1.151947389E8</v>
       </c>
       <c r="G45" t="n" s="146">
         <v>1.041E8</v>
@@ -2399,13 +2399,13 @@
         <v>112</v>
       </c>
       <c r="D46" t="n" s="147">
-        <v>-0.466144</v>
+        <v>-0.328479</v>
       </c>
       <c r="E46" t="n" s="148">
-        <v>1.716841E8</v>
+        <v>1.7413319E8</v>
       </c>
       <c r="F46" t="n" s="149">
-        <v>1.716841E8</v>
+        <v>1.7413319E8</v>
       </c>
       <c r="G46" t="n" s="150">
         <v>41300.0</v>
@@ -2422,13 +2422,13 @@
         <v>115</v>
       </c>
       <c r="D47" t="n" s="151">
-        <v>-0.61852</v>
+        <v>-0.60846</v>
       </c>
       <c r="E47" t="n" s="152">
-        <v>1.882951875E8</v>
+        <v>1.88409375E8</v>
       </c>
       <c r="F47" t="n" s="153">
-        <v>1.882951875E8</v>
+        <v>1.88409375E8</v>
       </c>
       <c r="G47" t="n" s="154">
         <v>1.827E8</v>
@@ -2445,13 +2445,13 @@
         <v>118</v>
       </c>
       <c r="D48" t="n" s="155">
-        <v>-0.793136</v>
+        <v>-0.817969</v>
       </c>
       <c r="E48" t="n" s="156">
-        <v>4.5154725E8</v>
+        <v>4.5100825E8</v>
       </c>
       <c r="F48" t="n" s="157">
-        <v>4.5154725E8</v>
+        <v>4.5100825E8</v>
       </c>
       <c r="G48" t="n" s="158">
         <v>4.312E8</v>

</xml_diff>

<commit_message>
Update ALLW XLSX 2026-10-13
</commit_message>
<xml_diff>
--- a/latest/allw-latest.xlsx
+++ b/latest/allw-latest.xlsx
@@ -192,7 +192,7 @@
     <t>ALLW</t>
   </si>
   <si>
-    <t>As of 09-Oct-2026</t>
+    <t>As of 12-Oct-2026</t>
   </si>
   <si>
     <t>Name</t>
@@ -1479,7 +1479,7 @@
         <v>22</v>
       </c>
       <c r="D6" t="n" s="19">
-        <v>33.794871</v>
+        <v>33.754015</v>
       </c>
       <c r="E6" t="n" s="20">
         <v>6.1390035639E8</v>
@@ -1502,10 +1502,10 @@
         <v>25</v>
       </c>
       <c r="D7" t="n" s="22">
-        <v>13.771398</v>
+        <v>13.745744</v>
       </c>
       <c r="E7" t="n" s="23">
-        <v>2.5016418712E8</v>
+        <v>2.5000039564E8</v>
       </c>
       <c r="F7" t="s" s="18">
         <v>21</v>
@@ -1525,7 +1525,7 @@
         <v>27</v>
       </c>
       <c r="D8" t="n" s="25">
-        <v>5.001418</v>
+        <v>4.995371</v>
       </c>
       <c r="E8" t="n" s="26">
         <v>9.085319589E7</v>
@@ -1548,7 +1548,7 @@
         <v>29</v>
       </c>
       <c r="D9" t="n" s="28">
-        <v>4.97475</v>
+        <v>4.968736</v>
       </c>
       <c r="E9" t="n" s="29">
         <v>9.036876634E7</v>
@@ -1571,10 +1571,10 @@
         <v>32</v>
       </c>
       <c r="D10" t="n" s="31">
-        <v>4.347698</v>
+        <v>4.334957</v>
       </c>
       <c r="E10" t="n" s="32">
-        <v>7.8978067E7</v>
+        <v>7.8841924E7</v>
       </c>
       <c r="F10" t="s" s="18">
         <v>21</v>
@@ -1594,16 +1594,16 @@
         <v>34</v>
       </c>
       <c r="D11" t="n" s="34">
-        <v>4.260765</v>
+        <v>4.256064</v>
       </c>
       <c r="E11" t="n" s="35">
-        <v>7.739888344E7</v>
+        <v>7.740706121E7</v>
       </c>
       <c r="F11" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G11" t="n" s="36">
-        <v>8.360033E7</v>
+        <v>8.3609163E7</v>
       </c>
     </row>
     <row r="12">
@@ -1617,16 +1617,16 @@
         <v>36</v>
       </c>
       <c r="D12" t="n" s="37">
-        <v>4.167787</v>
+        <v>4.163153</v>
       </c>
       <c r="E12" t="n" s="38">
-        <v>7.570988719E7</v>
+        <v>7.571724616E7</v>
       </c>
       <c r="F12" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G12" t="n" s="39">
-        <v>8.2510562E7</v>
+        <v>8.2518582E7</v>
       </c>
     </row>
     <row r="13">
@@ -1640,16 +1640,16 @@
         <v>38</v>
       </c>
       <c r="D13" t="n" s="40">
-        <v>3.986661</v>
+        <v>3.982255</v>
       </c>
       <c r="E13" t="n" s="41">
-        <v>7.241964088E7</v>
+        <v>7.242716123E7</v>
       </c>
       <c r="F13" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G13" t="n" s="42">
-        <v>7.6374088E7</v>
+        <v>7.6382019E7</v>
       </c>
     </row>
     <row r="14">
@@ -1663,16 +1663,16 @@
         <v>40</v>
       </c>
       <c r="D14" t="n" s="43">
-        <v>3.679182</v>
+        <v>3.675114</v>
       </c>
       <c r="E14" t="n" s="44">
-        <v>6.683414795E7</v>
+        <v>6.684104861E7</v>
       </c>
       <c r="F14" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G14" t="n" s="45">
-        <v>7.119335025E7</v>
+        <v>7.1200701E7</v>
       </c>
     </row>
     <row r="15">
@@ -1686,16 +1686,16 @@
         <v>42</v>
       </c>
       <c r="D15" t="n" s="46">
-        <v>3.506829</v>
+        <v>3.502944</v>
       </c>
       <c r="E15" t="n" s="47">
-        <v>6.370327265E7</v>
+        <v>6.370971608E7</v>
       </c>
       <c r="F15" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G15" t="n" s="48">
-        <v>6.82473176E7</v>
+        <v>6.825422065E7</v>
       </c>
     </row>
     <row r="16">
@@ -1709,10 +1709,10 @@
         <v>45</v>
       </c>
       <c r="D16" t="n" s="49">
-        <v>3.343982</v>
+        <v>3.307834</v>
       </c>
       <c r="E16" t="n" s="50">
-        <v>6.074506861E7</v>
+        <v>6.016114951E7</v>
       </c>
       <c r="F16" t="s" s="18">
         <v>21</v>
@@ -1732,16 +1732,16 @@
         <v>47</v>
       </c>
       <c r="D17" t="n" s="52">
-        <v>2.518836</v>
+        <v>2.516068</v>
       </c>
       <c r="E17" t="n" s="53">
-        <v>4.575589081E7</v>
+        <v>4.576091908E7</v>
       </c>
       <c r="F17" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G17" t="n" s="54">
-        <v>4.7846366E7</v>
+        <v>4.7851624E7</v>
       </c>
     </row>
     <row r="18">
@@ -1755,16 +1755,16 @@
         <v>49</v>
       </c>
       <c r="D18" t="n" s="55">
-        <v>1.467713</v>
+        <v>1.466092</v>
       </c>
       <c r="E18" t="n" s="56">
-        <v>2.666172852E7</v>
+        <v>2.666451666E7</v>
       </c>
       <c r="F18" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G18" t="n" s="57">
-        <v>3.55869678E7</v>
+        <v>3.55906893E7</v>
       </c>
     </row>
     <row r="19">
@@ -1778,16 +1778,16 @@
         <v>51</v>
       </c>
       <c r="D19" t="n" s="58">
-        <v>1.296206</v>
+        <v>1.294776</v>
       </c>
       <c r="E19" t="n" s="59">
-        <v>2.354621363E7</v>
+        <v>2.354870157E7</v>
       </c>
       <c r="F19" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G19" t="n" s="60">
-        <v>3.62499967E7</v>
+        <v>3.625382695E7</v>
       </c>
     </row>
     <row r="20">
@@ -1801,16 +1801,16 @@
         <v>53</v>
       </c>
       <c r="D20" t="n" s="61">
-        <v>1.214687</v>
+        <v>1.213344</v>
       </c>
       <c r="E20" t="n" s="62">
-        <v>2.20653792E7</v>
+        <v>2.206767028E7</v>
       </c>
       <c r="F20" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G20" t="n" s="63">
-        <v>2.68348553E7</v>
+        <v>2.68376416E7</v>
       </c>
     </row>
     <row r="21">
@@ -1824,16 +1824,16 @@
         <v>55</v>
       </c>
       <c r="D21" t="n" s="64">
-        <v>1.143693</v>
+        <v>1.142426</v>
       </c>
       <c r="E21" t="n" s="65">
-        <v>2.077574931E7</v>
+        <v>2.077784739E7</v>
       </c>
       <c r="F21" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G21" t="n" s="66">
-        <v>2.660493125E7</v>
+        <v>2.6607618E7</v>
       </c>
     </row>
     <row r="22">
@@ -1847,16 +1847,16 @@
         <v>57</v>
       </c>
       <c r="D22" t="n" s="67">
-        <v>1.119644</v>
+        <v>1.11841</v>
       </c>
       <c r="E22" t="n" s="68">
-        <v>2.033888755E7</v>
+        <v>2.034105653E7</v>
       </c>
       <c r="F22" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G22" t="n" s="69">
-        <v>2.475576E7</v>
+        <v>2.47584E7</v>
       </c>
     </row>
     <row r="23">
@@ -1870,16 +1870,16 @@
         <v>59</v>
       </c>
       <c r="D23" t="n" s="70">
-        <v>1.09084</v>
+        <v>1.089631</v>
       </c>
       <c r="E23" t="n" s="71">
-        <v>1.981563561E7</v>
+        <v>1.981764471E7</v>
       </c>
       <c r="F23" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G23" t="n" s="72">
-        <v>2.82277152E7</v>
+        <v>2.82305772E7</v>
       </c>
     </row>
     <row r="24">
@@ -1893,16 +1893,16 @@
         <v>61</v>
       </c>
       <c r="D24" t="n" s="73">
-        <v>0.93577</v>
+        <v>0.934739</v>
       </c>
       <c r="E24" t="n" s="74">
-        <v>1.699872616E7</v>
+        <v>1.700053998E7</v>
       </c>
       <c r="F24" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G24" t="n" s="75">
-        <v>2.5078803E7</v>
+        <v>2.5081479E7</v>
       </c>
     </row>
     <row r="25">
@@ -1916,16 +1916,16 @@
         <v>63</v>
       </c>
       <c r="D25" t="n" s="76">
-        <v>0.920132</v>
+        <v>0.919115</v>
       </c>
       <c r="E25" t="n" s="77">
-        <v>1.671465315E7</v>
+        <v>1.671637747E7</v>
       </c>
       <c r="F25" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G25" t="n" s="78">
-        <v>2.49946038E7</v>
+        <v>2.49971823E7</v>
       </c>
     </row>
     <row r="26">
@@ -1939,16 +1939,16 @@
         <v>65</v>
       </c>
       <c r="D26" t="n" s="79">
-        <v>0.873151</v>
+        <v>0.872183</v>
       </c>
       <c r="E26" t="n" s="80">
-        <v>1.586120604E7</v>
+        <v>1.58628095E7</v>
       </c>
       <c r="F26" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G26" t="n" s="81">
-        <v>2.4858237E7</v>
+        <v>2.486075E7</v>
       </c>
     </row>
     <row r="27">
@@ -1962,16 +1962,16 @@
         <v>67</v>
       </c>
       <c r="D27" t="n" s="82">
-        <v>0.722883</v>
+        <v>0.722081</v>
       </c>
       <c r="E27" t="n" s="83">
-        <v>1.313152551E7</v>
+        <v>1.313282856E7</v>
       </c>
       <c r="F27" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G27" t="n" s="84">
-        <v>1.95827368E7</v>
+        <v>1.958468E7</v>
       </c>
     </row>
     <row r="28">
@@ -1985,16 +1985,16 @@
         <v>69</v>
       </c>
       <c r="D28" t="n" s="85">
-        <v>0.709079</v>
+        <v>0.708292</v>
       </c>
       <c r="E28" t="n" s="86">
-        <v>1.288076099E7</v>
+        <v>1.288204812E7</v>
       </c>
       <c r="F28" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G28" t="n" s="87">
-        <v>2.8460856E7</v>
+        <v>2.84637E7</v>
       </c>
     </row>
     <row r="29">
@@ -2008,16 +2008,16 @@
         <v>71</v>
       </c>
       <c r="D29" t="n" s="88">
-        <v>0.702621</v>
+        <v>0.701842</v>
       </c>
       <c r="E29" t="n" s="89">
-        <v>1.276345534E7</v>
+        <v>1.276473141E7</v>
       </c>
       <c r="F29" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G29" t="n" s="90">
-        <v>2.55049922E7</v>
+        <v>2.550754215E7</v>
       </c>
     </row>
     <row r="30">
@@ -2031,16 +2031,16 @@
         <v>73</v>
       </c>
       <c r="D30" t="n" s="91">
-        <v>0.592872</v>
+        <v>0.59222</v>
       </c>
       <c r="E30" t="n" s="92">
-        <v>1.076981087E7</v>
+        <v>1.077098514E7</v>
       </c>
       <c r="F30" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G30" t="n" s="93">
-        <v>2.30736597E7</v>
+        <v>2.30761755E7</v>
       </c>
     </row>
     <row r="31">
@@ -2054,16 +2054,16 @@
         <v>75</v>
       </c>
       <c r="D31" t="n" s="94">
-        <v>0.562215</v>
+        <v>0.561594</v>
       </c>
       <c r="E31" t="n" s="95">
-        <v>1.021291397E7</v>
+        <v>1.021396869E7</v>
       </c>
       <c r="F31" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G31" t="n" s="96">
-        <v>1.5860871E7</v>
+        <v>1.5862509E7</v>
       </c>
     </row>
     <row r="32">
@@ -2077,16 +2077,16 @@
         <v>77</v>
       </c>
       <c r="D32" t="n" s="97">
-        <v>0.549956</v>
+        <v>0.549345</v>
       </c>
       <c r="E32" t="n" s="98">
-        <v>9990222.12</v>
+        <v>9991199.71</v>
       </c>
       <c r="F32" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G32" t="n" s="99">
-        <v>1.577581875E7</v>
+        <v>1.57773625E7</v>
       </c>
     </row>
     <row r="33">
@@ -2100,10 +2100,10 @@
         <v>21</v>
       </c>
       <c r="D33" t="n" s="100">
-        <v>0.367568</v>
+        <v>0.472811</v>
       </c>
       <c r="E33" t="n" s="101">
-        <v>6677053.59</v>
+        <v>8599245.95</v>
       </c>
       <c r="F33" t="n" s="102">
         <v>4.1426456199E8</v>
@@ -2123,10 +2123,10 @@
         <v>80</v>
       </c>
       <c r="D34" t="n" s="104">
-        <v>0.267947</v>
+        <v>0.267073</v>
       </c>
       <c r="E34" t="n" s="105">
-        <v>4867385.25</v>
+        <v>4857384.17</v>
       </c>
       <c r="F34" t="s" s="18">
         <v>21</v>
@@ -2146,10 +2146,10 @@
         <v>82</v>
       </c>
       <c r="D35" t="n" s="107">
-        <v>0.14804</v>
+        <v>0.147794</v>
       </c>
       <c r="E35" t="n" s="108">
-        <v>2689222.54</v>
+        <v>2688003.17</v>
       </c>
       <c r="F35" t="s" s="18">
         <v>21</v>
@@ -2169,13 +2169,13 @@
         <v>85</v>
       </c>
       <c r="D36" t="n" s="110">
-        <v>0.112867</v>
+        <v>0.112531</v>
       </c>
       <c r="E36" t="n" s="111">
-        <v>8.795915791E7</v>
+        <v>8.780396358E7</v>
       </c>
       <c r="F36" t="n" s="112">
-        <v>8.795915791E7</v>
+        <v>8.780396358E7</v>
       </c>
       <c r="G36" t="n" s="113">
         <v>3380000.0</v>
@@ -2192,13 +2192,13 @@
         <v>88</v>
       </c>
       <c r="D37" t="n" s="114">
-        <v>0.03417</v>
+        <v>0.044648</v>
       </c>
       <c r="E37" t="n" s="115">
-        <v>1.7062590858E8</v>
+        <v>1.7052473631E8</v>
       </c>
       <c r="F37" t="n" s="116">
-        <v>1.7062590858E8</v>
+        <v>1.7052473631E8</v>
       </c>
       <c r="G37" t="n" s="117">
         <v>2.331E8</v>
@@ -2215,13 +2215,13 @@
         <v>91</v>
       </c>
       <c r="D38" t="n" s="118">
-        <v>0.002619</v>
+        <v>0.025404</v>
       </c>
       <c r="E38" t="n" s="119">
-        <v>6.727925175E7</v>
+        <v>6.757803606E7</v>
       </c>
       <c r="F38" t="n" s="120">
-        <v>6.727925175E7</v>
+        <v>6.757803606E7</v>
       </c>
       <c r="G38" t="n" s="121">
         <v>11025.0</v>
@@ -2261,10 +2261,10 @@
         <v>95</v>
       </c>
       <c r="D40" t="n" s="125">
-        <v>-0.006834</v>
+        <v>-0.006814</v>
       </c>
       <c r="E40" t="n" s="126">
-        <v>-124138.39</v>
+        <v>-123924.81</v>
       </c>
       <c r="F40" t="s" s="18">
         <v>21</v>
@@ -2284,10 +2284,10 @@
         <v>97</v>
       </c>
       <c r="D41" t="n" s="128">
-        <v>-0.00779</v>
+        <v>-0.007767</v>
       </c>
       <c r="E41" t="n" s="129">
-        <v>-141516.31</v>
+        <v>-141266.62</v>
       </c>
       <c r="F41" t="s" s="18">
         <v>21</v>
@@ -2307,13 +2307,13 @@
         <v>100</v>
       </c>
       <c r="D42" t="n" s="131">
-        <v>-0.064588</v>
+        <v>-0.033403</v>
       </c>
       <c r="E42" t="n" s="132">
-        <v>7.095302963E7</v>
+        <v>7.148608383E7</v>
       </c>
       <c r="F42" t="n" s="133">
-        <v>7.095302963E7</v>
+        <v>7.148608383E7</v>
       </c>
       <c r="G42" t="n" s="134">
         <v>5060.0</v>
@@ -2330,13 +2330,13 @@
         <v>103</v>
       </c>
       <c r="D43" t="n" s="135">
-        <v>-0.104507</v>
+        <v>-0.076293</v>
       </c>
       <c r="E43" t="n" s="136">
-        <v>1.6562984227E8</v>
+        <v>1.6579646151E8</v>
       </c>
       <c r="F43" t="n" s="137">
-        <v>1.6562984227E8</v>
+        <v>1.6579646151E8</v>
       </c>
       <c r="G43" t="n" s="138">
         <v>23880.0</v>
@@ -2353,13 +2353,13 @@
         <v>106</v>
       </c>
       <c r="D44" t="n" s="139">
-        <v>-0.128715</v>
+        <v>-0.110536</v>
       </c>
       <c r="E44" t="n" s="140">
-        <v>3.2591959479E8</v>
+        <v>3.2557291219E8</v>
       </c>
       <c r="F44" t="n" s="141">
-        <v>3.2591959479E8</v>
+        <v>3.2557291219E8</v>
       </c>
       <c r="G44" t="n" s="142">
         <v>2.409E8</v>
@@ -2376,13 +2376,13 @@
         <v>109</v>
       </c>
       <c r="D45" t="n" s="143">
-        <v>-0.184768</v>
+        <v>-0.172354</v>
       </c>
       <c r="E45" t="n" s="144">
-        <v>1.151947389E8</v>
+        <v>1.1536269033E8</v>
       </c>
       <c r="F45" t="n" s="145">
-        <v>1.151947389E8</v>
+        <v>1.1536269033E8</v>
       </c>
       <c r="G45" t="n" s="146">
         <v>1.041E8</v>
@@ -2399,13 +2399,13 @@
         <v>112</v>
       </c>
       <c r="D46" t="n" s="147">
-        <v>-0.328479</v>
+        <v>-0.386441</v>
       </c>
       <c r="E46" t="n" s="148">
-        <v>1.7413319E8</v>
+        <v>1.7307178E8</v>
       </c>
       <c r="F46" t="n" s="149">
-        <v>1.7413319E8</v>
+        <v>1.7307178E8</v>
       </c>
       <c r="G46" t="n" s="150">
         <v>41300.0</v>
@@ -2422,13 +2422,13 @@
         <v>115</v>
       </c>
       <c r="D47" t="n" s="151">
-        <v>-0.60846</v>
+        <v>-0.604585</v>
       </c>
       <c r="E47" t="n" s="152">
-        <v>1.88409375E8</v>
+        <v>1.8846646875E8</v>
       </c>
       <c r="F47" t="n" s="153">
-        <v>1.88409375E8</v>
+        <v>1.8846646875E8</v>
       </c>
       <c r="G47" t="n" s="154">
         <v>1.827E8</v>
@@ -2445,13 +2445,13 @@
         <v>118</v>
       </c>
       <c r="D48" t="n" s="155">
-        <v>-0.817969</v>
+        <v>-0.824389</v>
       </c>
       <c r="E48" t="n" s="156">
-        <v>4.5100825E8</v>
+        <v>4.508735E8</v>
       </c>
       <c r="F48" t="n" s="157">
-        <v>4.5100825E8</v>
+        <v>4.508735E8</v>
       </c>
       <c r="G48" t="n" s="158">
         <v>4.312E8</v>

</xml_diff>

<commit_message>
Update ALLW XLSX 2026-10-14
</commit_message>
<xml_diff>
--- a/latest/allw-latest.xlsx
+++ b/latest/allw-latest.xlsx
@@ -192,7 +192,7 @@
     <t>ALLW</t>
   </si>
   <si>
-    <t>As of 12-Oct-2026</t>
+    <t>As of 13-Oct-2026</t>
   </si>
   <si>
     <t>Name</t>
@@ -234,27 +234,27 @@
     <t>78464A854</t>
   </si>
   <si>
+    <t>TREASURY BILL 02/27 0.00000</t>
+  </si>
+  <si>
+    <t>912797TV9</t>
+  </si>
+  <si>
+    <t>STATE STREET SPDR PORTFOLIO EM</t>
+  </si>
+  <si>
+    <t>SPEM</t>
+  </si>
+  <si>
+    <t>78463X509</t>
+  </si>
+  <si>
     <t>US DOLLAR</t>
   </si>
   <si>
     <t>999USDZ92</t>
   </si>
   <si>
-    <t>TREASURY BILL 02/27 0.00000</t>
-  </si>
-  <si>
-    <t>912797TV9</t>
-  </si>
-  <si>
-    <t>STATE STREET SPDR PORTFOLIO EM</t>
-  </si>
-  <si>
-    <t>SPEM</t>
-  </si>
-  <si>
-    <t>78463X509</t>
-  </si>
-  <si>
     <t>TSY INFL IX N/B 07/35 1.875</t>
   </si>
   <si>
@@ -459,6 +459,15 @@
     <t>ADI38QPG9</t>
   </si>
   <si>
+    <t>EURO-BUND FUTURE  DEC26</t>
+  </si>
+  <si>
+    <t>RXZ6</t>
+  </si>
+  <si>
+    <t>ADI39K4N9</t>
+  </si>
+  <si>
     <t>EURO STOXX 50     DEC26</t>
   </si>
   <si>
@@ -466,15 +475,6 @@
   </si>
   <si>
     <t>ADI2VHXS0</t>
-  </si>
-  <si>
-    <t>EURO-BUND FUTURE  DEC26</t>
-  </si>
-  <si>
-    <t>RXZ6</t>
-  </si>
-  <si>
-    <t>ADI39K4N9</t>
   </si>
   <si>
     <t>LONG GILT FUTURE  DEC26</t>
@@ -1479,16 +1479,16 @@
         <v>22</v>
       </c>
       <c r="D6" t="n" s="19">
-        <v>33.754015</v>
+        <v>34.173421</v>
       </c>
       <c r="E6" t="n" s="20">
-        <v>6.1390035639E8</v>
+        <v>6.2108583588E8</v>
       </c>
       <c r="F6" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G6" t="n" s="21">
-        <v>6.1390035639E8</v>
+        <v>6.2108583588E8</v>
       </c>
     </row>
     <row r="7">
@@ -1502,10 +1502,10 @@
         <v>25</v>
       </c>
       <c r="D7" t="n" s="22">
-        <v>13.745744</v>
+        <v>13.75103</v>
       </c>
       <c r="E7" t="n" s="23">
-        <v>2.5000039564E8</v>
+        <v>2.499184999E8</v>
       </c>
       <c r="F7" t="s" s="18">
         <v>21</v>
@@ -1525,16 +1525,16 @@
         <v>27</v>
       </c>
       <c r="D8" t="n" s="25">
-        <v>4.995371</v>
+        <v>4.972657</v>
       </c>
       <c r="E8" t="n" s="26">
-        <v>9.085319589E7</v>
+        <v>9.037570528E7</v>
       </c>
       <c r="F8" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G8" t="n" s="27">
-        <v>9.085319589E7</v>
+        <v>9.17E7</v>
       </c>
     </row>
     <row r="9">
@@ -1542,45 +1542,45 @@
         <v>28</v>
       </c>
       <c r="B9" t="s" s="18">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="C9" t="s" s="18">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D9" t="n" s="28">
-        <v>4.968736</v>
+        <v>4.340542</v>
       </c>
       <c r="E9" t="n" s="29">
-        <v>9.036876634E7</v>
+        <v>7.8887305E7</v>
       </c>
       <c r="F9" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G9" t="n" s="30">
-        <v>9.17E7</v>
+        <v>1512700.0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="18">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B10" t="s" s="18">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="C10" t="s" s="18">
         <v>32</v>
       </c>
       <c r="D10" t="n" s="31">
-        <v>4.334957</v>
+        <v>4.285398</v>
       </c>
       <c r="E10" t="n" s="32">
-        <v>7.8841924E7</v>
+        <v>7.788509181E7</v>
       </c>
       <c r="F10" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G10" t="n" s="33">
-        <v>1512700.0</v>
+        <v>7.788509181E7</v>
       </c>
     </row>
     <row r="11">
@@ -1594,16 +1594,16 @@
         <v>34</v>
       </c>
       <c r="D11" t="n" s="34">
-        <v>4.256064</v>
+        <v>4.265615</v>
       </c>
       <c r="E11" t="n" s="35">
-        <v>7.740706121E7</v>
+        <v>7.752555005E7</v>
       </c>
       <c r="F11" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G11" t="n" s="36">
-        <v>8.3609163E7</v>
+        <v>8.3617193E7</v>
       </c>
     </row>
     <row r="12">
@@ -1617,16 +1617,16 @@
         <v>36</v>
       </c>
       <c r="D12" t="n" s="37">
-        <v>4.163153</v>
+        <v>4.173482</v>
       </c>
       <c r="E12" t="n" s="38">
-        <v>7.571724616E7</v>
+        <v>7.585106576E7</v>
       </c>
       <c r="F12" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G12" t="n" s="39">
-        <v>8.2518582E7</v>
+        <v>8.2527404E7</v>
       </c>
     </row>
     <row r="13">
@@ -1640,16 +1640,16 @@
         <v>38</v>
       </c>
       <c r="D13" t="n" s="40">
-        <v>3.982255</v>
+        <v>3.990349</v>
       </c>
       <c r="E13" t="n" s="41">
-        <v>7.242716123E7</v>
+        <v>7.252270878E7</v>
       </c>
       <c r="F13" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G13" t="n" s="42">
-        <v>7.6382019E7</v>
+        <v>7.638995E7</v>
       </c>
     </row>
     <row r="14">
@@ -1663,16 +1663,16 @@
         <v>40</v>
       </c>
       <c r="D14" t="n" s="43">
-        <v>3.675114</v>
+        <v>3.681249</v>
       </c>
       <c r="E14" t="n" s="44">
-        <v>6.684104861E7</v>
+        <v>6.690497126E7</v>
       </c>
       <c r="F14" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G14" t="n" s="45">
-        <v>7.1200701E7</v>
+        <v>7.120805175E7</v>
       </c>
     </row>
     <row r="15">
@@ -1686,16 +1686,16 @@
         <v>42</v>
       </c>
       <c r="D15" t="n" s="46">
-        <v>3.502944</v>
+        <v>3.508687</v>
       </c>
       <c r="E15" t="n" s="47">
-        <v>6.370971608E7</v>
+        <v>6.376874162E7</v>
       </c>
       <c r="F15" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G15" t="n" s="48">
-        <v>6.825422065E7</v>
+        <v>6.826175125E7</v>
       </c>
     </row>
     <row r="16">
@@ -1709,10 +1709,10 @@
         <v>45</v>
       </c>
       <c r="D16" t="n" s="49">
-        <v>3.307834</v>
+        <v>3.313667</v>
       </c>
       <c r="E16" t="n" s="50">
-        <v>6.016114951E7</v>
+        <v>6.022433662E7</v>
       </c>
       <c r="F16" t="s" s="18">
         <v>21</v>
@@ -1732,16 +1732,16 @@
         <v>47</v>
       </c>
       <c r="D17" t="n" s="52">
-        <v>2.516068</v>
+        <v>2.522586</v>
       </c>
       <c r="E17" t="n" s="53">
-        <v>4.576091908E7</v>
+        <v>4.584680879E7</v>
       </c>
       <c r="F17" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G17" t="n" s="54">
-        <v>4.7851624E7</v>
+        <v>4.7856404E7</v>
       </c>
     </row>
     <row r="18">
@@ -1755,16 +1755,16 @@
         <v>49</v>
       </c>
       <c r="D18" t="n" s="55">
-        <v>1.466092</v>
+        <v>1.473706</v>
       </c>
       <c r="E18" t="n" s="56">
-        <v>2.666451666E7</v>
+        <v>2.678391228E7</v>
       </c>
       <c r="F18" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G18" t="n" s="57">
-        <v>3.55906893E7</v>
+        <v>3.55941627E7</v>
       </c>
     </row>
     <row r="19">
@@ -1778,16 +1778,16 @@
         <v>51</v>
       </c>
       <c r="D19" t="n" s="58">
-        <v>1.294776</v>
+        <v>1.302255</v>
       </c>
       <c r="E19" t="n" s="59">
-        <v>2.354870157E7</v>
+        <v>2.366786893E7</v>
       </c>
       <c r="F19" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G19" t="n" s="60">
-        <v>3.625382695E7</v>
+        <v>3.625740185E7</v>
       </c>
     </row>
     <row r="20">
@@ -1801,16 +1801,16 @@
         <v>53</v>
       </c>
       <c r="D20" t="n" s="61">
-        <v>1.213344</v>
+        <v>1.221909</v>
       </c>
       <c r="E20" t="n" s="62">
-        <v>2.206767028E7</v>
+        <v>2.220762327E7</v>
       </c>
       <c r="F20" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G20" t="n" s="63">
-        <v>2.68376416E7</v>
+        <v>2.68401746E7</v>
       </c>
     </row>
     <row r="21">
@@ -1824,16 +1824,16 @@
         <v>55</v>
       </c>
       <c r="D21" t="n" s="64">
-        <v>1.142426</v>
+        <v>1.150276</v>
       </c>
       <c r="E21" t="n" s="65">
-        <v>2.077784739E7</v>
+        <v>2.090572067E7</v>
       </c>
       <c r="F21" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G21" t="n" s="66">
-        <v>2.6607618E7</v>
+        <v>2.661030475E7</v>
       </c>
     </row>
     <row r="22">
@@ -1847,16 +1847,16 @@
         <v>57</v>
       </c>
       <c r="D22" t="n" s="67">
-        <v>1.11841</v>
+        <v>1.126404</v>
       </c>
       <c r="E22" t="n" s="68">
-        <v>2.034105653E7</v>
+        <v>2.047186679E7</v>
       </c>
       <c r="F22" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G22" t="n" s="69">
-        <v>2.47584E7</v>
+        <v>2.476104E7</v>
       </c>
     </row>
     <row r="23">
@@ -1870,16 +1870,16 @@
         <v>59</v>
       </c>
       <c r="D23" t="n" s="70">
-        <v>1.089631</v>
+        <v>1.095069</v>
       </c>
       <c r="E23" t="n" s="71">
-        <v>1.981764471E7</v>
+        <v>1.990236904E7</v>
       </c>
       <c r="F23" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G23" t="n" s="72">
-        <v>2.82305772E7</v>
+        <v>2.82334392E7</v>
       </c>
     </row>
     <row r="24">
@@ -1893,16 +1893,16 @@
         <v>61</v>
       </c>
       <c r="D24" t="n" s="73">
-        <v>0.934739</v>
+        <v>0.941561</v>
       </c>
       <c r="E24" t="n" s="74">
-        <v>1.700053998E7</v>
+        <v>1.711243475E7</v>
       </c>
       <c r="F24" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G24" t="n" s="75">
-        <v>2.5081479E7</v>
+        <v>2.5083932E7</v>
       </c>
     </row>
     <row r="25">
@@ -1916,16 +1916,16 @@
         <v>63</v>
       </c>
       <c r="D25" t="n" s="76">
-        <v>0.919115</v>
+        <v>0.924324</v>
       </c>
       <c r="E25" t="n" s="77">
-        <v>1.671637747E7</v>
+        <v>1.679915576E7</v>
       </c>
       <c r="F25" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G25" t="n" s="78">
-        <v>2.49971823E7</v>
+        <v>2.49997608E7</v>
       </c>
     </row>
     <row r="26">
@@ -1939,16 +1939,16 @@
         <v>65</v>
       </c>
       <c r="D26" t="n" s="79">
-        <v>0.872183</v>
+        <v>0.877809</v>
       </c>
       <c r="E26" t="n" s="80">
-        <v>1.58628095E7</v>
+        <v>1.595376531E7</v>
       </c>
       <c r="F26" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G26" t="n" s="81">
-        <v>2.486075E7</v>
+        <v>2.4863263E7</v>
       </c>
     </row>
     <row r="27">
@@ -1962,16 +1962,16 @@
         <v>67</v>
       </c>
       <c r="D27" t="n" s="82">
-        <v>0.722081</v>
+        <v>0.726377</v>
       </c>
       <c r="E27" t="n" s="83">
-        <v>1.313282856E7</v>
+        <v>1.320155417E7</v>
       </c>
       <c r="F27" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G27" t="n" s="84">
-        <v>1.958468E7</v>
+        <v>1.9586762E7</v>
       </c>
     </row>
     <row r="28">
@@ -1985,16 +1985,16 @@
         <v>69</v>
       </c>
       <c r="D28" t="n" s="85">
-        <v>0.708292</v>
+        <v>0.714502</v>
       </c>
       <c r="E28" t="n" s="86">
-        <v>1.288204812E7</v>
+        <v>1.298574501E7</v>
       </c>
       <c r="F28" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G28" t="n" s="87">
-        <v>2.84637E7</v>
+        <v>2.8466781E7</v>
       </c>
     </row>
     <row r="29">
@@ -2008,16 +2008,16 @@
         <v>71</v>
       </c>
       <c r="D29" t="n" s="88">
-        <v>0.701842</v>
+        <v>0.707292</v>
       </c>
       <c r="E29" t="n" s="89">
-        <v>1.276473141E7</v>
+        <v>1.285469485E7</v>
       </c>
       <c r="F29" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G29" t="n" s="90">
-        <v>2.550754215E7</v>
+        <v>2.55100921E7</v>
       </c>
     </row>
     <row r="30">
@@ -2031,16 +2031,16 @@
         <v>73</v>
       </c>
       <c r="D30" t="n" s="91">
-        <v>0.59222</v>
+        <v>0.596968</v>
       </c>
       <c r="E30" t="n" s="92">
-        <v>1.077098514E7</v>
+        <v>1.084960502E7</v>
       </c>
       <c r="F30" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G30" t="n" s="93">
-        <v>2.30761755E7</v>
+        <v>2.30785116E7</v>
       </c>
     </row>
     <row r="31">
@@ -2054,16 +2054,16 @@
         <v>75</v>
       </c>
       <c r="D31" t="n" s="94">
-        <v>0.561594</v>
+        <v>0.565376</v>
       </c>
       <c r="E31" t="n" s="95">
-        <v>1.021396869E7</v>
+        <v>1.027544344E7</v>
       </c>
       <c r="F31" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G31" t="n" s="96">
-        <v>1.5862509E7</v>
+        <v>1.5864147E7</v>
       </c>
     </row>
     <row r="32">
@@ -2077,16 +2077,16 @@
         <v>77</v>
       </c>
       <c r="D32" t="n" s="97">
-        <v>0.549345</v>
+        <v>0.552999</v>
       </c>
       <c r="E32" t="n" s="98">
-        <v>9991199.71</v>
+        <v>1.005049936E7</v>
       </c>
       <c r="F32" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G32" t="n" s="99">
-        <v>1.57773625E7</v>
+        <v>1.5779025E7</v>
       </c>
     </row>
     <row r="33">
@@ -2100,10 +2100,10 @@
         <v>21</v>
       </c>
       <c r="D33" t="n" s="100">
-        <v>0.472811</v>
+        <v>0.529361</v>
       </c>
       <c r="E33" t="n" s="101">
-        <v>8599245.95</v>
+        <v>9620893.83</v>
       </c>
       <c r="F33" t="n" s="102">
         <v>4.1426456199E8</v>
@@ -2123,16 +2123,16 @@
         <v>80</v>
       </c>
       <c r="D34" t="n" s="104">
-        <v>0.267073</v>
+        <v>0.267762</v>
       </c>
       <c r="E34" t="n" s="105">
-        <v>4857384.17</v>
+        <v>4866442.4</v>
       </c>
       <c r="F34" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G34" t="n" s="106">
-        <v>4347431.69</v>
+        <v>4347368.19</v>
       </c>
     </row>
     <row r="35">
@@ -2146,16 +2146,16 @@
         <v>82</v>
       </c>
       <c r="D35" t="n" s="107">
-        <v>0.147794</v>
+        <v>0.148223</v>
       </c>
       <c r="E35" t="n" s="108">
-        <v>2688003.17</v>
+        <v>2693886.61</v>
       </c>
       <c r="F35" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G35" t="n" s="109">
-        <v>2033361.5</v>
+        <v>2033351.0</v>
       </c>
     </row>
     <row r="36">
@@ -2169,13 +2169,13 @@
         <v>85</v>
       </c>
       <c r="D36" t="n" s="110">
-        <v>0.112531</v>
+        <v>0.111658</v>
       </c>
       <c r="E36" t="n" s="111">
-        <v>8.780396358E7</v>
+        <v>8.795447801E7</v>
       </c>
       <c r="F36" t="n" s="112">
-        <v>8.780396358E7</v>
+        <v>8.795447801E7</v>
       </c>
       <c r="G36" t="n" s="113">
         <v>3380000.0</v>
@@ -2192,13 +2192,13 @@
         <v>88</v>
       </c>
       <c r="D37" t="n" s="114">
-        <v>0.044648</v>
+        <v>0.066082</v>
       </c>
       <c r="E37" t="n" s="115">
-        <v>1.7052473631E8</v>
+        <v>1.7138901168E8</v>
       </c>
       <c r="F37" t="n" s="116">
-        <v>1.7052473631E8</v>
+        <v>1.7138901168E8</v>
       </c>
       <c r="G37" t="n" s="117">
         <v>2.331E8</v>
@@ -2215,13 +2215,13 @@
         <v>91</v>
       </c>
       <c r="D38" t="n" s="118">
-        <v>0.025404</v>
+        <v>0.031847</v>
       </c>
       <c r="E38" t="n" s="119">
-        <v>6.757803606E7</v>
+        <v>6.788277362E7</v>
       </c>
       <c r="F38" t="n" s="120">
-        <v>6.757803606E7</v>
+        <v>6.788277362E7</v>
       </c>
       <c r="G38" t="n" s="121">
         <v>11025.0</v>
@@ -2241,7 +2241,7 @@
         <v>0.0</v>
       </c>
       <c r="E39" t="n" s="123">
-        <v>7.41</v>
+        <v>7.44</v>
       </c>
       <c r="F39" t="s" s="18">
         <v>21</v>
@@ -2261,10 +2261,10 @@
         <v>95</v>
       </c>
       <c r="D40" t="n" s="125">
-        <v>-0.006814</v>
+        <v>-0.006838</v>
       </c>
       <c r="E40" t="n" s="126">
-        <v>-123924.81</v>
+        <v>-124271.88</v>
       </c>
       <c r="F40" t="s" s="18">
         <v>21</v>
@@ -2284,10 +2284,10 @@
         <v>97</v>
       </c>
       <c r="D41" t="n" s="128">
-        <v>-0.007767</v>
+        <v>-0.007788</v>
       </c>
       <c r="E41" t="n" s="129">
-        <v>-141266.62</v>
+        <v>-141543.11</v>
       </c>
       <c r="F41" t="s" s="18">
         <v>21</v>
@@ -2307,13 +2307,13 @@
         <v>100</v>
       </c>
       <c r="D42" t="n" s="131">
-        <v>-0.033403</v>
+        <v>-0.032578</v>
       </c>
       <c r="E42" t="n" s="132">
-        <v>7.148608383E7</v>
+        <v>7.165968029E7</v>
       </c>
       <c r="F42" t="n" s="133">
-        <v>7.148608383E7</v>
+        <v>7.165968029E7</v>
       </c>
       <c r="G42" t="n" s="134">
         <v>5060.0</v>
@@ -2330,16 +2330,16 @@
         <v>103</v>
       </c>
       <c r="D43" t="n" s="135">
-        <v>-0.076293</v>
+        <v>-0.091504</v>
       </c>
       <c r="E43" t="n" s="136">
-        <v>1.6579646151E8</v>
+        <v>3.3331278489E8</v>
       </c>
       <c r="F43" t="n" s="137">
-        <v>1.6579646151E8</v>
+        <v>3.3331278489E8</v>
       </c>
       <c r="G43" t="n" s="138">
-        <v>23880.0</v>
+        <v>2.459E8</v>
       </c>
     </row>
     <row r="44">
@@ -2353,16 +2353,16 @@
         <v>106</v>
       </c>
       <c r="D44" t="n" s="139">
-        <v>-0.110536</v>
+        <v>-0.119145</v>
       </c>
       <c r="E44" t="n" s="140">
-        <v>3.2557291219E8</v>
+        <v>1.6533286468E8</v>
       </c>
       <c r="F44" t="n" s="141">
-        <v>3.2557291219E8</v>
+        <v>1.6533286468E8</v>
       </c>
       <c r="G44" t="n" s="142">
-        <v>2.409E8</v>
+        <v>23880.0</v>
       </c>
     </row>
     <row r="45">
@@ -2376,16 +2376,16 @@
         <v>109</v>
       </c>
       <c r="D45" t="n" s="143">
-        <v>-0.172354</v>
+        <v>-0.170601</v>
       </c>
       <c r="E45" t="n" s="144">
-        <v>1.1536269033E8</v>
+        <v>1.1676818556E8</v>
       </c>
       <c r="F45" t="n" s="145">
-        <v>1.1536269033E8</v>
+        <v>1.1676818556E8</v>
       </c>
       <c r="G45" t="n" s="146">
-        <v>1.041E8</v>
+        <v>1.051E8</v>
       </c>
     </row>
     <row r="46">
@@ -2399,13 +2399,13 @@
         <v>112</v>
       </c>
       <c r="D46" t="n" s="147">
-        <v>-0.386441</v>
+        <v>-0.41694</v>
       </c>
       <c r="E46" t="n" s="148">
-        <v>1.7307178E8</v>
+        <v>1.7252249E8</v>
       </c>
       <c r="F46" t="n" s="149">
-        <v>1.7307178E8</v>
+        <v>1.7252249E8</v>
       </c>
       <c r="G46" t="n" s="150">
         <v>41300.0</v>
@@ -2422,16 +2422,16 @@
         <v>115</v>
       </c>
       <c r="D47" t="n" s="151">
-        <v>-0.604585</v>
+        <v>-0.545054</v>
       </c>
       <c r="E47" t="n" s="152">
-        <v>1.8846646875E8</v>
+        <v>1.9162625E8</v>
       </c>
       <c r="F47" t="n" s="153">
-        <v>1.8846646875E8</v>
+        <v>1.9162625E8</v>
       </c>
       <c r="G47" t="n" s="154">
-        <v>1.827E8</v>
+        <v>1.847E8</v>
       </c>
     </row>
     <row r="48">
@@ -2445,16 +2445,16 @@
         <v>118</v>
       </c>
       <c r="D48" t="n" s="155">
-        <v>-0.824389</v>
+        <v>-0.784069</v>
       </c>
       <c r="E48" t="n" s="156">
-        <v>4.508735E8</v>
+        <v>4.5475665625E8</v>
       </c>
       <c r="F48" t="n" s="157">
-        <v>4.508735E8</v>
+        <v>4.5475665625E8</v>
       </c>
       <c r="G48" t="n" s="158">
-        <v>4.312E8</v>
+        <v>4.342E8</v>
       </c>
     </row>
     <row r="49"/>

</xml_diff>

<commit_message>
Update ALLW XLSX 2026-10-15
</commit_message>
<xml_diff>
--- a/latest/allw-latest.xlsx
+++ b/latest/allw-latest.xlsx
@@ -192,7 +192,7 @@
     <t>ALLW</t>
   </si>
   <si>
-    <t>As of 13-Oct-2026</t>
+    <t>As of 14-Oct-2026</t>
   </si>
   <si>
     <t>Name</t>
@@ -240,6 +240,12 @@
     <t>912797TV9</t>
   </si>
   <si>
+    <t>US DOLLAR</t>
+  </si>
+  <si>
+    <t>999USDZ92</t>
+  </si>
+  <si>
     <t>STATE STREET SPDR PORTFOLIO EM</t>
   </si>
   <si>
@@ -249,12 +255,6 @@
     <t>78463X509</t>
   </si>
   <si>
-    <t>US DOLLAR</t>
-  </si>
-  <si>
-    <t>999USDZ92</t>
-  </si>
-  <si>
     <t>TSY INFL IX N/B 07/35 1.875</t>
   </si>
   <si>
@@ -438,6 +438,15 @@
     <t>999CADZ91</t>
   </si>
   <si>
+    <t>FTSE 100 IDX FUT  DEC26</t>
+  </si>
+  <si>
+    <t>Z Z6</t>
+  </si>
+  <si>
+    <t>ADI38QPG9</t>
+  </si>
+  <si>
     <t>AUSTRALIAN DOLLAR</t>
   </si>
   <si>
@@ -450,13 +459,13 @@
     <t>999JPYZ94</t>
   </si>
   <si>
-    <t>FTSE 100 IDX FUT  DEC26</t>
-  </si>
-  <si>
-    <t>Z Z6</t>
-  </si>
-  <si>
-    <t>ADI38QPG9</t>
+    <t>EURO STOXX 50     DEC26</t>
+  </si>
+  <si>
+    <t>VGZ6</t>
+  </si>
+  <si>
+    <t>ADI2VHXS0</t>
   </si>
   <si>
     <t>EURO-BUND FUTURE  DEC26</t>
@@ -468,15 +477,6 @@
     <t>ADI39K4N9</t>
   </si>
   <si>
-    <t>EURO STOXX 50     DEC26</t>
-  </si>
-  <si>
-    <t>VGZ6</t>
-  </si>
-  <si>
-    <t>ADI2VHXS0</t>
-  </si>
-  <si>
     <t>LONG GILT FUTURE  DEC26</t>
   </si>
   <si>
@@ -486,6 +486,15 @@
     <t>ADI3BKVP1</t>
   </si>
   <si>
+    <t>US LONG BOND(CBT) DEC26</t>
+  </si>
+  <si>
+    <t>USZ6</t>
+  </si>
+  <si>
+    <t>ADI39KYC0</t>
+  </si>
+  <si>
     <t>GOLD 100 OZ FUTR  DEC26</t>
   </si>
   <si>
@@ -493,15 +502,6 @@
   </si>
   <si>
     <t>ADI2XJBP4</t>
-  </si>
-  <si>
-    <t>US LONG BOND(CBT) DEC26</t>
-  </si>
-  <si>
-    <t>USZ6</t>
-  </si>
-  <si>
-    <t>ADI39KYC0</t>
   </si>
   <si>
     <t>US 10YR NOTE (CBT)DEC26</t>
@@ -993,22 +993,22 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
@@ -1479,16 +1479,16 @@
         <v>22</v>
       </c>
       <c r="D6" t="n" s="19">
-        <v>34.173421</v>
+        <v>34.012514</v>
       </c>
       <c r="E6" t="n" s="20">
-        <v>6.2108583588E8</v>
+        <v>6.1649870019E8</v>
       </c>
       <c r="F6" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G6" t="n" s="21">
-        <v>6.2108583588E8</v>
+        <v>6.1649870019E8</v>
       </c>
     </row>
     <row r="7">
@@ -1502,10 +1502,10 @@
         <v>25</v>
       </c>
       <c r="D7" t="n" s="22">
-        <v>13.75103</v>
+        <v>13.642028</v>
       </c>
       <c r="E7" t="n" s="23">
-        <v>2.499184999E8</v>
+        <v>2.4727053764E8</v>
       </c>
       <c r="F7" t="s" s="18">
         <v>21</v>
@@ -1525,10 +1525,10 @@
         <v>27</v>
       </c>
       <c r="D8" t="n" s="25">
-        <v>4.972657</v>
+        <v>4.986179</v>
       </c>
       <c r="E8" t="n" s="26">
-        <v>9.037570528E7</v>
+        <v>9.037770801E7</v>
       </c>
       <c r="F8" t="s" s="18">
         <v>21</v>
@@ -1542,45 +1542,45 @@
         <v>28</v>
       </c>
       <c r="B9" t="s" s="18">
+        <v>21</v>
+      </c>
+      <c r="C9" t="s" s="18">
         <v>29</v>
       </c>
-      <c r="C9" t="s" s="18">
-        <v>30</v>
-      </c>
       <c r="D9" t="n" s="28">
-        <v>4.340542</v>
+        <v>4.55003</v>
       </c>
       <c r="E9" t="n" s="29">
-        <v>7.8887305E7</v>
+        <v>8.24722275E7</v>
       </c>
       <c r="F9" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G9" t="n" s="30">
-        <v>1512700.0</v>
+        <v>8.24722275E7</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="18">
+        <v>30</v>
+      </c>
+      <c r="B10" t="s" s="18">
         <v>31</v>
-      </c>
-      <c r="B10" t="s" s="18">
-        <v>21</v>
       </c>
       <c r="C10" t="s" s="18">
         <v>32</v>
       </c>
       <c r="D10" t="n" s="31">
-        <v>4.285398</v>
+        <v>4.294664</v>
       </c>
       <c r="E10" t="n" s="32">
-        <v>7.788509181E7</v>
+        <v>7.7843542E7</v>
       </c>
       <c r="F10" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G10" t="n" s="33">
-        <v>7.788509181E7</v>
+        <v>1512700.0</v>
       </c>
     </row>
     <row r="11">
@@ -1594,16 +1594,16 @@
         <v>34</v>
       </c>
       <c r="D11" t="n" s="34">
-        <v>4.265615</v>
+        <v>4.290998</v>
       </c>
       <c r="E11" t="n" s="35">
-        <v>7.752555005E7</v>
+        <v>7.777710383E7</v>
       </c>
       <c r="F11" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G11" t="n" s="36">
-        <v>8.3617193E7</v>
+        <v>8.3626026E7</v>
       </c>
     </row>
     <row r="12">
@@ -1617,16 +1617,16 @@
         <v>36</v>
       </c>
       <c r="D12" t="n" s="37">
-        <v>4.173482</v>
+        <v>4.198752</v>
       </c>
       <c r="E12" t="n" s="38">
-        <v>7.585106576E7</v>
+        <v>7.610507591E7</v>
       </c>
       <c r="F12" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G12" t="n" s="39">
-        <v>8.2527404E7</v>
+        <v>8.2535424E7</v>
       </c>
     </row>
     <row r="13">
@@ -1640,16 +1640,16 @@
         <v>38</v>
       </c>
       <c r="D13" t="n" s="40">
-        <v>3.990349</v>
+        <v>4.012393</v>
       </c>
       <c r="E13" t="n" s="41">
-        <v>7.252270878E7</v>
+        <v>7.272720194E7</v>
       </c>
       <c r="F13" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G13" t="n" s="42">
-        <v>7.638995E7</v>
+        <v>7.6397881E7</v>
       </c>
     </row>
     <row r="14">
@@ -1663,16 +1663,16 @@
         <v>40</v>
       </c>
       <c r="D14" t="n" s="43">
-        <v>3.681249</v>
+        <v>3.700998</v>
       </c>
       <c r="E14" t="n" s="44">
-        <v>6.690497126E7</v>
+        <v>6.708296213E7</v>
       </c>
       <c r="F14" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G14" t="n" s="45">
-        <v>7.120805175E7</v>
+        <v>7.12154025E7</v>
       </c>
     </row>
     <row r="15">
@@ -1686,16 +1686,16 @@
         <v>42</v>
       </c>
       <c r="D15" t="n" s="46">
-        <v>3.508687</v>
+        <v>3.527187</v>
       </c>
       <c r="E15" t="n" s="47">
-        <v>6.376874162E7</v>
+        <v>6.39325284E7</v>
       </c>
       <c r="F15" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G15" t="n" s="48">
-        <v>6.826175125E7</v>
+        <v>6.82686543E7</v>
       </c>
     </row>
     <row r="16">
@@ -1709,10 +1709,10 @@
         <v>45</v>
       </c>
       <c r="D16" t="n" s="49">
-        <v>3.313667</v>
+        <v>3.272637</v>
       </c>
       <c r="E16" t="n" s="50">
-        <v>6.022433662E7</v>
+        <v>5.931865471E7</v>
       </c>
       <c r="F16" t="s" s="18">
         <v>21</v>
@@ -1732,16 +1732,16 @@
         <v>47</v>
       </c>
       <c r="D17" t="n" s="52">
-        <v>2.522586</v>
+        <v>2.537945</v>
       </c>
       <c r="E17" t="n" s="53">
-        <v>4.584680879E7</v>
+        <v>4.6001889E7</v>
       </c>
       <c r="F17" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G17" t="n" s="54">
-        <v>4.7856404E7</v>
+        <v>4.7861184E7</v>
       </c>
     </row>
     <row r="18">
@@ -1755,16 +1755,16 @@
         <v>49</v>
       </c>
       <c r="D18" t="n" s="55">
-        <v>1.473706</v>
+        <v>1.487195</v>
       </c>
       <c r="E18" t="n" s="56">
-        <v>2.678391228E7</v>
+        <v>2.695635862E7</v>
       </c>
       <c r="F18" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G18" t="n" s="57">
-        <v>3.55941627E7</v>
+        <v>3.55978842E7</v>
       </c>
     </row>
     <row r="19">
@@ -1778,16 +1778,16 @@
         <v>51</v>
       </c>
       <c r="D19" t="n" s="58">
-        <v>1.302255</v>
+        <v>1.315478</v>
       </c>
       <c r="E19" t="n" s="59">
-        <v>2.366786893E7</v>
+        <v>2.384388465E7</v>
       </c>
       <c r="F19" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G19" t="n" s="60">
-        <v>3.625740185E7</v>
+        <v>3.62612321E7</v>
       </c>
     </row>
     <row r="20">
@@ -1801,16 +1801,16 @@
         <v>53</v>
       </c>
       <c r="D20" t="n" s="61">
-        <v>1.221909</v>
+        <v>1.236497</v>
       </c>
       <c r="E20" t="n" s="62">
-        <v>2.220762327E7</v>
+        <v>2.241229962E7</v>
       </c>
       <c r="F20" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G20" t="n" s="63">
-        <v>2.68401746E7</v>
+        <v>2.68429609E7</v>
       </c>
     </row>
     <row r="21">
@@ -1824,16 +1824,16 @@
         <v>55</v>
       </c>
       <c r="D21" t="n" s="64">
-        <v>1.150276</v>
+        <v>1.164134</v>
       </c>
       <c r="E21" t="n" s="65">
-        <v>2.090572067E7</v>
+        <v>2.110067158E7</v>
       </c>
       <c r="F21" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G21" t="n" s="66">
-        <v>2.661030475E7</v>
+        <v>2.66129915E7</v>
       </c>
     </row>
     <row r="22">
@@ -1847,16 +1847,16 @@
         <v>57</v>
       </c>
       <c r="D22" t="n" s="67">
-        <v>1.126404</v>
+        <v>1.140199</v>
       </c>
       <c r="E22" t="n" s="68">
-        <v>2.047186679E7</v>
+        <v>2.06668318E7</v>
       </c>
       <c r="F22" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G22" t="n" s="69">
-        <v>2.476104E7</v>
+        <v>2.476344E7</v>
       </c>
     </row>
     <row r="23">
@@ -1870,16 +1870,16 @@
         <v>59</v>
       </c>
       <c r="D23" t="n" s="70">
-        <v>1.095069</v>
+        <v>1.104858</v>
       </c>
       <c r="E23" t="n" s="71">
-        <v>1.990236904E7</v>
+        <v>2.00262657E7</v>
       </c>
       <c r="F23" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G23" t="n" s="72">
-        <v>2.82334392E7</v>
+        <v>2.82363012E7</v>
       </c>
     </row>
     <row r="24">
@@ -1893,16 +1893,16 @@
         <v>61</v>
       </c>
       <c r="D24" t="n" s="73">
-        <v>0.941561</v>
+        <v>0.953014</v>
       </c>
       <c r="E24" t="n" s="74">
-        <v>1.711243475E7</v>
+        <v>1.727399154E7</v>
       </c>
       <c r="F24" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G24" t="n" s="75">
-        <v>2.5083932E7</v>
+        <v>2.5086608E7</v>
       </c>
     </row>
     <row r="25">
@@ -1916,16 +1916,16 @@
         <v>63</v>
       </c>
       <c r="D25" t="n" s="76">
-        <v>0.924324</v>
+        <v>0.932894</v>
       </c>
       <c r="E25" t="n" s="77">
-        <v>1.679915576E7</v>
+        <v>1.690929684E7</v>
       </c>
       <c r="F25" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G25" t="n" s="78">
-        <v>2.49997608E7</v>
+        <v>2.50023393E7</v>
       </c>
     </row>
     <row r="26">
@@ -1939,16 +1939,16 @@
         <v>65</v>
       </c>
       <c r="D26" t="n" s="79">
-        <v>0.877809</v>
+        <v>0.887747</v>
       </c>
       <c r="E26" t="n" s="80">
-        <v>1.595376531E7</v>
+        <v>1.609099305E7</v>
       </c>
       <c r="F26" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G26" t="n" s="81">
-        <v>2.4863263E7</v>
+        <v>2.48659555E7</v>
       </c>
     </row>
     <row r="27">
@@ -1962,16 +1962,16 @@
         <v>67</v>
       </c>
       <c r="D27" t="n" s="82">
-        <v>0.726377</v>
+        <v>0.733748</v>
       </c>
       <c r="E27" t="n" s="83">
-        <v>1.320155417E7</v>
+        <v>1.329965952E7</v>
       </c>
       <c r="F27" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G27" t="n" s="84">
-        <v>1.9586762E7</v>
+        <v>1.95887052E7</v>
       </c>
     </row>
     <row r="28">
@@ -1985,16 +1985,16 @@
         <v>69</v>
       </c>
       <c r="D28" t="n" s="85">
-        <v>0.714502</v>
+        <v>0.724999</v>
       </c>
       <c r="E28" t="n" s="86">
-        <v>1.298574501E7</v>
+        <v>1.31410673E7</v>
       </c>
       <c r="F28" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G28" t="n" s="87">
-        <v>2.8466781E7</v>
+        <v>2.8469625E7</v>
       </c>
     </row>
     <row r="29">
@@ -2008,16 +2008,16 @@
         <v>71</v>
       </c>
       <c r="D29" t="n" s="88">
-        <v>0.707292</v>
+        <v>0.716726</v>
       </c>
       <c r="E29" t="n" s="89">
-        <v>1.285469485E7</v>
+        <v>1.299111731E7</v>
       </c>
       <c r="F29" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G29" t="n" s="90">
-        <v>2.55100921E7</v>
+        <v>2.55128382E7</v>
       </c>
     </row>
     <row r="30">
@@ -2031,16 +2031,16 @@
         <v>73</v>
       </c>
       <c r="D30" t="n" s="91">
-        <v>0.596968</v>
+        <v>0.605353</v>
       </c>
       <c r="E30" t="n" s="92">
-        <v>1.084960502E7</v>
+        <v>1.097241873E7</v>
       </c>
       <c r="F30" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G30" t="n" s="93">
-        <v>2.30785116E7</v>
+        <v>2.30808477E7</v>
       </c>
     </row>
     <row r="31">
@@ -2054,16 +2054,16 @@
         <v>75</v>
       </c>
       <c r="D31" t="n" s="94">
-        <v>0.565376</v>
+        <v>0.571712</v>
       </c>
       <c r="E31" t="n" s="95">
-        <v>1.027544344E7</v>
+        <v>1.036265069E7</v>
       </c>
       <c r="F31" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G31" t="n" s="96">
-        <v>1.5864147E7</v>
+        <v>1.5865785E7</v>
       </c>
     </row>
     <row r="32">
@@ -2077,16 +2077,16 @@
         <v>77</v>
       </c>
       <c r="D32" t="n" s="97">
-        <v>0.552999</v>
+        <v>0.559514</v>
       </c>
       <c r="E32" t="n" s="98">
-        <v>1.005049936E7</v>
+        <v>1.014155745E7</v>
       </c>
       <c r="F32" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G32" t="n" s="99">
-        <v>1.5779025E7</v>
+        <v>1.57806875E7</v>
       </c>
     </row>
     <row r="33">
@@ -2100,10 +2100,10 @@
         <v>21</v>
       </c>
       <c r="D33" t="n" s="100">
-        <v>0.529361</v>
+        <v>0.403682</v>
       </c>
       <c r="E33" t="n" s="101">
-        <v>9620893.83</v>
+        <v>7316994.33</v>
       </c>
       <c r="F33" t="n" s="102">
         <v>4.1426456199E8</v>
@@ -2123,10 +2123,10 @@
         <v>80</v>
       </c>
       <c r="D34" t="n" s="104">
-        <v>0.267762</v>
+        <v>0.266745</v>
       </c>
       <c r="E34" t="n" s="105">
-        <v>4866442.4</v>
+        <v>4834927.07</v>
       </c>
       <c r="F34" t="s" s="18">
         <v>21</v>
@@ -2146,10 +2146,10 @@
         <v>82</v>
       </c>
       <c r="D35" t="n" s="107">
-        <v>0.148223</v>
+        <v>0.147613</v>
       </c>
       <c r="E35" t="n" s="108">
-        <v>2693886.61</v>
+        <v>2675585.06</v>
       </c>
       <c r="F35" t="s" s="18">
         <v>21</v>
@@ -2169,13 +2169,13 @@
         <v>85</v>
       </c>
       <c r="D36" t="n" s="110">
-        <v>0.111658</v>
+        <v>0.107519</v>
       </c>
       <c r="E36" t="n" s="111">
-        <v>8.795447801E7</v>
+        <v>8.761977904E7</v>
       </c>
       <c r="F36" t="n" s="112">
-        <v>8.795447801E7</v>
+        <v>8.761977904E7</v>
       </c>
       <c r="G36" t="n" s="113">
         <v>3380000.0</v>
@@ -2192,13 +2192,13 @@
         <v>88</v>
       </c>
       <c r="D37" t="n" s="114">
-        <v>0.066082</v>
+        <v>0.048311</v>
       </c>
       <c r="E37" t="n" s="115">
-        <v>1.7138901168E8</v>
+        <v>1.704787713E8</v>
       </c>
       <c r="F37" t="n" s="116">
-        <v>1.7138901168E8</v>
+        <v>1.704787713E8</v>
       </c>
       <c r="G37" t="n" s="117">
         <v>2.331E8</v>
@@ -2215,13 +2215,13 @@
         <v>91</v>
       </c>
       <c r="D38" t="n" s="118">
-        <v>0.031847</v>
+        <v>9.25E-4</v>
       </c>
       <c r="E38" t="n" s="119">
-        <v>6.788277362E7</v>
+        <v>6.708943623E7</v>
       </c>
       <c r="F38" t="n" s="120">
-        <v>6.788277362E7</v>
+        <v>6.708943623E7</v>
       </c>
       <c r="G38" t="n" s="121">
         <v>11025.0</v>
@@ -2241,7 +2241,7 @@
         <v>0.0</v>
       </c>
       <c r="E39" t="n" s="123">
-        <v>7.44</v>
+        <v>7.41</v>
       </c>
       <c r="F39" t="s" s="18">
         <v>21</v>
@@ -2255,68 +2255,68 @@
         <v>94</v>
       </c>
       <c r="B40" t="s" s="18">
-        <v>21</v>
+        <v>95</v>
       </c>
       <c r="C40" t="s" s="18">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D40" t="n" s="125">
-        <v>-0.006838</v>
+        <v>-0.00269</v>
       </c>
       <c r="E40" t="n" s="126">
-        <v>-124271.88</v>
-      </c>
-      <c r="F40" t="s" s="18">
-        <v>21</v>
-      </c>
-      <c r="G40" t="n" s="127">
-        <v>-177976.22</v>
+        <v>7.17121578E7</v>
+      </c>
+      <c r="F40" t="n" s="127">
+        <v>7.17121578E7</v>
+      </c>
+      <c r="G40" t="n" s="128">
+        <v>5060.0</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s" s="18">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B41" t="s" s="18">
         <v>21</v>
       </c>
       <c r="C41" t="s" s="18">
-        <v>97</v>
-      </c>
-      <c r="D41" t="n" s="128">
-        <v>-0.007788</v>
-      </c>
-      <c r="E41" t="n" s="129">
-        <v>-141543.11</v>
+        <v>98</v>
+      </c>
+      <c r="D41" t="n" s="129">
+        <v>-0.006833</v>
+      </c>
+      <c r="E41" t="n" s="130">
+        <v>-123844.78</v>
       </c>
       <c r="F41" t="s" s="18">
         <v>21</v>
       </c>
-      <c r="G41" t="n" s="130">
-        <v>-2.2418306E7</v>
+      <c r="G41" t="n" s="131">
+        <v>-177976.22</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s" s="18">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B42" t="s" s="18">
-        <v>99</v>
+        <v>21</v>
       </c>
       <c r="C42" t="s" s="18">
         <v>100</v>
       </c>
-      <c r="D42" t="n" s="131">
-        <v>-0.032578</v>
-      </c>
-      <c r="E42" t="n" s="132">
-        <v>7.165968029E7</v>
-      </c>
-      <c r="F42" t="n" s="133">
-        <v>7.165968029E7</v>
+      <c r="D42" t="n" s="132">
+        <v>-0.007786</v>
+      </c>
+      <c r="E42" t="n" s="133">
+        <v>-141124.33</v>
+      </c>
+      <c r="F42" t="s" s="18">
+        <v>21</v>
       </c>
       <c r="G42" t="n" s="134">
-        <v>5060.0</v>
+        <v>-2.2418306E7</v>
       </c>
     </row>
     <row r="43">
@@ -2330,16 +2330,16 @@
         <v>103</v>
       </c>
       <c r="D43" t="n" s="135">
-        <v>-0.091504</v>
+        <v>-0.076201</v>
       </c>
       <c r="E43" t="n" s="136">
-        <v>3.3331278489E8</v>
+        <v>1.6503234689E8</v>
       </c>
       <c r="F43" t="n" s="137">
-        <v>3.3331278489E8</v>
+        <v>1.6503234689E8</v>
       </c>
       <c r="G43" t="n" s="138">
-        <v>2.459E8</v>
+        <v>23880.0</v>
       </c>
     </row>
     <row r="44">
@@ -2353,16 +2353,16 @@
         <v>106</v>
       </c>
       <c r="D44" t="n" s="139">
-        <v>-0.119145</v>
+        <v>-0.110771</v>
       </c>
       <c r="E44" t="n" s="140">
-        <v>1.6533286468E8</v>
+        <v>3.3079871302E8</v>
       </c>
       <c r="F44" t="n" s="141">
-        <v>1.6533286468E8</v>
+        <v>3.3079871302E8</v>
       </c>
       <c r="G44" t="n" s="142">
-        <v>23880.0</v>
+        <v>2.459E8</v>
       </c>
     </row>
     <row r="45">
@@ -2376,13 +2376,13 @@
         <v>109</v>
       </c>
       <c r="D45" t="n" s="143">
-        <v>-0.170601</v>
+        <v>-0.166084</v>
       </c>
       <c r="E45" t="n" s="144">
-        <v>1.1676818556E8</v>
+        <v>1.160440415E8</v>
       </c>
       <c r="F45" t="n" s="145">
-        <v>1.1676818556E8</v>
+        <v>1.160440415E8</v>
       </c>
       <c r="G45" t="n" s="146">
         <v>1.051E8</v>
@@ -2399,16 +2399,16 @@
         <v>112</v>
       </c>
       <c r="D46" t="n" s="147">
-        <v>-0.41694</v>
+        <v>-0.501943</v>
       </c>
       <c r="E46" t="n" s="148">
-        <v>1.7252249E8</v>
+        <v>1.924343125E8</v>
       </c>
       <c r="F46" t="n" s="149">
-        <v>1.7252249E8</v>
+        <v>1.924343125E8</v>
       </c>
       <c r="G46" t="n" s="150">
-        <v>41300.0</v>
+        <v>1.847E8</v>
       </c>
     </row>
     <row r="47">
@@ -2422,16 +2422,16 @@
         <v>115</v>
       </c>
       <c r="D47" t="n" s="151">
-        <v>-0.545054</v>
+        <v>-0.576195</v>
       </c>
       <c r="E47" t="n" s="152">
-        <v>1.9162625E8</v>
+        <v>1.6965627E8</v>
       </c>
       <c r="F47" t="n" s="153">
-        <v>1.9162625E8</v>
+        <v>1.6965627E8</v>
       </c>
       <c r="G47" t="n" s="154">
-        <v>1.847E8</v>
+        <v>41300.0</v>
       </c>
     </row>
     <row r="48">
@@ -2445,13 +2445,13 @@
         <v>118</v>
       </c>
       <c r="D48" t="n" s="155">
-        <v>-0.784069</v>
+        <v>-0.752497</v>
       </c>
       <c r="E48" t="n" s="156">
-        <v>4.5475665625E8</v>
+        <v>4.5536725E8</v>
       </c>
       <c r="F48" t="n" s="157">
-        <v>4.5475665625E8</v>
+        <v>4.5536725E8</v>
       </c>
       <c r="G48" t="n" s="158">
         <v>4.342E8</v>

</xml_diff>

<commit_message>
Update ALLW XLSX 2026-10-16
</commit_message>
<xml_diff>
--- a/latest/allw-latest.xlsx
+++ b/latest/allw-latest.xlsx
@@ -192,7 +192,7 @@
     <t>ALLW</t>
   </si>
   <si>
-    <t>As of 14-Oct-2026</t>
+    <t>As of 15-Oct-2026</t>
   </si>
   <si>
     <t>Name</t>
@@ -246,6 +246,12 @@
     <t>999USDZ92</t>
   </si>
   <si>
+    <t>TSY INFL IX N/B 07/35 1.875</t>
+  </si>
+  <si>
+    <t>91282CNS6</t>
+  </si>
+  <si>
     <t>STATE STREET SPDR PORTFOLIO EM</t>
   </si>
   <si>
@@ -255,12 +261,6 @@
     <t>78463X509</t>
   </si>
   <si>
-    <t>TSY INFL IX N/B 07/35 1.875</t>
-  </si>
-  <si>
-    <t>91282CNS6</t>
-  </si>
-  <si>
     <t>TSY INFL IX N/B 01/36 1.875</t>
   </si>
   <si>
@@ -405,6 +405,60 @@
     <t>999GBPZ94</t>
   </si>
   <si>
+    <t>AUST 10Y BOND FUT DEC26</t>
+  </si>
+  <si>
+    <t>XMZ6</t>
+  </si>
+  <si>
+    <t>ADI3BDHZ1</t>
+  </si>
+  <si>
+    <t>FTSE 100 IDX FUT  DEC26</t>
+  </si>
+  <si>
+    <t>Z Z6</t>
+  </si>
+  <si>
+    <t>ADI38QPG9</t>
+  </si>
+  <si>
+    <t>SPI 200 FUTURES   DEC26</t>
+  </si>
+  <si>
+    <t>XPZ6</t>
+  </si>
+  <si>
+    <t>ADI391SG0</t>
+  </si>
+  <si>
+    <t>CANADIAN DOLLAR</t>
+  </si>
+  <si>
+    <t>999CADZ91</t>
+  </si>
+  <si>
+    <t>EURO-BUND FUTURE  DEC26</t>
+  </si>
+  <si>
+    <t>RXZ6</t>
+  </si>
+  <si>
+    <t>ADI39K4N9</t>
+  </si>
+  <si>
+    <t>AUSTRALIAN DOLLAR</t>
+  </si>
+  <si>
+    <t>999AUDZ93</t>
+  </si>
+  <si>
+    <t>JAPANESE YEN</t>
+  </si>
+  <si>
+    <t>999JPYZ94</t>
+  </si>
+  <si>
     <t>TOPIX INDX FUTR   DEC26</t>
   </si>
   <si>
@@ -414,49 +468,13 @@
     <t>ADI3917X6</t>
   </si>
   <si>
-    <t>AUST 10Y BOND FUT DEC26</t>
-  </si>
-  <si>
-    <t>XMZ6</t>
-  </si>
-  <si>
-    <t>ADI3BDHZ1</t>
-  </si>
-  <si>
-    <t>SPI 200 FUTURES   DEC26</t>
-  </si>
-  <si>
-    <t>XPZ6</t>
-  </si>
-  <si>
-    <t>ADI391SG0</t>
-  </si>
-  <si>
-    <t>CANADIAN DOLLAR</t>
-  </si>
-  <si>
-    <t>999CADZ91</t>
-  </si>
-  <si>
-    <t>FTSE 100 IDX FUT  DEC26</t>
-  </si>
-  <si>
-    <t>Z Z6</t>
-  </si>
-  <si>
-    <t>ADI38QPG9</t>
-  </si>
-  <si>
-    <t>AUSTRALIAN DOLLAR</t>
-  </si>
-  <si>
-    <t>999AUDZ93</t>
-  </si>
-  <si>
-    <t>JAPANESE YEN</t>
-  </si>
-  <si>
-    <t>999JPYZ94</t>
+    <t>LONG GILT FUTURE  DEC26</t>
+  </si>
+  <si>
+    <t>G Z6</t>
+  </si>
+  <si>
+    <t>ADI3BKVP1</t>
   </si>
   <si>
     <t>EURO STOXX 50     DEC26</t>
@@ -466,24 +484,6 @@
   </si>
   <si>
     <t>ADI2VHXS0</t>
-  </si>
-  <si>
-    <t>EURO-BUND FUTURE  DEC26</t>
-  </si>
-  <si>
-    <t>RXZ6</t>
-  </si>
-  <si>
-    <t>ADI39K4N9</t>
-  </si>
-  <si>
-    <t>LONG GILT FUTURE  DEC26</t>
-  </si>
-  <si>
-    <t>G Z6</t>
-  </si>
-  <si>
-    <t>ADI3BKVP1</t>
   </si>
   <si>
     <t>US LONG BOND(CBT) DEC26</t>
@@ -1479,16 +1479,16 @@
         <v>22</v>
       </c>
       <c r="D6" t="n" s="19">
-        <v>34.012514</v>
+        <v>33.574153</v>
       </c>
       <c r="E6" t="n" s="20">
-        <v>6.1649870019E8</v>
+        <v>6.1525597844E8</v>
       </c>
       <c r="F6" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G6" t="n" s="21">
-        <v>6.1649870019E8</v>
+        <v>6.1525597844E8</v>
       </c>
     </row>
     <row r="7">
@@ -1502,10 +1502,10 @@
         <v>25</v>
       </c>
       <c r="D7" t="n" s="22">
-        <v>13.642028</v>
+        <v>13.532138</v>
       </c>
       <c r="E7" t="n" s="23">
-        <v>2.4727053764E8</v>
+        <v>2.4798030072E8</v>
       </c>
       <c r="F7" t="s" s="18">
         <v>21</v>
@@ -1525,10 +1525,10 @@
         <v>27</v>
       </c>
       <c r="D8" t="n" s="25">
-        <v>4.986179</v>
+        <v>4.932452</v>
       </c>
       <c r="E8" t="n" s="26">
-        <v>9.037770801E7</v>
+        <v>9.038858913E7</v>
       </c>
       <c r="F8" t="s" s="18">
         <v>21</v>
@@ -1548,16 +1548,16 @@
         <v>29</v>
       </c>
       <c r="D9" t="n" s="28">
-        <v>4.55003</v>
+        <v>4.806679</v>
       </c>
       <c r="E9" t="n" s="29">
-        <v>8.24722275E7</v>
+        <v>8.808376156E7</v>
       </c>
       <c r="F9" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G9" t="n" s="30">
-        <v>8.24722275E7</v>
+        <v>8.808376156E7</v>
       </c>
     </row>
     <row r="10">
@@ -1565,45 +1565,45 @@
         <v>30</v>
       </c>
       <c r="B10" t="s" s="18">
+        <v>21</v>
+      </c>
+      <c r="C10" t="s" s="18">
         <v>31</v>
       </c>
-      <c r="C10" t="s" s="18">
-        <v>32</v>
-      </c>
       <c r="D10" t="n" s="31">
-        <v>4.294664</v>
+        <v>4.27034</v>
       </c>
       <c r="E10" t="n" s="32">
-        <v>7.7843542E7</v>
+        <v>7.825520553E7</v>
       </c>
       <c r="F10" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G10" t="n" s="33">
-        <v>1512700.0</v>
+        <v>8.3651722E7</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="18">
+        <v>32</v>
+      </c>
+      <c r="B11" t="s" s="18">
         <v>33</v>
-      </c>
-      <c r="B11" t="s" s="18">
-        <v>21</v>
       </c>
       <c r="C11" t="s" s="18">
         <v>34</v>
       </c>
       <c r="D11" t="n" s="34">
-        <v>4.290998</v>
+        <v>4.238796</v>
       </c>
       <c r="E11" t="n" s="35">
-        <v>7.777710383E7</v>
+        <v>7.7677145E7</v>
       </c>
       <c r="F11" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G11" t="n" s="36">
-        <v>8.3626026E7</v>
+        <v>1512700.0</v>
       </c>
     </row>
     <row r="12">
@@ -1617,16 +1617,16 @@
         <v>36</v>
       </c>
       <c r="D12" t="n" s="37">
-        <v>4.198752</v>
+        <v>4.179115</v>
       </c>
       <c r="E12" t="n" s="38">
-        <v>7.610507591E7</v>
+        <v>7.658347204E7</v>
       </c>
       <c r="F12" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G12" t="n" s="39">
-        <v>8.2535424E7</v>
+        <v>8.2561088E7</v>
       </c>
     </row>
     <row r="13">
@@ -1640,16 +1640,16 @@
         <v>38</v>
       </c>
       <c r="D13" t="n" s="40">
-        <v>4.012393</v>
+        <v>3.99187</v>
       </c>
       <c r="E13" t="n" s="41">
-        <v>7.272720194E7</v>
+        <v>7.315216595E7</v>
       </c>
       <c r="F13" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G13" t="n" s="42">
-        <v>7.6397881E7</v>
+        <v>7.6420953E7</v>
       </c>
     </row>
     <row r="14">
@@ -1663,16 +1663,16 @@
         <v>40</v>
       </c>
       <c r="D14" t="n" s="43">
-        <v>3.700998</v>
+        <v>3.681213</v>
       </c>
       <c r="E14" t="n" s="44">
-        <v>6.708296213E7</v>
+        <v>6.74592892E7</v>
       </c>
       <c r="F14" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G14" t="n" s="45">
-        <v>7.12154025E7</v>
+        <v>7.12367865E7</v>
       </c>
     </row>
     <row r="15">
@@ -1686,16 +1686,16 @@
         <v>42</v>
       </c>
       <c r="D15" t="n" s="46">
-        <v>3.527187</v>
+        <v>3.50685</v>
       </c>
       <c r="E15" t="n" s="47">
-        <v>6.39325284E7</v>
+        <v>6.426402575E7</v>
       </c>
       <c r="F15" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G15" t="n" s="48">
-        <v>6.82686543E7</v>
+        <v>6.828936345E7</v>
       </c>
     </row>
     <row r="16">
@@ -1709,10 +1709,10 @@
         <v>45</v>
       </c>
       <c r="D16" t="n" s="49">
-        <v>3.272637</v>
+        <v>3.248094</v>
       </c>
       <c r="E16" t="n" s="50">
-        <v>5.931865471E7</v>
+        <v>5.952225762E7</v>
       </c>
       <c r="F16" t="s" s="18">
         <v>21</v>
@@ -1732,16 +1732,16 @@
         <v>47</v>
       </c>
       <c r="D17" t="n" s="52">
-        <v>2.537945</v>
+        <v>2.526687</v>
       </c>
       <c r="E17" t="n" s="53">
-        <v>4.6001889E7</v>
+        <v>4.630226563E7</v>
       </c>
       <c r="F17" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G17" t="n" s="54">
-        <v>4.7861184E7</v>
+        <v>4.7876002E7</v>
       </c>
     </row>
     <row r="18">
@@ -1755,16 +1755,16 @@
         <v>49</v>
       </c>
       <c r="D18" t="n" s="55">
-        <v>1.487195</v>
+        <v>1.486549</v>
       </c>
       <c r="E18" t="n" s="56">
-        <v>2.695635862E7</v>
+        <v>2.72414279E7</v>
       </c>
       <c r="F18" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G18" t="n" s="57">
-        <v>3.55978842E7</v>
+        <v>3.56088006E7</v>
       </c>
     </row>
     <row r="19">
@@ -1778,16 +1778,16 @@
         <v>51</v>
       </c>
       <c r="D19" t="n" s="58">
-        <v>1.315478</v>
+        <v>1.316434</v>
       </c>
       <c r="E19" t="n" s="59">
-        <v>2.384388465E7</v>
+        <v>2.412402486E7</v>
       </c>
       <c r="F19" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G19" t="n" s="60">
-        <v>3.62612321E7</v>
+        <v>3.62724675E7</v>
       </c>
     </row>
     <row r="20">
@@ -1801,16 +1801,16 @@
         <v>53</v>
       </c>
       <c r="D20" t="n" s="61">
-        <v>1.236497</v>
+        <v>1.240091</v>
       </c>
       <c r="E20" t="n" s="62">
-        <v>2.241229962E7</v>
+        <v>2.272502727E7</v>
       </c>
       <c r="F20" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G20" t="n" s="63">
-        <v>2.68429609E7</v>
+        <v>2.68513198E7</v>
       </c>
     </row>
     <row r="21">
@@ -1824,16 +1824,16 @@
         <v>55</v>
       </c>
       <c r="D21" t="n" s="64">
-        <v>1.164134</v>
+        <v>1.166791</v>
       </c>
       <c r="E21" t="n" s="65">
-        <v>2.110067158E7</v>
+        <v>2.138178809E7</v>
       </c>
       <c r="F21" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G21" t="n" s="66">
-        <v>2.66129915E7</v>
+        <v>2.6621296E7</v>
       </c>
     </row>
     <row r="22">
@@ -1847,16 +1847,16 @@
         <v>57</v>
       </c>
       <c r="D22" t="n" s="67">
-        <v>1.140199</v>
+        <v>1.143677</v>
       </c>
       <c r="E22" t="n" s="68">
-        <v>2.06668318E7</v>
+        <v>2.095820603E7</v>
       </c>
       <c r="F22" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G22" t="n" s="69">
-        <v>2.476344E7</v>
+        <v>2.477112E7</v>
       </c>
     </row>
     <row r="23">
@@ -1870,16 +1870,16 @@
         <v>59</v>
       </c>
       <c r="D23" t="n" s="70">
-        <v>1.104858</v>
+        <v>1.103968</v>
       </c>
       <c r="E23" t="n" s="71">
-        <v>2.00262657E7</v>
+        <v>2.023053712E7</v>
       </c>
       <c r="F23" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G23" t="n" s="72">
-        <v>2.82363012E7</v>
+        <v>2.8245078E7</v>
       </c>
     </row>
     <row r="24">
@@ -1893,16 +1893,16 @@
         <v>61</v>
       </c>
       <c r="D24" t="n" s="73">
-        <v>0.953014</v>
+        <v>0.956022</v>
       </c>
       <c r="E24" t="n" s="74">
-        <v>1.727399154E7</v>
+        <v>1.751937148E7</v>
       </c>
       <c r="F24" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G24" t="n" s="75">
-        <v>2.5086608E7</v>
+        <v>2.509419E7</v>
       </c>
     </row>
     <row r="25">
@@ -1916,16 +1916,16 @@
         <v>63</v>
       </c>
       <c r="D25" t="n" s="76">
-        <v>0.932894</v>
+        <v>0.932579</v>
       </c>
       <c r="E25" t="n" s="77">
-        <v>1.690929684E7</v>
+        <v>1.70897746E7</v>
       </c>
       <c r="F25" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G25" t="n" s="78">
-        <v>2.50023393E7</v>
+        <v>2.50099029E7</v>
       </c>
     </row>
     <row r="26">
@@ -1939,16 +1939,16 @@
         <v>65</v>
       </c>
       <c r="D26" t="n" s="79">
-        <v>0.887747</v>
+        <v>0.889344</v>
       </c>
       <c r="E26" t="n" s="80">
-        <v>1.609099305E7</v>
+        <v>1.629748272E7</v>
       </c>
       <c r="F26" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G26" t="n" s="81">
-        <v>2.48659555E7</v>
+        <v>2.48734945E7</v>
       </c>
     </row>
     <row r="27">
@@ -1962,16 +1962,16 @@
         <v>67</v>
       </c>
       <c r="D27" t="n" s="82">
-        <v>0.733748</v>
+        <v>0.734559</v>
       </c>
       <c r="E27" t="n" s="83">
-        <v>1.329965952E7</v>
+        <v>1.346100504E7</v>
       </c>
       <c r="F27" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G27" t="n" s="84">
-        <v>1.95887052E7</v>
+        <v>1.95946736E7</v>
       </c>
     </row>
     <row r="28">
@@ -1985,16 +1985,16 @@
         <v>69</v>
       </c>
       <c r="D28" t="n" s="85">
-        <v>0.724999</v>
+        <v>0.729371</v>
       </c>
       <c r="E28" t="n" s="86">
-        <v>1.31410673E7</v>
+        <v>1.336593382E7</v>
       </c>
       <c r="F28" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G28" t="n" s="87">
-        <v>2.8469625E7</v>
+        <v>2.8478394E7</v>
       </c>
     </row>
     <row r="29">
@@ -2008,16 +2008,16 @@
         <v>71</v>
       </c>
       <c r="D29" t="n" s="88">
-        <v>0.716726</v>
+        <v>0.719798</v>
       </c>
       <c r="E29" t="n" s="89">
-        <v>1.299111731E7</v>
+        <v>1.319050523E7</v>
       </c>
       <c r="F29" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G29" t="n" s="90">
-        <v>2.55128382E7</v>
+        <v>2.55206842E7</v>
       </c>
     </row>
     <row r="30">
@@ -2031,16 +2031,16 @@
         <v>73</v>
       </c>
       <c r="D30" t="n" s="91">
-        <v>0.605353</v>
+        <v>0.608685</v>
       </c>
       <c r="E30" t="n" s="92">
-        <v>1.097241873E7</v>
+        <v>1.115432043E7</v>
       </c>
       <c r="F30" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G30" t="n" s="93">
-        <v>2.30808477E7</v>
+        <v>2.3087856E7</v>
       </c>
     </row>
     <row r="31">
@@ -2054,16 +2054,16 @@
         <v>75</v>
       </c>
       <c r="D31" t="n" s="94">
-        <v>0.571712</v>
+        <v>0.572831</v>
       </c>
       <c r="E31" t="n" s="95">
-        <v>1.036265069E7</v>
+        <v>1.049728947E7</v>
       </c>
       <c r="F31" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G31" t="n" s="96">
-        <v>1.5865785E7</v>
+        <v>1.5870699E7</v>
       </c>
     </row>
     <row r="32">
@@ -2077,16 +2077,16 @@
         <v>77</v>
       </c>
       <c r="D32" t="n" s="97">
-        <v>0.559514</v>
+        <v>0.560874</v>
       </c>
       <c r="E32" t="n" s="98">
-        <v>1.014155745E7</v>
+        <v>1.027818531E7</v>
       </c>
       <c r="F32" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G32" t="n" s="99">
-        <v>1.57806875E7</v>
+        <v>1.578555625E7</v>
       </c>
     </row>
     <row r="33">
@@ -2100,10 +2100,10 @@
         <v>21</v>
       </c>
       <c r="D33" t="n" s="100">
-        <v>0.403682</v>
+        <v>0.373675</v>
       </c>
       <c r="E33" t="n" s="101">
-        <v>7316994.33</v>
+        <v>6847704.46</v>
       </c>
       <c r="F33" t="n" s="102">
         <v>4.1426456199E8</v>
@@ -2123,10 +2123,10 @@
         <v>80</v>
       </c>
       <c r="D34" t="n" s="104">
-        <v>0.266745</v>
+        <v>0.265725</v>
       </c>
       <c r="E34" t="n" s="105">
-        <v>4834927.07</v>
+        <v>4869489.46</v>
       </c>
       <c r="F34" t="s" s="18">
         <v>21</v>
@@ -2146,10 +2146,10 @@
         <v>82</v>
       </c>
       <c r="D35" t="n" s="107">
-        <v>0.147613</v>
+        <v>0.147037</v>
       </c>
       <c r="E35" t="n" s="108">
-        <v>2675585.06</v>
+        <v>2694493.47</v>
       </c>
       <c r="F35" t="s" s="18">
         <v>21</v>
@@ -2169,16 +2169,16 @@
         <v>85</v>
       </c>
       <c r="D36" t="n" s="110">
-        <v>0.107519</v>
+        <v>0.117514</v>
       </c>
       <c r="E36" t="n" s="111">
-        <v>8.761977904E7</v>
+        <v>1.7085466184E8</v>
       </c>
       <c r="F36" t="n" s="112">
-        <v>8.761977904E7</v>
+        <v>1.7085466184E8</v>
       </c>
       <c r="G36" t="n" s="113">
-        <v>3380000.0</v>
+        <v>2.331E8</v>
       </c>
     </row>
     <row r="37">
@@ -2192,16 +2192,16 @@
         <v>88</v>
       </c>
       <c r="D37" t="n" s="114">
-        <v>0.048311</v>
+        <v>0.037387</v>
       </c>
       <c r="E37" t="n" s="115">
-        <v>1.704787713E8</v>
+        <v>7.295317453E7</v>
       </c>
       <c r="F37" t="n" s="116">
-        <v>1.704787713E8</v>
+        <v>7.295317453E7</v>
       </c>
       <c r="G37" t="n" s="117">
-        <v>2.331E8</v>
+        <v>5060.0</v>
       </c>
     </row>
     <row r="38">
@@ -2215,13 +2215,13 @@
         <v>91</v>
       </c>
       <c r="D38" t="n" s="118">
-        <v>9.25E-4</v>
+        <v>0.003409</v>
       </c>
       <c r="E38" t="n" s="119">
-        <v>6.708943623E7</v>
+        <v>6.677845462E7</v>
       </c>
       <c r="F38" t="n" s="120">
-        <v>6.708943623E7</v>
+        <v>6.677845462E7</v>
       </c>
       <c r="G38" t="n" s="121">
         <v>11025.0</v>
@@ -2241,7 +2241,7 @@
         <v>0.0</v>
       </c>
       <c r="E39" t="n" s="123">
-        <v>7.41</v>
+        <v>7.45</v>
       </c>
       <c r="F39" t="s" s="18">
         <v>21</v>
@@ -2261,16 +2261,16 @@
         <v>96</v>
       </c>
       <c r="D40" t="n" s="125">
-        <v>-0.00269</v>
+        <v>-0.005136</v>
       </c>
       <c r="E40" t="n" s="126">
-        <v>7.17121578E7</v>
+        <v>3.3509145061E8</v>
       </c>
       <c r="F40" t="n" s="127">
-        <v>7.17121578E7</v>
+        <v>3.3509145061E8</v>
       </c>
       <c r="G40" t="n" s="128">
-        <v>5060.0</v>
+        <v>2.459E8</v>
       </c>
     </row>
     <row r="41">
@@ -2284,10 +2284,10 @@
         <v>98</v>
       </c>
       <c r="D41" t="n" s="129">
-        <v>-0.006833</v>
+        <v>-0.006722</v>
       </c>
       <c r="E41" t="n" s="130">
-        <v>-123844.78</v>
+        <v>-123186.2</v>
       </c>
       <c r="F41" t="s" s="18">
         <v>21</v>
@@ -2307,10 +2307,10 @@
         <v>100</v>
       </c>
       <c r="D42" t="n" s="132">
-        <v>-0.007786</v>
+        <v>-0.007739</v>
       </c>
       <c r="E42" t="n" s="133">
-        <v>-141124.33</v>
+        <v>-141811.72</v>
       </c>
       <c r="F42" t="s" s="18">
         <v>21</v>
@@ -2330,16 +2330,16 @@
         <v>103</v>
       </c>
       <c r="D43" t="n" s="135">
-        <v>-0.076201</v>
+        <v>-0.013309</v>
       </c>
       <c r="E43" t="n" s="136">
-        <v>1.6503234689E8</v>
+        <v>8.584432426E7</v>
       </c>
       <c r="F43" t="n" s="137">
-        <v>1.6503234689E8</v>
+        <v>8.584432426E7</v>
       </c>
       <c r="G43" t="n" s="138">
-        <v>23880.0</v>
+        <v>3380000.0</v>
       </c>
     </row>
     <row r="44">
@@ -2353,16 +2353,16 @@
         <v>106</v>
       </c>
       <c r="D44" t="n" s="139">
-        <v>-0.110771</v>
+        <v>-0.108435</v>
       </c>
       <c r="E44" t="n" s="140">
-        <v>3.3079871302E8</v>
+        <v>1.1790867602E8</v>
       </c>
       <c r="F44" t="n" s="141">
-        <v>3.3079871302E8</v>
+        <v>1.1790867602E8</v>
       </c>
       <c r="G44" t="n" s="142">
-        <v>2.459E8</v>
+        <v>1.051E8</v>
       </c>
     </row>
     <row r="45">
@@ -2376,16 +2376,16 @@
         <v>109</v>
       </c>
       <c r="D45" t="n" s="143">
-        <v>-0.166084</v>
+        <v>-0.122617</v>
       </c>
       <c r="E45" t="n" s="144">
-        <v>1.160440415E8</v>
+        <v>1.6535614157E8</v>
       </c>
       <c r="F45" t="n" s="145">
-        <v>1.160440415E8</v>
+        <v>1.6535614157E8</v>
       </c>
       <c r="G45" t="n" s="146">
-        <v>1.051E8</v>
+        <v>23880.0</v>
       </c>
     </row>
     <row r="46">
@@ -2399,13 +2399,13 @@
         <v>112</v>
       </c>
       <c r="D46" t="n" s="147">
-        <v>-0.501943</v>
+        <v>-0.370487</v>
       </c>
       <c r="E46" t="n" s="148">
-        <v>1.924343125E8</v>
+        <v>1.947430625E8</v>
       </c>
       <c r="F46" t="n" s="149">
-        <v>1.924343125E8</v>
+        <v>1.947430625E8</v>
       </c>
       <c r="G46" t="n" s="150">
         <v>1.847E8</v>
@@ -2422,13 +2422,13 @@
         <v>115</v>
       </c>
       <c r="D47" t="n" s="151">
-        <v>-0.576195</v>
+        <v>-0.429737</v>
       </c>
       <c r="E47" t="n" s="152">
-        <v>1.6965627E8</v>
+        <v>1.7222513E8</v>
       </c>
       <c r="F47" t="n" s="153">
-        <v>1.6965627E8</v>
+        <v>1.7222513E8</v>
       </c>
       <c r="G47" t="n" s="154">
         <v>41300.0</v>
@@ -2445,13 +2445,13 @@
         <v>118</v>
       </c>
       <c r="D48" t="n" s="155">
-        <v>-0.752497</v>
+        <v>-0.588807</v>
       </c>
       <c r="E48" t="n" s="156">
-        <v>4.5536725E8</v>
+        <v>4.582166875E8</v>
       </c>
       <c r="F48" t="n" s="157">
-        <v>4.5536725E8</v>
+        <v>4.582166875E8</v>
       </c>
       <c r="G48" t="n" s="158">
         <v>4.342E8</v>

</xml_diff>

<commit_message>
Update ALLW XLSX 2026-10-19
</commit_message>
<xml_diff>
--- a/latest/allw-latest.xlsx
+++ b/latest/allw-latest.xlsx
@@ -192,7 +192,7 @@
     <t>ALLW</t>
   </si>
   <si>
-    <t>As of 15-Oct-2026</t>
+    <t>As of 16-Oct-2026</t>
   </si>
   <si>
     <t>Name</t>
@@ -240,33 +240,33 @@
     <t>912797TV9</t>
   </si>
   <si>
+    <t>TSY INFL IX N/B 07/35 1.875</t>
+  </si>
+  <si>
+    <t>91282CNS6</t>
+  </si>
+  <si>
+    <t>TSY INFL IX N/B 01/36 1.875</t>
+  </si>
+  <si>
+    <t>91282CPU9</t>
+  </si>
+  <si>
+    <t>STATE STREET SPDR PORTFOLIO EM</t>
+  </si>
+  <si>
+    <t>SPEM</t>
+  </si>
+  <si>
+    <t>78463X509</t>
+  </si>
+  <si>
     <t>US DOLLAR</t>
   </si>
   <si>
     <t>999USDZ92</t>
   </si>
   <si>
-    <t>TSY INFL IX N/B 07/35 1.875</t>
-  </si>
-  <si>
-    <t>91282CNS6</t>
-  </si>
-  <si>
-    <t>STATE STREET SPDR PORTFOLIO EM</t>
-  </si>
-  <si>
-    <t>SPEM</t>
-  </si>
-  <si>
-    <t>78463X509</t>
-  </si>
-  <si>
-    <t>TSY INFL IX N/B 01/36 1.875</t>
-  </si>
-  <si>
-    <t>91282CPU9</t>
-  </si>
-  <si>
     <t>TSY INFL IX N/B 01/35 2.125</t>
   </si>
   <si>
@@ -414,6 +414,15 @@
     <t>ADI3BDHZ1</t>
   </si>
   <si>
+    <t>TOPIX INDX FUTR   DEC26</t>
+  </si>
+  <si>
+    <t>TPZ6</t>
+  </si>
+  <si>
+    <t>ADI3917X6</t>
+  </si>
+  <si>
     <t>FTSE 100 IDX FUT  DEC26</t>
   </si>
   <si>
@@ -438,6 +447,18 @@
     <t>999CADZ91</t>
   </si>
   <si>
+    <t>AUSTRALIAN DOLLAR</t>
+  </si>
+  <si>
+    <t>999AUDZ93</t>
+  </si>
+  <si>
+    <t>JAPANESE YEN</t>
+  </si>
+  <si>
+    <t>999JPYZ94</t>
+  </si>
+  <si>
     <t>EURO-BUND FUTURE  DEC26</t>
   </si>
   <si>
@@ -447,25 +468,13 @@
     <t>ADI39K4N9</t>
   </si>
   <si>
-    <t>AUSTRALIAN DOLLAR</t>
-  </si>
-  <si>
-    <t>999AUDZ93</t>
-  </si>
-  <si>
-    <t>JAPANESE YEN</t>
-  </si>
-  <si>
-    <t>999JPYZ94</t>
-  </si>
-  <si>
-    <t>TOPIX INDX FUTR   DEC26</t>
-  </si>
-  <si>
-    <t>TPZ6</t>
-  </si>
-  <si>
-    <t>ADI3917X6</t>
+    <t>EURO STOXX 50     DEC26</t>
+  </si>
+  <si>
+    <t>VGZ6</t>
+  </si>
+  <si>
+    <t>ADI2VHXS0</t>
   </si>
   <si>
     <t>LONG GILT FUTURE  DEC26</t>
@@ -475,15 +484,6 @@
   </si>
   <si>
     <t>ADI3BKVP1</t>
-  </si>
-  <si>
-    <t>EURO STOXX 50     DEC26</t>
-  </si>
-  <si>
-    <t>VGZ6</t>
-  </si>
-  <si>
-    <t>ADI2VHXS0</t>
   </si>
   <si>
     <t>US LONG BOND(CBT) DEC26</t>
@@ -984,13 +984,13 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
@@ -1479,16 +1479,16 @@
         <v>22</v>
       </c>
       <c r="D6" t="n" s="19">
-        <v>33.574153</v>
+        <v>34.231807</v>
       </c>
       <c r="E6" t="n" s="20">
-        <v>6.1525597844E8</v>
+        <v>6.2926325071E8</v>
       </c>
       <c r="F6" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G6" t="n" s="21">
-        <v>6.1525597844E8</v>
+        <v>6.2926325071E8</v>
       </c>
     </row>
     <row r="7">
@@ -1502,10 +1502,10 @@
         <v>25</v>
       </c>
       <c r="D7" t="n" s="22">
-        <v>13.532138</v>
+        <v>13.340095</v>
       </c>
       <c r="E7" t="n" s="23">
-        <v>2.4798030072E8</v>
+        <v>2.4522314414E8</v>
       </c>
       <c r="F7" t="s" s="18">
         <v>21</v>
@@ -1525,10 +1525,10 @@
         <v>27</v>
       </c>
       <c r="D8" t="n" s="25">
-        <v>4.932452</v>
+        <v>4.91919</v>
       </c>
       <c r="E8" t="n" s="26">
-        <v>9.038858913E7</v>
+        <v>9.042658961E7</v>
       </c>
       <c r="F8" t="s" s="18">
         <v>21</v>
@@ -1548,16 +1548,16 @@
         <v>29</v>
       </c>
       <c r="D9" t="n" s="28">
-        <v>4.806679</v>
+        <v>4.270141</v>
       </c>
       <c r="E9" t="n" s="29">
-        <v>8.808376156E7</v>
+        <v>7.849549623E7</v>
       </c>
       <c r="F9" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G9" t="n" s="30">
-        <v>8.808376156E7</v>
+        <v>8.3660555E7</v>
       </c>
     </row>
     <row r="10">
@@ -1571,16 +1571,16 @@
         <v>31</v>
       </c>
       <c r="D10" t="n" s="31">
-        <v>4.27034</v>
+        <v>4.178287</v>
       </c>
       <c r="E10" t="n" s="32">
-        <v>7.825520553E7</v>
+        <v>7.680700959E7</v>
       </c>
       <c r="F10" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G10" t="n" s="33">
-        <v>8.3651722E7</v>
+        <v>8.2569108E7</v>
       </c>
     </row>
     <row r="11">
@@ -1594,10 +1594,10 @@
         <v>34</v>
       </c>
       <c r="D11" t="n" s="34">
-        <v>4.238796</v>
+        <v>4.171311</v>
       </c>
       <c r="E11" t="n" s="35">
-        <v>7.7677145E7</v>
+        <v>7.6678763E7</v>
       </c>
       <c r="F11" t="s" s="18">
         <v>21</v>
@@ -1617,16 +1617,16 @@
         <v>36</v>
       </c>
       <c r="D12" t="n" s="37">
-        <v>4.179115</v>
+        <v>4.102548</v>
       </c>
       <c r="E12" t="n" s="38">
-        <v>7.658347204E7</v>
+        <v>7.541473772E7</v>
       </c>
       <c r="F12" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G12" t="n" s="39">
-        <v>8.2561088E7</v>
+        <v>7.541473772E7</v>
       </c>
     </row>
     <row r="13">
@@ -1640,16 +1640,16 @@
         <v>38</v>
       </c>
       <c r="D13" t="n" s="40">
-        <v>3.99187</v>
+        <v>3.991246</v>
       </c>
       <c r="E13" t="n" s="41">
-        <v>7.315216595E7</v>
+        <v>7.336874333E7</v>
       </c>
       <c r="F13" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G13" t="n" s="42">
-        <v>7.6420953E7</v>
+        <v>7.6428884E7</v>
       </c>
     </row>
     <row r="14">
@@ -1663,16 +1663,16 @@
         <v>40</v>
       </c>
       <c r="D14" t="n" s="43">
-        <v>3.681213</v>
+        <v>3.681658</v>
       </c>
       <c r="E14" t="n" s="44">
-        <v>6.74592892E7</v>
+        <v>6.767775619E7</v>
       </c>
       <c r="F14" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G14" t="n" s="45">
-        <v>7.12367865E7</v>
+        <v>7.124413725E7</v>
       </c>
     </row>
     <row r="15">
@@ -1686,16 +1686,16 @@
         <v>42</v>
       </c>
       <c r="D15" t="n" s="46">
-        <v>3.50685</v>
+        <v>3.506464</v>
       </c>
       <c r="E15" t="n" s="47">
-        <v>6.426402575E7</v>
+        <v>6.445726916E7</v>
       </c>
       <c r="F15" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G15" t="n" s="48">
-        <v>6.828936345E7</v>
+        <v>6.82962665E7</v>
       </c>
     </row>
     <row r="16">
@@ -1709,10 +1709,10 @@
         <v>45</v>
       </c>
       <c r="D16" t="n" s="49">
-        <v>3.248094</v>
+        <v>3.209737</v>
       </c>
       <c r="E16" t="n" s="50">
-        <v>5.952225762E7</v>
+        <v>5.900271916E7</v>
       </c>
       <c r="F16" t="s" s="18">
         <v>21</v>
@@ -1732,16 +1732,16 @@
         <v>47</v>
       </c>
       <c r="D17" t="n" s="52">
-        <v>2.526687</v>
+        <v>2.526514</v>
       </c>
       <c r="E17" t="n" s="53">
-        <v>4.630226563E7</v>
+        <v>4.644342343E7</v>
       </c>
       <c r="F17" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G17" t="n" s="54">
-        <v>4.7876002E7</v>
+        <v>4.7880782E7</v>
       </c>
     </row>
     <row r="18">
@@ -1755,16 +1755,16 @@
         <v>49</v>
       </c>
       <c r="D18" t="n" s="55">
-        <v>1.486549</v>
+        <v>1.48583</v>
       </c>
       <c r="E18" t="n" s="56">
-        <v>2.72414279E7</v>
+        <v>2.731313529E7</v>
       </c>
       <c r="F18" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G18" t="n" s="57">
-        <v>3.56088006E7</v>
+        <v>3.56125221E7</v>
       </c>
     </row>
     <row r="19">
@@ -1778,16 +1778,16 @@
         <v>51</v>
       </c>
       <c r="D19" t="n" s="58">
-        <v>1.316434</v>
+        <v>1.316249</v>
       </c>
       <c r="E19" t="n" s="59">
-        <v>2.412402486E7</v>
+        <v>2.419583696E7</v>
       </c>
       <c r="F19" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G19" t="n" s="60">
-        <v>3.62724675E7</v>
+        <v>3.62760424E7</v>
       </c>
     </row>
     <row r="20">
@@ -1801,16 +1801,16 @@
         <v>53</v>
       </c>
       <c r="D20" t="n" s="61">
-        <v>1.240091</v>
+        <v>1.239504</v>
       </c>
       <c r="E20" t="n" s="62">
-        <v>2.272502727E7</v>
+        <v>2.278507957E7</v>
       </c>
       <c r="F20" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G20" t="n" s="63">
-        <v>2.68513198E7</v>
+        <v>2.68541061E7</v>
       </c>
     </row>
     <row r="21">
@@ -1824,16 +1824,16 @@
         <v>55</v>
       </c>
       <c r="D21" t="n" s="64">
-        <v>1.166791</v>
+        <v>1.16614</v>
       </c>
       <c r="E21" t="n" s="65">
-        <v>2.138178809E7</v>
+        <v>2.143646611E7</v>
       </c>
       <c r="F21" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G21" t="n" s="66">
-        <v>2.6621296E7</v>
+        <v>2.662398275E7</v>
       </c>
     </row>
     <row r="22">
@@ -1847,16 +1847,16 @@
         <v>57</v>
       </c>
       <c r="D22" t="n" s="67">
-        <v>1.143677</v>
+        <v>1.143102</v>
       </c>
       <c r="E22" t="n" s="68">
-        <v>2.095820603E7</v>
+        <v>2.101297721E7</v>
       </c>
       <c r="F22" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G22" t="n" s="69">
-        <v>2.477112E7</v>
+        <v>2.477352E7</v>
       </c>
     </row>
     <row r="23">
@@ -1870,16 +1870,16 @@
         <v>59</v>
       </c>
       <c r="D23" t="n" s="70">
-        <v>1.103968</v>
+        <v>1.10335</v>
       </c>
       <c r="E23" t="n" s="71">
-        <v>2.023053712E7</v>
+        <v>2.028224154E7</v>
       </c>
       <c r="F23" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G23" t="n" s="72">
-        <v>2.8245078E7</v>
+        <v>2.824794E7</v>
       </c>
     </row>
     <row r="24">
@@ -1893,16 +1893,16 @@
         <v>61</v>
       </c>
       <c r="D24" t="n" s="73">
-        <v>0.956022</v>
+        <v>0.955659</v>
       </c>
       <c r="E24" t="n" s="74">
-        <v>1.751937148E7</v>
+        <v>1.756731606E7</v>
       </c>
       <c r="F24" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G24" t="n" s="75">
-        <v>2.509419E7</v>
+        <v>2.5096866E7</v>
       </c>
     </row>
     <row r="25">
@@ -1916,16 +1916,16 @@
         <v>63</v>
       </c>
       <c r="D25" t="n" s="76">
-        <v>0.932579</v>
+        <v>0.932062</v>
       </c>
       <c r="E25" t="n" s="77">
-        <v>1.70897746E7</v>
+        <v>1.713354976E7</v>
       </c>
       <c r="F25" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G25" t="n" s="78">
-        <v>2.50099029E7</v>
+        <v>2.50124814E7</v>
       </c>
     </row>
     <row r="26">
@@ -1939,16 +1939,16 @@
         <v>65</v>
       </c>
       <c r="D26" t="n" s="79">
-        <v>0.889344</v>
+        <v>0.889022</v>
       </c>
       <c r="E26" t="n" s="80">
-        <v>1.629748272E7</v>
+        <v>1.634237099E7</v>
       </c>
       <c r="F26" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G26" t="n" s="81">
-        <v>2.48734945E7</v>
+        <v>2.48760075E7</v>
       </c>
     </row>
     <row r="27">
@@ -1962,16 +1962,16 @@
         <v>67</v>
       </c>
       <c r="D27" t="n" s="82">
-        <v>0.734559</v>
+        <v>0.733978</v>
       </c>
       <c r="E27" t="n" s="83">
-        <v>1.346100504E7</v>
+        <v>1.349228961E7</v>
       </c>
       <c r="F27" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G27" t="n" s="84">
-        <v>1.95946736E7</v>
+        <v>1.95967556E7</v>
       </c>
     </row>
     <row r="28">
@@ -1985,16 +1985,16 @@
         <v>69</v>
       </c>
       <c r="D28" t="n" s="85">
-        <v>0.729371</v>
+        <v>0.729356</v>
       </c>
       <c r="E28" t="n" s="86">
-        <v>1.336593382E7</v>
+        <v>1.340732035E7</v>
       </c>
       <c r="F28" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G28" t="n" s="87">
-        <v>2.8478394E7</v>
+        <v>2.8481238E7</v>
       </c>
     </row>
     <row r="29">
@@ -2008,16 +2008,16 @@
         <v>71</v>
       </c>
       <c r="D29" t="n" s="88">
-        <v>0.719798</v>
+        <v>0.719884</v>
       </c>
       <c r="E29" t="n" s="89">
-        <v>1.319050523E7</v>
+        <v>1.323319864E7</v>
       </c>
       <c r="F29" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G29" t="n" s="90">
-        <v>2.55206842E7</v>
+        <v>2.552323415E7</v>
       </c>
     </row>
     <row r="30">
@@ -2031,16 +2031,16 @@
         <v>73</v>
       </c>
       <c r="D30" t="n" s="91">
-        <v>0.608685</v>
+        <v>0.608621</v>
       </c>
       <c r="E30" t="n" s="92">
-        <v>1.115432043E7</v>
+        <v>1.118791964E7</v>
       </c>
       <c r="F30" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G30" t="n" s="93">
-        <v>2.3087856E7</v>
+        <v>2.30901921E7</v>
       </c>
     </row>
     <row r="31">
@@ -2054,16 +2054,16 @@
         <v>75</v>
       </c>
       <c r="D31" t="n" s="94">
-        <v>0.572831</v>
+        <v>0.572678</v>
       </c>
       <c r="E31" t="n" s="95">
-        <v>1.049728947E7</v>
+        <v>1.052720355E7</v>
       </c>
       <c r="F31" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G31" t="n" s="96">
-        <v>1.5870699E7</v>
+        <v>1.5872337E7</v>
       </c>
     </row>
     <row r="32">
@@ -2077,16 +2077,16 @@
         <v>77</v>
       </c>
       <c r="D32" t="n" s="97">
-        <v>0.560874</v>
+        <v>0.560562</v>
       </c>
       <c r="E32" t="n" s="98">
-        <v>1.027818531E7</v>
+        <v>1.030447445E7</v>
       </c>
       <c r="F32" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G32" t="n" s="99">
-        <v>1.578555625E7</v>
+        <v>1.57871E7</v>
       </c>
     </row>
     <row r="33">
@@ -2100,10 +2100,10 @@
         <v>21</v>
       </c>
       <c r="D33" t="n" s="100">
-        <v>0.373675</v>
+        <v>0.459146</v>
       </c>
       <c r="E33" t="n" s="101">
-        <v>6847704.46</v>
+        <v>8440220.12</v>
       </c>
       <c r="F33" t="n" s="102">
         <v>4.1426456199E8</v>
@@ -2123,16 +2123,16 @@
         <v>80</v>
       </c>
       <c r="D34" t="n" s="104">
-        <v>0.265725</v>
+        <v>0.26612</v>
       </c>
       <c r="E34" t="n" s="105">
-        <v>4869489.46</v>
+        <v>4891919.6</v>
       </c>
       <c r="F34" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G34" t="n" s="106">
-        <v>4347368.19</v>
+        <v>4347214.14</v>
       </c>
     </row>
     <row r="35">
@@ -2146,16 +2146,16 @@
         <v>82</v>
       </c>
       <c r="D35" t="n" s="107">
-        <v>0.147037</v>
+        <v>0.147702</v>
       </c>
       <c r="E35" t="n" s="108">
-        <v>2694493.47</v>
+        <v>2715127.96</v>
       </c>
       <c r="F35" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G35" t="n" s="109">
-        <v>2033351.0</v>
+        <v>2033345.75</v>
       </c>
     </row>
     <row r="36">
@@ -2169,13 +2169,13 @@
         <v>85</v>
       </c>
       <c r="D36" t="n" s="110">
-        <v>0.117514</v>
+        <v>0.107328</v>
       </c>
       <c r="E36" t="n" s="111">
-        <v>1.7085466184E8</v>
+        <v>1.7175882627E8</v>
       </c>
       <c r="F36" t="n" s="112">
-        <v>1.7085466184E8</v>
+        <v>1.7175882627E8</v>
       </c>
       <c r="G36" t="n" s="113">
         <v>2.331E8</v>
@@ -2192,16 +2192,16 @@
         <v>88</v>
       </c>
       <c r="D37" t="n" s="114">
-        <v>0.037387</v>
+        <v>0.064143</v>
       </c>
       <c r="E37" t="n" s="115">
-        <v>7.295317453E7</v>
+        <v>8.735180143E7</v>
       </c>
       <c r="F37" t="n" s="116">
-        <v>7.295317453E7</v>
+        <v>8.735180143E7</v>
       </c>
       <c r="G37" t="n" s="117">
-        <v>5060.0</v>
+        <v>3380000.0</v>
       </c>
     </row>
     <row r="38">
@@ -2215,16 +2215,16 @@
         <v>91</v>
       </c>
       <c r="D38" t="n" s="118">
-        <v>0.003409</v>
+        <v>0.052626</v>
       </c>
       <c r="E38" t="n" s="119">
-        <v>6.677845462E7</v>
+        <v>7.378906255E7</v>
       </c>
       <c r="F38" t="n" s="120">
-        <v>6.677845462E7</v>
+        <v>7.378906255E7</v>
       </c>
       <c r="G38" t="n" s="121">
-        <v>11025.0</v>
+        <v>5060.0</v>
       </c>
     </row>
     <row r="39">
@@ -2232,45 +2232,45 @@
         <v>92</v>
       </c>
       <c r="B39" t="s" s="18">
-        <v>21</v>
+        <v>93</v>
       </c>
       <c r="C39" t="s" s="18">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D39" t="n" s="122">
-        <v>0.0</v>
+        <v>0.03935</v>
       </c>
       <c r="E39" t="n" s="123">
-        <v>7.45</v>
-      </c>
-      <c r="F39" t="s" s="18">
-        <v>21</v>
-      </c>
-      <c r="G39" t="n" s="124">
-        <v>10.58</v>
+        <v>6.786829592E7</v>
+      </c>
+      <c r="F39" t="n" s="124">
+        <v>6.786829592E7</v>
+      </c>
+      <c r="G39" t="n" s="125">
+        <v>11025.0</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s" s="18">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B40" t="s" s="18">
-        <v>95</v>
+        <v>21</v>
       </c>
       <c r="C40" t="s" s="18">
         <v>96</v>
       </c>
-      <c r="D40" t="n" s="125">
-        <v>-0.005136</v>
-      </c>
-      <c r="E40" t="n" s="126">
-        <v>3.3509145061E8</v>
-      </c>
-      <c r="F40" t="n" s="127">
-        <v>3.3509145061E8</v>
+      <c r="D40" t="n" s="126">
+        <v>0.0</v>
+      </c>
+      <c r="E40" t="n" s="127">
+        <v>7.48</v>
+      </c>
+      <c r="F40" t="s" s="18">
+        <v>21</v>
       </c>
       <c r="G40" t="n" s="128">
-        <v>2.459E8</v>
+        <v>10.58</v>
       </c>
     </row>
     <row r="41">
@@ -2284,10 +2284,10 @@
         <v>98</v>
       </c>
       <c r="D41" t="n" s="129">
-        <v>-0.006722</v>
+        <v>-0.006744</v>
       </c>
       <c r="E41" t="n" s="130">
-        <v>-123186.2</v>
+        <v>-123978.24</v>
       </c>
       <c r="F41" t="s" s="18">
         <v>21</v>
@@ -2307,10 +2307,10 @@
         <v>100</v>
       </c>
       <c r="D42" t="n" s="132">
-        <v>-0.007739</v>
+        <v>-0.007722</v>
       </c>
       <c r="E42" t="n" s="133">
-        <v>-141811.72</v>
+        <v>-141950.9</v>
       </c>
       <c r="F42" t="s" s="18">
         <v>21</v>
@@ -2330,16 +2330,16 @@
         <v>103</v>
       </c>
       <c r="D43" t="n" s="135">
-        <v>-0.013309</v>
+        <v>-0.011082</v>
       </c>
       <c r="E43" t="n" s="136">
-        <v>8.584432426E7</v>
+        <v>3.3858909899E8</v>
       </c>
       <c r="F43" t="n" s="137">
-        <v>8.584432426E7</v>
+        <v>3.3858909899E8</v>
       </c>
       <c r="G43" t="n" s="138">
-        <v>3380000.0</v>
+        <v>2.474E8</v>
       </c>
     </row>
     <row r="44">
@@ -2353,16 +2353,16 @@
         <v>106</v>
       </c>
       <c r="D44" t="n" s="139">
-        <v>-0.108435</v>
+        <v>-0.066771</v>
       </c>
       <c r="E44" t="n" s="140">
-        <v>1.1790867602E8</v>
+        <v>1.7417220689E8</v>
       </c>
       <c r="F44" t="n" s="141">
-        <v>1.1790867602E8</v>
+        <v>1.7417220689E8</v>
       </c>
       <c r="G44" t="n" s="142">
-        <v>1.051E8</v>
+        <v>24880.0</v>
       </c>
     </row>
     <row r="45">
@@ -2376,16 +2376,16 @@
         <v>109</v>
       </c>
       <c r="D45" t="n" s="143">
-        <v>-0.122617</v>
+        <v>-0.101986</v>
       </c>
       <c r="E45" t="n" s="144">
-        <v>1.6535614157E8</v>
+        <v>1.1950406933E8</v>
       </c>
       <c r="F45" t="n" s="145">
-        <v>1.6535614157E8</v>
+        <v>1.1950406933E8</v>
       </c>
       <c r="G45" t="n" s="146">
-        <v>23880.0</v>
+        <v>1.056E8</v>
       </c>
     </row>
     <row r="46">
@@ -2399,16 +2399,16 @@
         <v>112</v>
       </c>
       <c r="D46" t="n" s="147">
-        <v>-0.370487</v>
+        <v>-0.37218</v>
       </c>
       <c r="E46" t="n" s="148">
-        <v>1.947430625E8</v>
+        <v>2.0100971875E8</v>
       </c>
       <c r="F46" t="n" s="149">
-        <v>1.947430625E8</v>
+        <v>2.0100971875E8</v>
       </c>
       <c r="G46" t="n" s="150">
-        <v>1.847E8</v>
+        <v>1.907E8</v>
       </c>
     </row>
     <row r="47">
@@ -2422,16 +2422,16 @@
         <v>115</v>
       </c>
       <c r="D47" t="n" s="151">
-        <v>-0.429737</v>
+        <v>-0.404827</v>
       </c>
       <c r="E47" t="n" s="152">
-        <v>1.7222513E8</v>
+        <v>1.7769675E8</v>
       </c>
       <c r="F47" t="n" s="153">
-        <v>1.7222513E8</v>
+        <v>1.7769675E8</v>
       </c>
       <c r="G47" t="n" s="154">
-        <v>41300.0</v>
+        <v>42500.0</v>
       </c>
     </row>
     <row r="48">
@@ -2445,16 +2445,16 @@
         <v>118</v>
       </c>
       <c r="D48" t="n" s="155">
-        <v>-0.588807</v>
+        <v>-0.58518</v>
       </c>
       <c r="E48" t="n" s="156">
-        <v>4.582166875E8</v>
+        <v>4.4364129685E8</v>
       </c>
       <c r="F48" t="n" s="157">
-        <v>4.582166875E8</v>
+        <v>4.4364129685E8</v>
       </c>
       <c r="G48" t="n" s="158">
-        <v>4.342E8</v>
+        <v>4.207E8</v>
       </c>
     </row>
     <row r="49"/>

</xml_diff>

<commit_message>
Update ALLW XLSX 2026-10-20
</commit_message>
<xml_diff>
--- a/latest/allw-latest.xlsx
+++ b/latest/allw-latest.xlsx
@@ -192,7 +192,7 @@
     <t>ALLW</t>
   </si>
   <si>
-    <t>As of 16-Oct-2026</t>
+    <t>As of 19-Oct-2026</t>
   </si>
   <si>
     <t>Name</t>
@@ -246,19 +246,25 @@
     <t>91282CNS6</t>
   </si>
   <si>
+    <t>STATE STREET SPDR PORTFOLIO EM</t>
+  </si>
+  <si>
+    <t>SPEM</t>
+  </si>
+  <si>
+    <t>78463X509</t>
+  </si>
+  <si>
     <t>TSY INFL IX N/B 01/36 1.875</t>
   </si>
   <si>
     <t>91282CPU9</t>
   </si>
   <si>
-    <t>STATE STREET SPDR PORTFOLIO EM</t>
-  </si>
-  <si>
-    <t>SPEM</t>
-  </si>
-  <si>
-    <t>78463X509</t>
+    <t>TSY INFL IX N/B 01/35 2.125</t>
+  </si>
+  <si>
+    <t>91282CML2</t>
   </si>
   <si>
     <t>US DOLLAR</t>
@@ -267,12 +273,6 @@
     <t>999USDZ92</t>
   </si>
   <si>
-    <t>TSY INFL IX N/B 01/35 2.125</t>
-  </si>
-  <si>
-    <t>91282CML2</t>
-  </si>
-  <si>
     <t>TSY INFL IX N/B 07/34 1.875</t>
   </si>
   <si>
@@ -423,6 +423,15 @@
     <t>ADI3917X6</t>
   </si>
   <si>
+    <t>SPI 200 FUTURES   DEC26</t>
+  </si>
+  <si>
+    <t>XPZ6</t>
+  </si>
+  <si>
+    <t>ADI391SG0</t>
+  </si>
+  <si>
     <t>FTSE 100 IDX FUT  DEC26</t>
   </si>
   <si>
@@ -432,15 +441,6 @@
     <t>ADI38QPG9</t>
   </si>
   <si>
-    <t>SPI 200 FUTURES   DEC26</t>
-  </si>
-  <si>
-    <t>XPZ6</t>
-  </si>
-  <si>
-    <t>ADI391SG0</t>
-  </si>
-  <si>
     <t>CANADIAN DOLLAR</t>
   </si>
   <si>
@@ -468,6 +468,15 @@
     <t>ADI39K4N9</t>
   </si>
   <si>
+    <t>LONG GILT FUTURE  DEC26</t>
+  </si>
+  <si>
+    <t>G Z6</t>
+  </si>
+  <si>
+    <t>ADI3BKVP1</t>
+  </si>
+  <si>
     <t>EURO STOXX 50     DEC26</t>
   </si>
   <si>
@@ -475,15 +484,6 @@
   </si>
   <si>
     <t>ADI2VHXS0</t>
-  </si>
-  <si>
-    <t>LONG GILT FUTURE  DEC26</t>
-  </si>
-  <si>
-    <t>G Z6</t>
-  </si>
-  <si>
-    <t>ADI3BKVP1</t>
   </si>
   <si>
     <t>US LONG BOND(CBT) DEC26</t>
@@ -1479,16 +1479,16 @@
         <v>22</v>
       </c>
       <c r="D6" t="n" s="19">
-        <v>34.231807</v>
+        <v>34.688478</v>
       </c>
       <c r="E6" t="n" s="20">
-        <v>6.2926325071E8</v>
+        <v>6.3360390101E8</v>
       </c>
       <c r="F6" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G6" t="n" s="21">
-        <v>6.2926325071E8</v>
+        <v>6.3360390101E8</v>
       </c>
     </row>
     <row r="7">
@@ -1502,10 +1502,10 @@
         <v>25</v>
       </c>
       <c r="D7" t="n" s="22">
-        <v>13.340095</v>
+        <v>13.485232</v>
       </c>
       <c r="E7" t="n" s="23">
-        <v>2.4522314414E8</v>
+        <v>2.4631508734E8</v>
       </c>
       <c r="F7" t="s" s="18">
         <v>21</v>
@@ -1525,10 +1525,10 @@
         <v>27</v>
       </c>
       <c r="D8" t="n" s="25">
-        <v>4.91919</v>
+        <v>4.951055</v>
       </c>
       <c r="E8" t="n" s="26">
-        <v>9.042658961E7</v>
+        <v>9.043371562E7</v>
       </c>
       <c r="F8" t="s" s="18">
         <v>21</v>
@@ -1548,16 +1548,16 @@
         <v>29</v>
       </c>
       <c r="D9" t="n" s="28">
-        <v>4.270141</v>
+        <v>4.277567</v>
       </c>
       <c r="E9" t="n" s="29">
-        <v>7.849549623E7</v>
+        <v>7.813207827E7</v>
       </c>
       <c r="F9" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G9" t="n" s="30">
-        <v>8.3660555E7</v>
+        <v>8.3668585E7</v>
       </c>
     </row>
     <row r="10">
@@ -1565,45 +1565,45 @@
         <v>30</v>
       </c>
       <c r="B10" t="s" s="18">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="C10" t="s" s="18">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D10" t="n" s="31">
-        <v>4.178287</v>
+        <v>4.196344</v>
       </c>
       <c r="E10" t="n" s="32">
-        <v>7.680700959E7</v>
+        <v>7.6648509E7</v>
       </c>
       <c r="F10" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G10" t="n" s="33">
-        <v>8.2569108E7</v>
+        <v>1512700.0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="18">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B11" t="s" s="18">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="C11" t="s" s="18">
         <v>34</v>
       </c>
       <c r="D11" t="n" s="34">
-        <v>4.171311</v>
+        <v>4.185339</v>
       </c>
       <c r="E11" t="n" s="35">
-        <v>7.6678763E7</v>
+        <v>7.644748651E7</v>
       </c>
       <c r="F11" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G11" t="n" s="36">
-        <v>1512700.0</v>
+        <v>8.257793E7</v>
       </c>
     </row>
     <row r="12">
@@ -1617,16 +1617,16 @@
         <v>36</v>
       </c>
       <c r="D12" t="n" s="37">
-        <v>4.102548</v>
+        <v>4.000119</v>
       </c>
       <c r="E12" t="n" s="38">
-        <v>7.541473772E7</v>
+        <v>7.306433941E7</v>
       </c>
       <c r="F12" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G12" t="n" s="39">
-        <v>7.541473772E7</v>
+        <v>7.6436815E7</v>
       </c>
     </row>
     <row r="13">
@@ -1640,16 +1640,16 @@
         <v>38</v>
       </c>
       <c r="D13" t="n" s="40">
-        <v>3.991246</v>
+        <v>3.891156</v>
       </c>
       <c r="E13" t="n" s="41">
-        <v>7.336874333E7</v>
+        <v>7.107408742E7</v>
       </c>
       <c r="F13" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G13" t="n" s="42">
-        <v>7.6428884E7</v>
+        <v>7.107408742E7</v>
       </c>
     </row>
     <row r="14">
@@ -1663,16 +1663,16 @@
         <v>40</v>
       </c>
       <c r="D14" t="n" s="43">
-        <v>3.681658</v>
+        <v>3.690283</v>
       </c>
       <c r="E14" t="n" s="44">
-        <v>6.767775619E7</v>
+        <v>6.740502131E7</v>
       </c>
       <c r="F14" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G14" t="n" s="45">
-        <v>7.124413725E7</v>
+        <v>7.1251488E7</v>
       </c>
     </row>
     <row r="15">
@@ -1686,16 +1686,16 @@
         <v>42</v>
       </c>
       <c r="D15" t="n" s="46">
-        <v>3.506464</v>
+        <v>3.515306</v>
       </c>
       <c r="E15" t="n" s="47">
-        <v>6.445726916E7</v>
+        <v>6.420898126E7</v>
       </c>
       <c r="F15" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G15" t="n" s="48">
-        <v>6.82962665E7</v>
+        <v>6.830316955E7</v>
       </c>
     </row>
     <row r="16">
@@ -1709,10 +1709,10 @@
         <v>45</v>
       </c>
       <c r="D16" t="n" s="49">
-        <v>3.209737</v>
+        <v>3.221565</v>
       </c>
       <c r="E16" t="n" s="50">
-        <v>5.900271916E7</v>
+        <v>5.884362806E7</v>
       </c>
       <c r="F16" t="s" s="18">
         <v>21</v>
@@ -1732,16 +1732,16 @@
         <v>47</v>
       </c>
       <c r="D17" t="n" s="52">
-        <v>2.526514</v>
+        <v>2.530388</v>
       </c>
       <c r="E17" t="n" s="53">
-        <v>4.644342343E7</v>
+        <v>4.621891986E7</v>
       </c>
       <c r="F17" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G17" t="n" s="54">
-        <v>4.7880782E7</v>
+        <v>4.7885562E7</v>
       </c>
     </row>
     <row r="18">
@@ -1755,16 +1755,16 @@
         <v>49</v>
       </c>
       <c r="D18" t="n" s="55">
-        <v>1.48583</v>
+        <v>1.484438</v>
       </c>
       <c r="E18" t="n" s="56">
-        <v>2.731313529E7</v>
+        <v>2.711406774E7</v>
       </c>
       <c r="F18" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G18" t="n" s="57">
-        <v>3.56125221E7</v>
+        <v>3.56159955E7</v>
       </c>
     </row>
     <row r="19">
@@ -1778,16 +1778,16 @@
         <v>51</v>
       </c>
       <c r="D19" t="n" s="58">
-        <v>1.316249</v>
+        <v>1.313561</v>
       </c>
       <c r="E19" t="n" s="59">
-        <v>2.419583696E7</v>
+        <v>2.399290034E7</v>
       </c>
       <c r="F19" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G19" t="n" s="60">
-        <v>3.62760424E7</v>
+        <v>3.627987265E7</v>
       </c>
     </row>
     <row r="20">
@@ -1801,16 +1801,16 @@
         <v>53</v>
       </c>
       <c r="D20" t="n" s="61">
-        <v>1.239504</v>
+        <v>1.235388</v>
       </c>
       <c r="E20" t="n" s="62">
-        <v>2.278507957E7</v>
+        <v>2.256503504E7</v>
       </c>
       <c r="F20" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G20" t="n" s="63">
-        <v>2.68541061E7</v>
+        <v>2.68568924E7</v>
       </c>
     </row>
     <row r="21">
@@ -1824,16 +1824,16 @@
         <v>55</v>
       </c>
       <c r="D21" t="n" s="64">
-        <v>1.16614</v>
+        <v>1.162445</v>
       </c>
       <c r="E21" t="n" s="65">
-        <v>2.143646611E7</v>
+        <v>2.123268885E7</v>
       </c>
       <c r="F21" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G21" t="n" s="66">
-        <v>2.662398275E7</v>
+        <v>2.66266695E7</v>
       </c>
     </row>
     <row r="22">
@@ -1847,16 +1847,16 @@
         <v>57</v>
       </c>
       <c r="D22" t="n" s="67">
-        <v>1.143102</v>
+        <v>1.139067</v>
       </c>
       <c r="E22" t="n" s="68">
-        <v>2.101297721E7</v>
+        <v>2.080568349E7</v>
       </c>
       <c r="F22" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G22" t="n" s="69">
-        <v>2.477352E7</v>
+        <v>2.477616E7</v>
       </c>
     </row>
     <row r="23">
@@ -1870,16 +1870,16 @@
         <v>59</v>
       </c>
       <c r="D23" t="n" s="70">
-        <v>1.10335</v>
+        <v>1.10297</v>
       </c>
       <c r="E23" t="n" s="71">
-        <v>2.028224154E7</v>
+        <v>2.014635318E7</v>
       </c>
       <c r="F23" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G23" t="n" s="72">
-        <v>2.824794E7</v>
+        <v>2.8250802E7</v>
       </c>
     </row>
     <row r="24">
@@ -1893,16 +1893,16 @@
         <v>61</v>
       </c>
       <c r="D24" t="n" s="73">
-        <v>0.955659</v>
+        <v>0.952232</v>
       </c>
       <c r="E24" t="n" s="74">
-        <v>1.756731606E7</v>
+        <v>1.739304371E7</v>
       </c>
       <c r="F24" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G24" t="n" s="75">
-        <v>2.5096866E7</v>
+        <v>2.5099319E7</v>
       </c>
     </row>
     <row r="25">
@@ -1916,16 +1916,16 @@
         <v>63</v>
       </c>
       <c r="D25" t="n" s="76">
-        <v>0.932062</v>
+        <v>0.931355</v>
       </c>
       <c r="E25" t="n" s="77">
-        <v>1.713354976E7</v>
+        <v>1.701170636E7</v>
       </c>
       <c r="F25" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G25" t="n" s="78">
-        <v>2.50124814E7</v>
+        <v>2.50150599E7</v>
       </c>
     </row>
     <row r="26">
@@ -1939,16 +1939,16 @@
         <v>65</v>
       </c>
       <c r="D26" t="n" s="79">
-        <v>0.889022</v>
+        <v>0.886693</v>
       </c>
       <c r="E26" t="n" s="80">
-        <v>1.634237099E7</v>
+        <v>1.619593642E7</v>
       </c>
       <c r="F26" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G26" t="n" s="81">
-        <v>2.48760075E7</v>
+        <v>2.48787E7</v>
       </c>
     </row>
     <row r="27">
@@ -1962,16 +1962,16 @@
         <v>67</v>
       </c>
       <c r="D27" t="n" s="82">
-        <v>0.733978</v>
+        <v>0.732712</v>
       </c>
       <c r="E27" t="n" s="83">
-        <v>1.349228961E7</v>
+        <v>1.338338481E7</v>
       </c>
       <c r="F27" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G27" t="n" s="84">
-        <v>1.95967556E7</v>
+        <v>1.95986988E7</v>
       </c>
     </row>
     <row r="28">
@@ -1985,16 +1985,16 @@
         <v>69</v>
       </c>
       <c r="D28" t="n" s="85">
-        <v>0.729356</v>
+        <v>0.72505</v>
       </c>
       <c r="E28" t="n" s="86">
-        <v>1.340732035E7</v>
+        <v>1.324342925E7</v>
       </c>
       <c r="F28" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G28" t="n" s="87">
-        <v>2.8481238E7</v>
+        <v>2.8484082E7</v>
       </c>
     </row>
     <row r="29">
@@ -2008,16 +2008,16 @@
         <v>71</v>
       </c>
       <c r="D29" t="n" s="88">
-        <v>0.719884</v>
+        <v>0.716647</v>
       </c>
       <c r="E29" t="n" s="89">
-        <v>1.323319864E7</v>
+        <v>1.308994116E7</v>
       </c>
       <c r="F29" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G29" t="n" s="90">
-        <v>2.552323415E7</v>
+        <v>2.55257841E7</v>
       </c>
     </row>
     <row r="30">
@@ -2031,16 +2031,16 @@
         <v>73</v>
       </c>
       <c r="D30" t="n" s="91">
-        <v>0.608621</v>
+        <v>0.605692</v>
       </c>
       <c r="E30" t="n" s="92">
-        <v>1.118791964E7</v>
+        <v>1.106330138E7</v>
       </c>
       <c r="F30" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G30" t="n" s="93">
-        <v>2.30901921E7</v>
+        <v>2.30927079E7</v>
       </c>
     </row>
     <row r="31">
@@ -2054,16 +2054,16 @@
         <v>75</v>
       </c>
       <c r="D31" t="n" s="94">
-        <v>0.572678</v>
+        <v>0.57114</v>
       </c>
       <c r="E31" t="n" s="95">
-        <v>1.052720355E7</v>
+        <v>1.043217795E7</v>
       </c>
       <c r="F31" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G31" t="n" s="96">
-        <v>1.5872337E7</v>
+        <v>1.5873975E7</v>
       </c>
     </row>
     <row r="32">
@@ -2077,16 +2077,16 @@
         <v>77</v>
       </c>
       <c r="D32" t="n" s="97">
-        <v>0.560562</v>
+        <v>0.558957</v>
       </c>
       <c r="E32" t="n" s="98">
-        <v>1.030447445E7</v>
+        <v>1.020965533E7</v>
       </c>
       <c r="F32" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G32" t="n" s="99">
-        <v>1.57871E7</v>
+        <v>1.57887625E7</v>
       </c>
     </row>
     <row r="33">
@@ -2100,10 +2100,10 @@
         <v>21</v>
       </c>
       <c r="D33" t="n" s="100">
-        <v>0.459146</v>
+        <v>0.406948</v>
       </c>
       <c r="E33" t="n" s="101">
-        <v>8440220.12</v>
+        <v>7433131.73</v>
       </c>
       <c r="F33" t="n" s="102">
         <v>4.1426456199E8</v>
@@ -2123,10 +2123,10 @@
         <v>80</v>
       </c>
       <c r="D34" t="n" s="104">
-        <v>0.26612</v>
+        <v>0.266965</v>
       </c>
       <c r="E34" t="n" s="105">
-        <v>4891919.6</v>
+        <v>4876269.92</v>
       </c>
       <c r="F34" t="s" s="18">
         <v>21</v>
@@ -2146,10 +2146,10 @@
         <v>82</v>
       </c>
       <c r="D35" t="n" s="107">
-        <v>0.147702</v>
+        <v>0.148252</v>
       </c>
       <c r="E35" t="n" s="108">
-        <v>2715127.96</v>
+        <v>2707907.06</v>
       </c>
       <c r="F35" t="s" s="18">
         <v>21</v>
@@ -2169,13 +2169,13 @@
         <v>85</v>
       </c>
       <c r="D36" t="n" s="110">
-        <v>0.107328</v>
+        <v>0.111856</v>
       </c>
       <c r="E36" t="n" s="111">
-        <v>1.7175882627E8</v>
+        <v>1.7227986102E8</v>
       </c>
       <c r="F36" t="n" s="112">
-        <v>1.7175882627E8</v>
+        <v>1.7227986102E8</v>
       </c>
       <c r="G36" t="n" s="113">
         <v>2.331E8</v>
@@ -2192,13 +2192,13 @@
         <v>88</v>
       </c>
       <c r="D37" t="n" s="114">
-        <v>0.064143</v>
+        <v>0.05792</v>
       </c>
       <c r="E37" t="n" s="115">
-        <v>8.735180143E7</v>
+        <v>8.695055066E7</v>
       </c>
       <c r="F37" t="n" s="116">
-        <v>8.735180143E7</v>
+        <v>8.695055066E7</v>
       </c>
       <c r="G37" t="n" s="117">
         <v>3380000.0</v>
@@ -2215,16 +2215,16 @@
         <v>91</v>
       </c>
       <c r="D38" t="n" s="118">
-        <v>0.052626</v>
+        <v>0.049403</v>
       </c>
       <c r="E38" t="n" s="119">
-        <v>7.378906255E7</v>
+        <v>6.822563004E7</v>
       </c>
       <c r="F38" t="n" s="120">
-        <v>7.378906255E7</v>
+        <v>6.822563004E7</v>
       </c>
       <c r="G38" t="n" s="121">
-        <v>5060.0</v>
+        <v>11025.0</v>
       </c>
     </row>
     <row r="39">
@@ -2238,16 +2238,16 @@
         <v>94</v>
       </c>
       <c r="D39" t="n" s="122">
-        <v>0.03935</v>
+        <v>0.008735</v>
       </c>
       <c r="E39" t="n" s="123">
-        <v>6.786829592E7</v>
+        <v>7.278755134E7</v>
       </c>
       <c r="F39" t="n" s="124">
-        <v>6.786829592E7</v>
+        <v>7.278755134E7</v>
       </c>
       <c r="G39" t="n" s="125">
-        <v>11025.0</v>
+        <v>5060.0</v>
       </c>
     </row>
     <row r="40">
@@ -2264,7 +2264,7 @@
         <v>0.0</v>
       </c>
       <c r="E40" t="n" s="127">
-        <v>7.48</v>
+        <v>7.51</v>
       </c>
       <c r="F40" t="s" s="18">
         <v>21</v>
@@ -2284,10 +2284,10 @@
         <v>98</v>
       </c>
       <c r="D41" t="n" s="129">
-        <v>-0.006744</v>
+        <v>-0.006806</v>
       </c>
       <c r="E41" t="n" s="130">
-        <v>-123978.24</v>
+        <v>-124307.47</v>
       </c>
       <c r="F41" t="s" s="18">
         <v>21</v>
@@ -2307,10 +2307,10 @@
         <v>100</v>
       </c>
       <c r="D42" t="n" s="132">
-        <v>-0.007722</v>
+        <v>-0.007746</v>
       </c>
       <c r="E42" t="n" s="133">
-        <v>-141950.9</v>
+        <v>-141489.51</v>
       </c>
       <c r="F42" t="s" s="18">
         <v>21</v>
@@ -2330,13 +2330,13 @@
         <v>103</v>
       </c>
       <c r="D43" t="n" s="135">
-        <v>-0.011082</v>
+        <v>-0.084044</v>
       </c>
       <c r="E43" t="n" s="136">
-        <v>3.3858909899E8</v>
+        <v>3.3617388144E8</v>
       </c>
       <c r="F43" t="n" s="137">
-        <v>3.3858909899E8</v>
+        <v>3.3617388144E8</v>
       </c>
       <c r="G43" t="n" s="138">
         <v>2.474E8</v>
@@ -2353,16 +2353,16 @@
         <v>106</v>
       </c>
       <c r="D44" t="n" s="139">
-        <v>-0.066771</v>
+        <v>-0.157031</v>
       </c>
       <c r="E44" t="n" s="140">
-        <v>1.7417220689E8</v>
+        <v>1.1818775536E8</v>
       </c>
       <c r="F44" t="n" s="141">
-        <v>1.7417220689E8</v>
+        <v>1.1818775536E8</v>
       </c>
       <c r="G44" t="n" s="142">
-        <v>24880.0</v>
+        <v>1.056E8</v>
       </c>
     </row>
     <row r="45">
@@ -2376,16 +2376,16 @@
         <v>109</v>
       </c>
       <c r="D45" t="n" s="143">
-        <v>-0.101986</v>
+        <v>-0.164769</v>
       </c>
       <c r="E45" t="n" s="144">
-        <v>1.1950406933E8</v>
+        <v>1.7182890935E8</v>
       </c>
       <c r="F45" t="n" s="145">
-        <v>1.1950406933E8</v>
+        <v>1.7182890935E8</v>
       </c>
       <c r="G45" t="n" s="146">
-        <v>1.056E8</v>
+        <v>24880.0</v>
       </c>
     </row>
     <row r="46">
@@ -2399,13 +2399,13 @@
         <v>112</v>
       </c>
       <c r="D46" t="n" s="147">
-        <v>-0.37218</v>
+        <v>-0.423501</v>
       </c>
       <c r="E46" t="n" s="148">
-        <v>2.0100971875E8</v>
+        <v>2.001158125E8</v>
       </c>
       <c r="F46" t="n" s="149">
-        <v>2.0100971875E8</v>
+        <v>2.001158125E8</v>
       </c>
       <c r="G46" t="n" s="150">
         <v>1.907E8</v>
@@ -2422,13 +2422,13 @@
         <v>115</v>
       </c>
       <c r="D47" t="n" s="151">
-        <v>-0.404827</v>
+        <v>-0.456279</v>
       </c>
       <c r="E47" t="n" s="152">
-        <v>1.7769675E8</v>
+        <v>1.7680425E8</v>
       </c>
       <c r="F47" t="n" s="153">
-        <v>1.7769675E8</v>
+        <v>1.7680425E8</v>
       </c>
       <c r="G47" t="n" s="154">
         <v>42500.0</v>
@@ -2445,13 +2445,13 @@
         <v>118</v>
       </c>
       <c r="D48" t="n" s="155">
-        <v>-0.58518</v>
+        <v>-0.635709</v>
       </c>
       <c r="E48" t="n" s="156">
-        <v>4.4364129685E8</v>
+        <v>4.4278675E8</v>
       </c>
       <c r="F48" t="n" s="157">
-        <v>4.4364129685E8</v>
+        <v>4.4278675E8</v>
       </c>
       <c r="G48" t="n" s="158">
         <v>4.207E8</v>

</xml_diff>

<commit_message>
Update ALLW XLSX 2026-10-21
</commit_message>
<xml_diff>
--- a/latest/allw-latest.xlsx
+++ b/latest/allw-latest.xlsx
@@ -192,7 +192,7 @@
     <t>ALLW</t>
   </si>
   <si>
-    <t>As of 19-Oct-2026</t>
+    <t>As of 20-Oct-2026</t>
   </si>
   <si>
     <t>Name</t>
@@ -240,6 +240,12 @@
     <t>912797TV9</t>
   </si>
   <si>
+    <t>US DOLLAR</t>
+  </si>
+  <si>
+    <t>999USDZ92</t>
+  </si>
+  <si>
     <t>TSY INFL IX N/B 07/35 1.875</t>
   </si>
   <si>
@@ -267,12 +273,6 @@
     <t>91282CML2</t>
   </si>
   <si>
-    <t>US DOLLAR</t>
-  </si>
-  <si>
-    <t>999USDZ92</t>
-  </si>
-  <si>
     <t>TSY INFL IX N/B 07/34 1.875</t>
   </si>
   <si>
@@ -414,6 +414,30 @@
     <t>ADI3BDHZ1</t>
   </si>
   <si>
+    <t>SPI 200 FUTURES   DEC26</t>
+  </si>
+  <si>
+    <t>XPZ6</t>
+  </si>
+  <si>
+    <t>ADI391SG0</t>
+  </si>
+  <si>
+    <t>EURO-BUND FUTURE  DEC26</t>
+  </si>
+  <si>
+    <t>RXZ6</t>
+  </si>
+  <si>
+    <t>ADI39K4N9</t>
+  </si>
+  <si>
+    <t>CANADIAN DOLLAR</t>
+  </si>
+  <si>
+    <t>999CADZ91</t>
+  </si>
+  <si>
     <t>TOPIX INDX FUTR   DEC26</t>
   </si>
   <si>
@@ -423,15 +447,6 @@
     <t>ADI3917X6</t>
   </si>
   <si>
-    <t>SPI 200 FUTURES   DEC26</t>
-  </si>
-  <si>
-    <t>XPZ6</t>
-  </si>
-  <si>
-    <t>ADI391SG0</t>
-  </si>
-  <si>
     <t>FTSE 100 IDX FUT  DEC26</t>
   </si>
   <si>
@@ -441,12 +456,6 @@
     <t>ADI38QPG9</t>
   </si>
   <si>
-    <t>CANADIAN DOLLAR</t>
-  </si>
-  <si>
-    <t>999CADZ91</t>
-  </si>
-  <si>
     <t>AUSTRALIAN DOLLAR</t>
   </si>
   <si>
@@ -457,15 +466,6 @@
   </si>
   <si>
     <t>999JPYZ94</t>
-  </si>
-  <si>
-    <t>EURO-BUND FUTURE  DEC26</t>
-  </si>
-  <si>
-    <t>RXZ6</t>
-  </si>
-  <si>
-    <t>ADI39K4N9</t>
   </si>
   <si>
     <t>LONG GILT FUTURE  DEC26</t>
@@ -984,43 +984,43 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
@@ -1479,16 +1479,16 @@
         <v>22</v>
       </c>
       <c r="D6" t="n" s="19">
-        <v>34.688478</v>
+        <v>34.228802</v>
       </c>
       <c r="E6" t="n" s="20">
-        <v>6.3360390101E8</v>
+        <v>6.2635107145E8</v>
       </c>
       <c r="F6" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G6" t="n" s="21">
-        <v>6.3360390101E8</v>
+        <v>6.2635107145E8</v>
       </c>
     </row>
     <row r="7">
@@ -1502,10 +1502,10 @@
         <v>25</v>
       </c>
       <c r="D7" t="n" s="22">
-        <v>13.485232</v>
+        <v>13.505369</v>
       </c>
       <c r="E7" t="n" s="23">
-        <v>2.4631508734E8</v>
+        <v>2.4713404474E8</v>
       </c>
       <c r="F7" t="s" s="18">
         <v>21</v>
@@ -1525,10 +1525,10 @@
         <v>27</v>
       </c>
       <c r="D8" t="n" s="25">
-        <v>4.951055</v>
+        <v>4.942543</v>
       </c>
       <c r="E8" t="n" s="26">
-        <v>9.043371562E7</v>
+        <v>9.044333495E7</v>
       </c>
       <c r="F8" t="s" s="18">
         <v>21</v>
@@ -1548,16 +1548,16 @@
         <v>29</v>
       </c>
       <c r="D9" t="n" s="28">
-        <v>4.277567</v>
+        <v>4.280399</v>
       </c>
       <c r="E9" t="n" s="29">
-        <v>7.813207827E7</v>
+        <v>7.83268028E7</v>
       </c>
       <c r="F9" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G9" t="n" s="30">
-        <v>8.3668585E7</v>
+        <v>7.83268028E7</v>
       </c>
     </row>
     <row r="10">
@@ -1565,45 +1565,45 @@
         <v>30</v>
       </c>
       <c r="B10" t="s" s="18">
+        <v>21</v>
+      </c>
+      <c r="C10" t="s" s="18">
         <v>31</v>
       </c>
-      <c r="C10" t="s" s="18">
-        <v>32</v>
-      </c>
       <c r="D10" t="n" s="31">
-        <v>4.196344</v>
+        <v>4.279586</v>
       </c>
       <c r="E10" t="n" s="32">
-        <v>7.6648509E7</v>
+        <v>7.831193075E7</v>
       </c>
       <c r="F10" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G10" t="n" s="33">
-        <v>1512700.0</v>
+        <v>8.3677418E7</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="18">
+        <v>32</v>
+      </c>
+      <c r="B11" t="s" s="18">
         <v>33</v>
-      </c>
-      <c r="B11" t="s" s="18">
-        <v>21</v>
       </c>
       <c r="C11" t="s" s="18">
         <v>34</v>
       </c>
       <c r="D11" t="n" s="34">
-        <v>4.185339</v>
+        <v>4.208524</v>
       </c>
       <c r="E11" t="n" s="35">
-        <v>7.644748651E7</v>
+        <v>7.7011557E7</v>
       </c>
       <c r="F11" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G11" t="n" s="36">
-        <v>8.257793E7</v>
+        <v>1512700.0</v>
       </c>
     </row>
     <row r="12">
@@ -1617,16 +1617,16 @@
         <v>36</v>
       </c>
       <c r="D12" t="n" s="37">
-        <v>4.000119</v>
+        <v>4.188017</v>
       </c>
       <c r="E12" t="n" s="38">
-        <v>7.306433941E7</v>
+        <v>7.66363121E7</v>
       </c>
       <c r="F12" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G12" t="n" s="39">
-        <v>7.6436815E7</v>
+        <v>8.2586752E7</v>
       </c>
     </row>
     <row r="13">
@@ -1640,16 +1640,16 @@
         <v>38</v>
       </c>
       <c r="D13" t="n" s="40">
-        <v>3.891156</v>
+        <v>4.000574</v>
       </c>
       <c r="E13" t="n" s="41">
-        <v>7.107408742E7</v>
+        <v>7.320629582E7</v>
       </c>
       <c r="F13" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G13" t="n" s="42">
-        <v>7.107408742E7</v>
+        <v>7.6444746E7</v>
       </c>
     </row>
     <row r="14">
@@ -1663,16 +1663,16 @@
         <v>40</v>
       </c>
       <c r="D14" t="n" s="43">
-        <v>3.690283</v>
+        <v>3.690391</v>
       </c>
       <c r="E14" t="n" s="44">
-        <v>6.740502131E7</v>
+        <v>6.753027559E7</v>
       </c>
       <c r="F14" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G14" t="n" s="45">
-        <v>7.1251488E7</v>
+        <v>7.125883875E7</v>
       </c>
     </row>
     <row r="15">
@@ -1686,16 +1686,16 @@
         <v>42</v>
       </c>
       <c r="D15" t="n" s="46">
-        <v>3.515306</v>
+        <v>3.515182</v>
       </c>
       <c r="E15" t="n" s="47">
-        <v>6.420898126E7</v>
+        <v>6.432413072E7</v>
       </c>
       <c r="F15" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G15" t="n" s="48">
-        <v>6.830316955E7</v>
+        <v>6.831070015E7</v>
       </c>
     </row>
     <row r="16">
@@ -1709,10 +1709,10 @@
         <v>45</v>
       </c>
       <c r="D16" t="n" s="49">
-        <v>3.221565</v>
+        <v>3.227627</v>
       </c>
       <c r="E16" t="n" s="50">
-        <v>5.884362806E7</v>
+        <v>5.906218525E7</v>
       </c>
       <c r="F16" t="s" s="18">
         <v>21</v>
@@ -1732,16 +1732,16 @@
         <v>47</v>
       </c>
       <c r="D17" t="n" s="52">
-        <v>2.530388</v>
+        <v>2.532283</v>
       </c>
       <c r="E17" t="n" s="53">
-        <v>4.621891986E7</v>
+        <v>4.633811006E7</v>
       </c>
       <c r="F17" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G17" t="n" s="54">
-        <v>4.7885562E7</v>
+        <v>4.789082E7</v>
       </c>
     </row>
     <row r="18">
@@ -1755,16 +1755,16 @@
         <v>49</v>
       </c>
       <c r="D18" t="n" s="55">
-        <v>1.484438</v>
+        <v>1.492908</v>
       </c>
       <c r="E18" t="n" s="56">
-        <v>2.711406774E7</v>
+        <v>2.731865344E7</v>
       </c>
       <c r="F18" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G18" t="n" s="57">
-        <v>3.56159955E7</v>
+        <v>3.5619717E7</v>
       </c>
     </row>
     <row r="19">
@@ -1778,16 +1778,16 @@
         <v>51</v>
       </c>
       <c r="D19" t="n" s="58">
-        <v>1.313561</v>
+        <v>1.322755</v>
       </c>
       <c r="E19" t="n" s="59">
-        <v>2.399290034E7</v>
+        <v>2.42050282E7</v>
       </c>
       <c r="F19" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G19" t="n" s="60">
-        <v>3.627987265E7</v>
+        <v>3.628344755E7</v>
       </c>
     </row>
     <row r="20">
@@ -1801,16 +1801,16 @@
         <v>53</v>
       </c>
       <c r="D20" t="n" s="61">
-        <v>1.235388</v>
+        <v>1.246093</v>
       </c>
       <c r="E20" t="n" s="62">
-        <v>2.256503504E7</v>
+        <v>2.280218322E7</v>
       </c>
       <c r="F20" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G20" t="n" s="63">
-        <v>2.68568924E7</v>
+        <v>2.68594254E7</v>
       </c>
     </row>
     <row r="21">
@@ -1824,16 +1824,16 @@
         <v>55</v>
       </c>
       <c r="D21" t="n" s="64">
-        <v>1.162445</v>
+        <v>1.172605</v>
       </c>
       <c r="E21" t="n" s="65">
-        <v>2.123268885E7</v>
+        <v>2.145743597E7</v>
       </c>
       <c r="F21" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G21" t="n" s="66">
-        <v>2.66266695E7</v>
+        <v>2.662935625E7</v>
       </c>
     </row>
     <row r="22">
@@ -1847,16 +1847,16 @@
         <v>57</v>
       </c>
       <c r="D22" t="n" s="67">
-        <v>1.139067</v>
+        <v>1.148905</v>
       </c>
       <c r="E22" t="n" s="68">
-        <v>2.080568349E7</v>
+        <v>2.102374705E7</v>
       </c>
       <c r="F22" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G22" t="n" s="69">
-        <v>2.477616E7</v>
+        <v>2.47788E7</v>
       </c>
     </row>
     <row r="23">
@@ -1870,16 +1870,16 @@
         <v>59</v>
       </c>
       <c r="D23" t="n" s="70">
-        <v>1.10297</v>
+        <v>1.10903</v>
       </c>
       <c r="E23" t="n" s="71">
-        <v>2.014635318E7</v>
+        <v>2.02940771E7</v>
       </c>
       <c r="F23" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G23" t="n" s="72">
-        <v>2.8250802E7</v>
+        <v>2.8253664E7</v>
       </c>
     </row>
     <row r="24">
@@ -1893,16 +1893,16 @@
         <v>61</v>
       </c>
       <c r="D24" t="n" s="73">
-        <v>0.952232</v>
+        <v>0.960937</v>
       </c>
       <c r="E24" t="n" s="74">
-        <v>1.739304371E7</v>
+        <v>1.758414354E7</v>
       </c>
       <c r="F24" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G24" t="n" s="75">
-        <v>2.5099319E7</v>
+        <v>2.5101995E7</v>
       </c>
     </row>
     <row r="25">
@@ -1916,16 +1916,16 @@
         <v>63</v>
       </c>
       <c r="D25" t="n" s="76">
-        <v>0.931355</v>
+        <v>0.936854</v>
       </c>
       <c r="E25" t="n" s="77">
-        <v>1.701170636E7</v>
+        <v>1.714343453E7</v>
       </c>
       <c r="F25" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G25" t="n" s="78">
-        <v>2.50150599E7</v>
+        <v>2.50176384E7</v>
       </c>
     </row>
     <row r="26">
@@ -1939,16 +1939,16 @@
         <v>65</v>
       </c>
       <c r="D26" t="n" s="79">
-        <v>0.886693</v>
+        <v>0.893769</v>
       </c>
       <c r="E26" t="n" s="80">
-        <v>1.619593642E7</v>
+        <v>1.635502393E7</v>
       </c>
       <c r="F26" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G26" t="n" s="81">
-        <v>2.48787E7</v>
+        <v>2.4881213E7</v>
       </c>
     </row>
     <row r="27">
@@ -1962,16 +1962,16 @@
         <v>67</v>
       </c>
       <c r="D27" t="n" s="82">
-        <v>0.732712</v>
+        <v>0.738021</v>
       </c>
       <c r="E27" t="n" s="83">
-        <v>1.338338481E7</v>
+        <v>1.350501461E7</v>
       </c>
       <c r="F27" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G27" t="n" s="84">
-        <v>1.95986988E7</v>
+        <v>1.96007808E7</v>
       </c>
     </row>
     <row r="28">
@@ -1985,16 +1985,16 @@
         <v>69</v>
       </c>
       <c r="D28" t="n" s="85">
-        <v>0.72505</v>
+        <v>0.733473</v>
       </c>
       <c r="E28" t="n" s="86">
-        <v>1.324342925E7</v>
+        <v>1.342179351E7</v>
       </c>
       <c r="F28" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G28" t="n" s="87">
-        <v>2.8484082E7</v>
+        <v>2.8487163E7</v>
       </c>
     </row>
     <row r="29">
@@ -2008,16 +2008,16 @@
         <v>71</v>
       </c>
       <c r="D29" t="n" s="88">
-        <v>0.716647</v>
+        <v>0.723808</v>
       </c>
       <c r="E29" t="n" s="89">
-        <v>1.308994116E7</v>
+        <v>1.324491959E7</v>
       </c>
       <c r="F29" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G29" t="n" s="90">
-        <v>2.55257841E7</v>
+        <v>2.55285302E7</v>
       </c>
     </row>
     <row r="30">
@@ -2031,16 +2031,16 @@
         <v>73</v>
       </c>
       <c r="D30" t="n" s="91">
-        <v>0.605692</v>
+        <v>0.612142</v>
       </c>
       <c r="E30" t="n" s="92">
-        <v>1.106330138E7</v>
+        <v>1.120154739E7</v>
       </c>
       <c r="F30" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G30" t="n" s="93">
-        <v>2.30927079E7</v>
+        <v>2.3095044E7</v>
       </c>
     </row>
     <row r="31">
@@ -2054,16 +2054,16 @@
         <v>75</v>
       </c>
       <c r="D31" t="n" s="94">
-        <v>0.57114</v>
+        <v>0.575697</v>
       </c>
       <c r="E31" t="n" s="95">
-        <v>1.043217795E7</v>
+        <v>1.053464751E7</v>
       </c>
       <c r="F31" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G31" t="n" s="96">
-        <v>1.5873975E7</v>
+        <v>1.5875613E7</v>
       </c>
     </row>
     <row r="32">
@@ -2077,16 +2077,16 @@
         <v>77</v>
       </c>
       <c r="D32" t="n" s="97">
-        <v>0.558957</v>
+        <v>0.563688</v>
       </c>
       <c r="E32" t="n" s="98">
-        <v>1.020965533E7</v>
+        <v>1.031489424E7</v>
       </c>
       <c r="F32" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G32" t="n" s="99">
-        <v>1.57887625E7</v>
+        <v>1.579030625E7</v>
       </c>
     </row>
     <row r="33">
@@ -2100,10 +2100,10 @@
         <v>21</v>
       </c>
       <c r="D33" t="n" s="100">
-        <v>0.406948</v>
+        <v>0.296468</v>
       </c>
       <c r="E33" t="n" s="101">
-        <v>7433131.73</v>
+        <v>5425049.61</v>
       </c>
       <c r="F33" t="n" s="102">
         <v>4.1426456199E8</v>
@@ -2123,10 +2123,10 @@
         <v>80</v>
       </c>
       <c r="D34" t="n" s="104">
-        <v>0.266965</v>
+        <v>0.267155</v>
       </c>
       <c r="E34" t="n" s="105">
-        <v>4876269.92</v>
+        <v>4888657.39</v>
       </c>
       <c r="F34" t="s" s="18">
         <v>21</v>
@@ -2146,10 +2146,10 @@
         <v>82</v>
       </c>
       <c r="D35" t="n" s="107">
-        <v>0.148252</v>
+        <v>0.14876</v>
       </c>
       <c r="E35" t="n" s="108">
-        <v>2707907.06</v>
+        <v>2722143.27</v>
       </c>
       <c r="F35" t="s" s="18">
         <v>21</v>
@@ -2169,13 +2169,13 @@
         <v>85</v>
       </c>
       <c r="D36" t="n" s="110">
-        <v>0.111856</v>
+        <v>0.094276</v>
       </c>
       <c r="E36" t="n" s="111">
-        <v>1.7227986102E8</v>
+        <v>1.7259561455E8</v>
       </c>
       <c r="F36" t="n" s="112">
-        <v>1.7227986102E8</v>
+        <v>1.7259561455E8</v>
       </c>
       <c r="G36" t="n" s="113">
         <v>2.331E8</v>
@@ -2192,16 +2192,16 @@
         <v>88</v>
       </c>
       <c r="D37" t="n" s="114">
-        <v>0.05792</v>
+        <v>0.038515</v>
       </c>
       <c r="E37" t="n" s="115">
-        <v>8.695055066E7</v>
+        <v>6.82786491E7</v>
       </c>
       <c r="F37" t="n" s="116">
-        <v>8.695055066E7</v>
+        <v>6.82786491E7</v>
       </c>
       <c r="G37" t="n" s="117">
-        <v>3380000.0</v>
+        <v>11025.0</v>
       </c>
     </row>
     <row r="38">
@@ -2215,16 +2215,16 @@
         <v>91</v>
       </c>
       <c r="D38" t="n" s="118">
-        <v>0.049403</v>
+        <v>0.002558</v>
       </c>
       <c r="E38" t="n" s="119">
-        <v>6.822563004E7</v>
+        <v>3.3861370039E8</v>
       </c>
       <c r="F38" t="n" s="120">
-        <v>6.822563004E7</v>
+        <v>3.3861370039E8</v>
       </c>
       <c r="G38" t="n" s="121">
-        <v>11025.0</v>
+        <v>2.474E8</v>
       </c>
     </row>
     <row r="39">
@@ -2232,45 +2232,45 @@
         <v>92</v>
       </c>
       <c r="B39" t="s" s="18">
+        <v>21</v>
+      </c>
+      <c r="C39" t="s" s="18">
         <v>93</v>
       </c>
-      <c r="C39" t="s" s="18">
-        <v>94</v>
-      </c>
       <c r="D39" t="n" s="122">
-        <v>0.008735</v>
+        <v>0.0</v>
       </c>
       <c r="E39" t="n" s="123">
-        <v>7.278755134E7</v>
-      </c>
-      <c r="F39" t="n" s="124">
-        <v>7.278755134E7</v>
-      </c>
-      <c r="G39" t="n" s="125">
-        <v>5060.0</v>
+        <v>7.53</v>
+      </c>
+      <c r="F39" t="s" s="18">
+        <v>21</v>
+      </c>
+      <c r="G39" t="n" s="124">
+        <v>10.58</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s" s="18">
+        <v>94</v>
+      </c>
+      <c r="B40" t="s" s="18">
         <v>95</v>
-      </c>
-      <c r="B40" t="s" s="18">
-        <v>21</v>
       </c>
       <c r="C40" t="s" s="18">
         <v>96</v>
       </c>
-      <c r="D40" t="n" s="126">
-        <v>0.0</v>
-      </c>
-      <c r="E40" t="n" s="127">
-        <v>7.51</v>
-      </c>
-      <c r="F40" t="s" s="18">
-        <v>21</v>
+      <c r="D40" t="n" s="125">
+        <v>-0.001645</v>
+      </c>
+      <c r="E40" t="n" s="126">
+        <v>8.612350837E7</v>
+      </c>
+      <c r="F40" t="n" s="127">
+        <v>8.612350837E7</v>
       </c>
       <c r="G40" t="n" s="128">
-        <v>10.58</v>
+        <v>3380000.0</v>
       </c>
     </row>
     <row r="41">
@@ -2278,68 +2278,68 @@
         <v>97</v>
       </c>
       <c r="B41" t="s" s="18">
-        <v>21</v>
+        <v>98</v>
       </c>
       <c r="C41" t="s" s="18">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D41" t="n" s="129">
-        <v>-0.006806</v>
+        <v>-0.004006</v>
       </c>
       <c r="E41" t="n" s="130">
-        <v>-124307.47</v>
-      </c>
-      <c r="F41" t="s" s="18">
-        <v>21</v>
-      </c>
-      <c r="G41" t="n" s="131">
-        <v>-177976.22</v>
+        <v>7.293650974E7</v>
+      </c>
+      <c r="F41" t="n" s="131">
+        <v>7.293650974E7</v>
+      </c>
+      <c r="G41" t="n" s="132">
+        <v>5060.0</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s" s="18">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B42" t="s" s="18">
         <v>21</v>
       </c>
       <c r="C42" t="s" s="18">
-        <v>100</v>
-      </c>
-      <c r="D42" t="n" s="132">
-        <v>-0.007746</v>
-      </c>
-      <c r="E42" t="n" s="133">
-        <v>-141489.51</v>
+        <v>101</v>
+      </c>
+      <c r="D42" t="n" s="133">
+        <v>-0.006818</v>
+      </c>
+      <c r="E42" t="n" s="134">
+        <v>-124770.21</v>
       </c>
       <c r="F42" t="s" s="18">
         <v>21</v>
       </c>
-      <c r="G42" t="n" s="134">
-        <v>-2.2418306E7</v>
+      <c r="G42" t="n" s="135">
+        <v>-177976.22</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="s" s="18">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B43" t="s" s="18">
-        <v>102</v>
+        <v>21</v>
       </c>
       <c r="C43" t="s" s="18">
         <v>103</v>
       </c>
-      <c r="D43" t="n" s="135">
-        <v>-0.084044</v>
-      </c>
-      <c r="E43" t="n" s="136">
-        <v>3.3617388144E8</v>
-      </c>
-      <c r="F43" t="n" s="137">
-        <v>3.3617388144E8</v>
+      <c r="D43" t="n" s="136">
+        <v>-0.007756</v>
+      </c>
+      <c r="E43" t="n" s="137">
+        <v>-141919.45</v>
+      </c>
+      <c r="F43" t="s" s="18">
+        <v>21</v>
       </c>
       <c r="G43" t="n" s="138">
-        <v>2.474E8</v>
+        <v>-2.2418306E7</v>
       </c>
     </row>
     <row r="44">
@@ -2353,13 +2353,13 @@
         <v>106</v>
       </c>
       <c r="D44" t="n" s="139">
-        <v>-0.157031</v>
+        <v>-0.135936</v>
       </c>
       <c r="E44" t="n" s="140">
-        <v>1.1818775536E8</v>
+        <v>1.1920494267E8</v>
       </c>
       <c r="F44" t="n" s="141">
-        <v>1.1818775536E8</v>
+        <v>1.1920494267E8</v>
       </c>
       <c r="G44" t="n" s="142">
         <v>1.056E8</v>
@@ -2376,13 +2376,13 @@
         <v>109</v>
       </c>
       <c r="D45" t="n" s="143">
-        <v>-0.164769</v>
+        <v>-0.18935</v>
       </c>
       <c r="E45" t="n" s="144">
-        <v>1.7182890935E8</v>
+        <v>1.7181775551E8</v>
       </c>
       <c r="F45" t="n" s="145">
-        <v>1.7182890935E8</v>
+        <v>1.7181775551E8</v>
       </c>
       <c r="G45" t="n" s="146">
         <v>24880.0</v>
@@ -2399,16 +2399,16 @@
         <v>112</v>
       </c>
       <c r="D46" t="n" s="147">
-        <v>-0.423501</v>
+        <v>-0.351194</v>
       </c>
       <c r="E46" t="n" s="148">
-        <v>2.001158125E8</v>
+        <v>2.08398125E8</v>
       </c>
       <c r="F46" t="n" s="149">
-        <v>2.001158125E8</v>
+        <v>2.08398125E8</v>
       </c>
       <c r="G46" t="n" s="150">
-        <v>1.907E8</v>
+        <v>1.973E8</v>
       </c>
     </row>
     <row r="47">
@@ -2422,13 +2422,13 @@
         <v>115</v>
       </c>
       <c r="D47" t="n" s="151">
-        <v>-0.456279</v>
+        <v>-0.496091</v>
       </c>
       <c r="E47" t="n" s="152">
-        <v>1.7680425E8</v>
+        <v>1.760605E8</v>
       </c>
       <c r="F47" t="n" s="153">
-        <v>1.7680425E8</v>
+        <v>1.760605E8</v>
       </c>
       <c r="G47" t="n" s="154">
         <v>42500.0</v>
@@ -2445,13 +2445,13 @@
         <v>118</v>
       </c>
       <c r="D48" t="n" s="155">
-        <v>-0.635709</v>
+        <v>-0.620179</v>
       </c>
       <c r="E48" t="n" s="156">
-        <v>4.4278675E8</v>
+        <v>4.430496875E8</v>
       </c>
       <c r="F48" t="n" s="157">
-        <v>4.4278675E8</v>
+        <v>4.430496875E8</v>
       </c>
       <c r="G48" t="n" s="158">
         <v>4.207E8</v>

</xml_diff>

<commit_message>
Update ALLW XLSX 2026-10-22
</commit_message>
<xml_diff>
--- a/latest/allw-latest.xlsx
+++ b/latest/allw-latest.xlsx
@@ -192,7 +192,7 @@
     <t>ALLW</t>
   </si>
   <si>
-    <t>As of 20-Oct-2026</t>
+    <t>As of 21-Oct-2026</t>
   </si>
   <si>
     <t>Name</t>
@@ -240,18 +240,18 @@
     <t>912797TV9</t>
   </si>
   <si>
+    <t>TSY INFL IX N/B 07/35 1.875</t>
+  </si>
+  <si>
+    <t>91282CNS6</t>
+  </si>
+  <si>
     <t>US DOLLAR</t>
   </si>
   <si>
     <t>999USDZ92</t>
   </si>
   <si>
-    <t>TSY INFL IX N/B 07/35 1.875</t>
-  </si>
-  <si>
-    <t>91282CNS6</t>
-  </si>
-  <si>
     <t>STATE STREET SPDR PORTFOLIO EM</t>
   </si>
   <si>
@@ -390,15 +390,15 @@
     <t>912810SG4</t>
   </si>
   <si>
+    <t>EURO CURRENCY</t>
+  </si>
+  <si>
+    <t>999EURZ94</t>
+  </si>
+  <si>
     <t>TRS USD BCOMTR</t>
   </si>
   <si>
-    <t>EURO CURRENCY</t>
-  </si>
-  <si>
-    <t>999EURZ94</t>
-  </si>
-  <si>
     <t>POUND STERLING</t>
   </si>
   <si>
@@ -423,6 +423,42 @@
     <t>ADI391SG0</t>
   </si>
   <si>
+    <t>TOPIX INDX FUTR   DEC26</t>
+  </si>
+  <si>
+    <t>TPZ6</t>
+  </si>
+  <si>
+    <t>ADI3917X6</t>
+  </si>
+  <si>
+    <t>FTSE 100 IDX FUT  DEC26</t>
+  </si>
+  <si>
+    <t>Z Z6</t>
+  </si>
+  <si>
+    <t>ADI38QPG9</t>
+  </si>
+  <si>
+    <t>CANADIAN DOLLAR</t>
+  </si>
+  <si>
+    <t>999CADZ91</t>
+  </si>
+  <si>
+    <t>AUSTRALIAN DOLLAR</t>
+  </si>
+  <si>
+    <t>999AUDZ93</t>
+  </si>
+  <si>
+    <t>JAPANESE YEN</t>
+  </si>
+  <si>
+    <t>999JPYZ94</t>
+  </si>
+  <si>
     <t>EURO-BUND FUTURE  DEC26</t>
   </si>
   <si>
@@ -432,40 +468,13 @@
     <t>ADI39K4N9</t>
   </si>
   <si>
-    <t>CANADIAN DOLLAR</t>
-  </si>
-  <si>
-    <t>999CADZ91</t>
-  </si>
-  <si>
-    <t>TOPIX INDX FUTR   DEC26</t>
-  </si>
-  <si>
-    <t>TPZ6</t>
-  </si>
-  <si>
-    <t>ADI3917X6</t>
-  </si>
-  <si>
-    <t>FTSE 100 IDX FUT  DEC26</t>
-  </si>
-  <si>
-    <t>Z Z6</t>
-  </si>
-  <si>
-    <t>ADI38QPG9</t>
-  </si>
-  <si>
-    <t>AUSTRALIAN DOLLAR</t>
-  </si>
-  <si>
-    <t>999AUDZ93</t>
-  </si>
-  <si>
-    <t>JAPANESE YEN</t>
-  </si>
-  <si>
-    <t>999JPYZ94</t>
+    <t>EURO STOXX 50     DEC26</t>
+  </si>
+  <si>
+    <t>VGZ6</t>
+  </si>
+  <si>
+    <t>ADI2VHXS0</t>
   </si>
   <si>
     <t>LONG GILT FUTURE  DEC26</t>
@@ -475,15 +484,6 @@
   </si>
   <si>
     <t>ADI3BKVP1</t>
-  </si>
-  <si>
-    <t>EURO STOXX 50     DEC26</t>
-  </si>
-  <si>
-    <t>VGZ6</t>
-  </si>
-  <si>
-    <t>ADI2VHXS0</t>
   </si>
   <si>
     <t>US LONG BOND(CBT) DEC26</t>
@@ -918,109 +918,109 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
@@ -1479,16 +1479,16 @@
         <v>22</v>
       </c>
       <c r="D6" t="n" s="19">
-        <v>34.228802</v>
+        <v>34.220157</v>
       </c>
       <c r="E6" t="n" s="20">
-        <v>6.2635107145E8</v>
+        <v>6.2657007632E8</v>
       </c>
       <c r="F6" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G6" t="n" s="21">
-        <v>6.2635107145E8</v>
+        <v>6.2657007632E8</v>
       </c>
     </row>
     <row r="7">
@@ -1502,10 +1502,10 @@
         <v>25</v>
       </c>
       <c r="D7" t="n" s="22">
-        <v>13.505369</v>
+        <v>13.565821</v>
       </c>
       <c r="E7" t="n" s="23">
-        <v>2.4713404474E8</v>
+        <v>2.4838977942E8</v>
       </c>
       <c r="F7" t="s" s="18">
         <v>21</v>
@@ -1525,10 +1525,10 @@
         <v>27</v>
       </c>
       <c r="D8" t="n" s="25">
-        <v>4.942543</v>
+        <v>4.940418</v>
       </c>
       <c r="E8" t="n" s="26">
-        <v>9.044333495E7</v>
+        <v>9.045890836E7</v>
       </c>
       <c r="F8" t="s" s="18">
         <v>21</v>
@@ -1548,16 +1548,16 @@
         <v>29</v>
       </c>
       <c r="D9" t="n" s="28">
-        <v>4.280399</v>
+        <v>4.279961</v>
       </c>
       <c r="E9" t="n" s="29">
-        <v>7.83268028E7</v>
+        <v>7.836596287E7</v>
       </c>
       <c r="F9" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G9" t="n" s="30">
-        <v>7.83268028E7</v>
+        <v>8.3686251E7</v>
       </c>
     </row>
     <row r="10">
@@ -1571,16 +1571,16 @@
         <v>31</v>
       </c>
       <c r="D10" t="n" s="31">
-        <v>4.279586</v>
+        <v>4.265861</v>
       </c>
       <c r="E10" t="n" s="32">
-        <v>7.831193075E7</v>
+        <v>7.810779793E7</v>
       </c>
       <c r="F10" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G10" t="n" s="33">
-        <v>8.3677418E7</v>
+        <v>7.810779793E7</v>
       </c>
     </row>
     <row r="11">
@@ -1594,10 +1594,10 @@
         <v>34</v>
       </c>
       <c r="D11" t="n" s="34">
-        <v>4.208524</v>
+        <v>4.201033</v>
       </c>
       <c r="E11" t="n" s="35">
-        <v>7.7011557E7</v>
+        <v>7.6920795E7</v>
       </c>
       <c r="F11" t="s" s="18">
         <v>21</v>
@@ -1617,16 +1617,16 @@
         <v>36</v>
       </c>
       <c r="D12" t="n" s="37">
-        <v>4.188017</v>
+        <v>4.188898</v>
       </c>
       <c r="E12" t="n" s="38">
-        <v>7.66363121E7</v>
+        <v>7.669860214E7</v>
       </c>
       <c r="F12" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G12" t="n" s="39">
-        <v>8.2586752E7</v>
+        <v>8.2594772E7</v>
       </c>
     </row>
     <row r="13">
@@ -1640,16 +1640,16 @@
         <v>38</v>
       </c>
       <c r="D13" t="n" s="40">
-        <v>4.000574</v>
+        <v>4.000619</v>
       </c>
       <c r="E13" t="n" s="41">
-        <v>7.320629582E7</v>
+        <v>7.325122115E7</v>
       </c>
       <c r="F13" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G13" t="n" s="42">
-        <v>7.6444746E7</v>
+        <v>7.6452677E7</v>
       </c>
     </row>
     <row r="14">
@@ -1663,16 +1663,16 @@
         <v>40</v>
       </c>
       <c r="D14" t="n" s="43">
-        <v>3.690391</v>
+        <v>3.689842</v>
       </c>
       <c r="E14" t="n" s="44">
-        <v>6.753027559E7</v>
+        <v>6.756090423E7</v>
       </c>
       <c r="F14" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G14" t="n" s="45">
-        <v>7.125883875E7</v>
+        <v>7.12661895E7</v>
       </c>
     </row>
     <row r="15">
@@ -1686,16 +1686,16 @@
         <v>42</v>
       </c>
       <c r="D15" t="n" s="46">
-        <v>3.515182</v>
+        <v>3.514587</v>
       </c>
       <c r="E15" t="n" s="47">
-        <v>6.432413072E7</v>
+        <v>6.435198017E7</v>
       </c>
       <c r="F15" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G15" t="n" s="48">
-        <v>6.831070015E7</v>
+        <v>6.83176032E7</v>
       </c>
     </row>
     <row r="16">
@@ -1709,10 +1709,10 @@
         <v>45</v>
       </c>
       <c r="D16" t="n" s="49">
-        <v>3.227627</v>
+        <v>3.182175</v>
       </c>
       <c r="E16" t="n" s="50">
-        <v>5.906218525E7</v>
+        <v>5.826553621E7</v>
       </c>
       <c r="F16" t="s" s="18">
         <v>21</v>
@@ -1732,16 +1732,16 @@
         <v>47</v>
       </c>
       <c r="D17" t="n" s="52">
-        <v>2.532283</v>
+        <v>2.532595</v>
       </c>
       <c r="E17" t="n" s="53">
-        <v>4.633811006E7</v>
+        <v>4.637173395E7</v>
       </c>
       <c r="F17" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G17" t="n" s="54">
-        <v>4.789082E7</v>
+        <v>4.78956E7</v>
       </c>
     </row>
     <row r="18">
@@ -1755,16 +1755,16 @@
         <v>49</v>
       </c>
       <c r="D18" t="n" s="55">
-        <v>1.492908</v>
+        <v>1.495737</v>
       </c>
       <c r="E18" t="n" s="56">
-        <v>2.731865344E7</v>
+        <v>2.73869098E7</v>
       </c>
       <c r="F18" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G18" t="n" s="57">
-        <v>3.5619717E7</v>
+        <v>3.56234385E7</v>
       </c>
     </row>
     <row r="19">
@@ -1778,16 +1778,16 @@
         <v>51</v>
       </c>
       <c r="D19" t="n" s="58">
-        <v>1.322755</v>
+        <v>1.325698</v>
       </c>
       <c r="E19" t="n" s="59">
-        <v>2.42050282E7</v>
+        <v>2.427349561E7</v>
       </c>
       <c r="F19" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G19" t="n" s="60">
-        <v>3.628344755E7</v>
+        <v>3.62872778E7</v>
       </c>
     </row>
     <row r="20">
@@ -1801,16 +1801,16 @@
         <v>53</v>
       </c>
       <c r="D20" t="n" s="61">
-        <v>1.246093</v>
+        <v>1.249254</v>
       </c>
       <c r="E20" t="n" s="62">
-        <v>2.280218322E7</v>
+        <v>2.287380291E7</v>
       </c>
       <c r="F20" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G20" t="n" s="63">
-        <v>2.68594254E7</v>
+        <v>2.68622117E7</v>
       </c>
     </row>
     <row r="21">
@@ -1824,16 +1824,16 @@
         <v>55</v>
       </c>
       <c r="D21" t="n" s="64">
-        <v>1.172605</v>
+        <v>1.175579</v>
       </c>
       <c r="E21" t="n" s="65">
-        <v>2.145743597E7</v>
+        <v>2.152481804E7</v>
       </c>
       <c r="F21" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G21" t="n" s="66">
-        <v>2.662935625E7</v>
+        <v>2.663228725E7</v>
       </c>
     </row>
     <row r="22">
@@ -1847,16 +1847,16 @@
         <v>57</v>
       </c>
       <c r="D22" t="n" s="67">
-        <v>1.148905</v>
+        <v>1.151972</v>
       </c>
       <c r="E22" t="n" s="68">
-        <v>2.102374705E7</v>
+        <v>2.109257637E7</v>
       </c>
       <c r="F22" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G22" t="n" s="69">
-        <v>2.47788E7</v>
+        <v>2.47812E7</v>
       </c>
     </row>
     <row r="23">
@@ -1870,16 +1870,16 @@
         <v>59</v>
       </c>
       <c r="D23" t="n" s="70">
-        <v>1.10903</v>
+        <v>1.110795</v>
       </c>
       <c r="E23" t="n" s="71">
-        <v>2.02940771E7</v>
+        <v>2.033862809E7</v>
       </c>
       <c r="F23" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G23" t="n" s="72">
-        <v>2.8253664E7</v>
+        <v>2.8256526E7</v>
       </c>
     </row>
     <row r="24">
@@ -1893,16 +1893,16 @@
         <v>61</v>
       </c>
       <c r="D24" t="n" s="73">
-        <v>0.960937</v>
+        <v>0.963211</v>
       </c>
       <c r="E24" t="n" s="74">
-        <v>1.758414354E7</v>
+        <v>1.763636501E7</v>
       </c>
       <c r="F24" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G24" t="n" s="75">
-        <v>2.5101995E7</v>
+        <v>2.5104448E7</v>
       </c>
     </row>
     <row r="25">
@@ -1916,16 +1916,16 @@
         <v>63</v>
       </c>
       <c r="D25" t="n" s="76">
-        <v>0.936854</v>
+        <v>0.938601</v>
       </c>
       <c r="E25" t="n" s="77">
-        <v>1.714343453E7</v>
+        <v>1.718576148E7</v>
       </c>
       <c r="F25" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G25" t="n" s="78">
-        <v>2.50176384E7</v>
+        <v>2.50202169E7</v>
       </c>
     </row>
     <row r="26">
@@ -1939,16 +1939,16 @@
         <v>65</v>
       </c>
       <c r="D26" t="n" s="79">
-        <v>0.893769</v>
+        <v>0.895816</v>
       </c>
       <c r="E26" t="n" s="80">
-        <v>1.635502393E7</v>
+        <v>1.640236081E7</v>
       </c>
       <c r="F26" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G26" t="n" s="81">
-        <v>2.4881213E7</v>
+        <v>2.4883726E7</v>
       </c>
     </row>
     <row r="27">
@@ -1962,16 +1962,16 @@
         <v>67</v>
       </c>
       <c r="D27" t="n" s="82">
-        <v>0.738021</v>
+        <v>0.739595</v>
       </c>
       <c r="E27" t="n" s="83">
-        <v>1.350501461E7</v>
+        <v>1.354195987E7</v>
       </c>
       <c r="F27" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G27" t="n" s="84">
-        <v>1.96007808E7</v>
+        <v>1.9602724E7</v>
       </c>
     </row>
     <row r="28">
@@ -1985,16 +1985,16 @@
         <v>69</v>
       </c>
       <c r="D28" t="n" s="85">
-        <v>0.733473</v>
+        <v>0.735992</v>
       </c>
       <c r="E28" t="n" s="86">
-        <v>1.342179351E7</v>
+        <v>1.347599582E7</v>
       </c>
       <c r="F28" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G28" t="n" s="87">
-        <v>2.8487163E7</v>
+        <v>2.8490007E7</v>
       </c>
     </row>
     <row r="29">
@@ -2008,16 +2008,16 @@
         <v>71</v>
       </c>
       <c r="D29" t="n" s="88">
-        <v>0.723808</v>
+        <v>0.726059</v>
       </c>
       <c r="E29" t="n" s="89">
-        <v>1.324491959E7</v>
+        <v>1.329411335E7</v>
       </c>
       <c r="F29" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G29" t="n" s="90">
-        <v>2.55285302E7</v>
+        <v>2.553108015E7</v>
       </c>
     </row>
     <row r="30">
@@ -2031,16 +2031,16 @@
         <v>73</v>
       </c>
       <c r="D30" t="n" s="91">
-        <v>0.612142</v>
+        <v>0.614323</v>
       </c>
       <c r="E30" t="n" s="92">
-        <v>1.120154739E7</v>
+        <v>1.124824372E7</v>
       </c>
       <c r="F30" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G30" t="n" s="93">
-        <v>2.3095044E7</v>
+        <v>2.30973801E7</v>
       </c>
     </row>
     <row r="31">
@@ -2054,16 +2054,16 @@
         <v>75</v>
       </c>
       <c r="D31" t="n" s="94">
-        <v>0.575697</v>
+        <v>0.57715</v>
       </c>
       <c r="E31" t="n" s="95">
-        <v>1.053464751E7</v>
+        <v>1.056759716E7</v>
       </c>
       <c r="F31" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G31" t="n" s="96">
-        <v>1.5875613E7</v>
+        <v>1.5877134E7</v>
       </c>
     </row>
     <row r="32">
@@ -2077,16 +2077,16 @@
         <v>77</v>
       </c>
       <c r="D32" t="n" s="97">
-        <v>0.563688</v>
+        <v>0.565042</v>
       </c>
       <c r="E32" t="n" s="98">
-        <v>1.031489424E7</v>
+        <v>1.034589861E7</v>
       </c>
       <c r="F32" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G32" t="n" s="99">
-        <v>1.579030625E7</v>
+        <v>1.579196875E7</v>
       </c>
     </row>
     <row r="33">
@@ -2097,42 +2097,42 @@
         <v>21</v>
       </c>
       <c r="C33" t="s" s="18">
-        <v>21</v>
+        <v>79</v>
       </c>
       <c r="D33" t="n" s="100">
-        <v>0.296468</v>
+        <v>0.266484</v>
       </c>
       <c r="E33" t="n" s="101">
-        <v>5425049.61</v>
-      </c>
-      <c r="F33" t="n" s="102">
-        <v>4.1426456199E8</v>
-      </c>
-      <c r="G33" t="n" s="103">
-        <v>1128643.27</v>
+        <v>4879312.98</v>
+      </c>
+      <c r="F33" t="s" s="18">
+        <v>21</v>
+      </c>
+      <c r="G33" t="n" s="102">
+        <v>4347214.14</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s" s="18">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B34" t="s" s="18">
         <v>21</v>
       </c>
       <c r="C34" t="s" s="18">
-        <v>80</v>
-      </c>
-      <c r="D34" t="n" s="104">
-        <v>0.267155</v>
-      </c>
-      <c r="E34" t="n" s="105">
-        <v>4888657.39</v>
-      </c>
-      <c r="F34" t="s" s="18">
-        <v>21</v>
+        <v>21</v>
+      </c>
+      <c r="D34" t="n" s="103">
+        <v>0.199538</v>
+      </c>
+      <c r="E34" t="n" s="104">
+        <v>3653531.14</v>
+      </c>
+      <c r="F34" t="n" s="105">
+        <v>4.1426456199E8</v>
       </c>
       <c r="G34" t="n" s="106">
-        <v>4347214.14</v>
+        <v>1128643.27</v>
       </c>
     </row>
     <row r="35">
@@ -2146,10 +2146,10 @@
         <v>82</v>
       </c>
       <c r="D35" t="n" s="107">
-        <v>0.14876</v>
+        <v>0.148631</v>
       </c>
       <c r="E35" t="n" s="108">
-        <v>2722143.27</v>
+        <v>2721429.18</v>
       </c>
       <c r="F35" t="s" s="18">
         <v>21</v>
@@ -2169,13 +2169,13 @@
         <v>85</v>
       </c>
       <c r="D36" t="n" s="110">
-        <v>0.094276</v>
+        <v>0.076665</v>
       </c>
       <c r="E36" t="n" s="111">
-        <v>1.7259561455E8</v>
+        <v>1.7268858458E8</v>
       </c>
       <c r="F36" t="n" s="112">
-        <v>1.7259561455E8</v>
+        <v>1.7268858458E8</v>
       </c>
       <c r="G36" t="n" s="113">
         <v>2.331E8</v>
@@ -2192,13 +2192,13 @@
         <v>88</v>
       </c>
       <c r="D37" t="n" s="114">
-        <v>0.038515</v>
+        <v>0.044932</v>
       </c>
       <c r="E37" t="n" s="115">
-        <v>6.82786491E7</v>
+        <v>6.856045513E7</v>
       </c>
       <c r="F37" t="n" s="116">
-        <v>6.82786491E7</v>
+        <v>6.856045513E7</v>
       </c>
       <c r="G37" t="n" s="117">
         <v>11025.0</v>
@@ -2215,16 +2215,16 @@
         <v>91</v>
       </c>
       <c r="D38" t="n" s="118">
-        <v>0.002558</v>
+        <v>0.029882</v>
       </c>
       <c r="E38" t="n" s="119">
-        <v>3.3861370039E8</v>
+        <v>8.662445843E7</v>
       </c>
       <c r="F38" t="n" s="120">
-        <v>3.3861370039E8</v>
+        <v>8.662445843E7</v>
       </c>
       <c r="G38" t="n" s="121">
-        <v>2.474E8</v>
+        <v>3380000.0</v>
       </c>
     </row>
     <row r="39">
@@ -2232,45 +2232,45 @@
         <v>92</v>
       </c>
       <c r="B39" t="s" s="18">
-        <v>21</v>
+        <v>93</v>
       </c>
       <c r="C39" t="s" s="18">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D39" t="n" s="122">
-        <v>0.0</v>
+        <v>0.00358</v>
       </c>
       <c r="E39" t="n" s="123">
-        <v>7.53</v>
-      </c>
-      <c r="F39" t="s" s="18">
-        <v>21</v>
-      </c>
-      <c r="G39" t="n" s="124">
-        <v>10.58</v>
+        <v>7.305620877E7</v>
+      </c>
+      <c r="F39" t="n" s="124">
+        <v>7.305620877E7</v>
+      </c>
+      <c r="G39" t="n" s="125">
+        <v>5060.0</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s" s="18">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B40" t="s" s="18">
-        <v>95</v>
+        <v>21</v>
       </c>
       <c r="C40" t="s" s="18">
         <v>96</v>
       </c>
-      <c r="D40" t="n" s="125">
-        <v>-0.001645</v>
-      </c>
-      <c r="E40" t="n" s="126">
-        <v>8.612350837E7</v>
-      </c>
-      <c r="F40" t="n" s="127">
-        <v>8.612350837E7</v>
+      <c r="D40" t="n" s="126">
+        <v>0.0</v>
+      </c>
+      <c r="E40" t="n" s="127">
+        <v>7.52</v>
+      </c>
+      <c r="F40" t="s" s="18">
+        <v>21</v>
       </c>
       <c r="G40" t="n" s="128">
-        <v>3380000.0</v>
+        <v>10.58</v>
       </c>
     </row>
     <row r="41">
@@ -2278,68 +2278,68 @@
         <v>97</v>
       </c>
       <c r="B41" t="s" s="18">
+        <v>21</v>
+      </c>
+      <c r="C41" t="s" s="18">
         <v>98</v>
       </c>
-      <c r="C41" t="s" s="18">
-        <v>99</v>
-      </c>
       <c r="D41" t="n" s="129">
-        <v>-0.004006</v>
+        <v>-0.006831</v>
       </c>
       <c r="E41" t="n" s="130">
-        <v>7.293650974E7</v>
-      </c>
-      <c r="F41" t="n" s="131">
-        <v>7.293650974E7</v>
-      </c>
-      <c r="G41" t="n" s="132">
-        <v>5060.0</v>
+        <v>-125072.8</v>
+      </c>
+      <c r="F41" t="s" s="18">
+        <v>21</v>
+      </c>
+      <c r="G41" t="n" s="131">
+        <v>-177976.22</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s" s="18">
+        <v>99</v>
+      </c>
+      <c r="B42" t="s" s="18">
+        <v>21</v>
+      </c>
+      <c r="C42" t="s" s="18">
         <v>100</v>
       </c>
-      <c r="B42" t="s" s="18">
-        <v>21</v>
-      </c>
-      <c r="C42" t="s" s="18">
-        <v>101</v>
-      </c>
-      <c r="D42" t="n" s="133">
-        <v>-0.006818</v>
-      </c>
-      <c r="E42" t="n" s="134">
-        <v>-124770.21</v>
+      <c r="D42" t="n" s="132">
+        <v>-0.007744</v>
+      </c>
+      <c r="E42" t="n" s="133">
+        <v>-141793.78</v>
       </c>
       <c r="F42" t="s" s="18">
         <v>21</v>
       </c>
-      <c r="G42" t="n" s="135">
-        <v>-177976.22</v>
+      <c r="G42" t="n" s="134">
+        <v>-2.2418306E7</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="s" s="18">
+        <v>101</v>
+      </c>
+      <c r="B43" t="s" s="18">
         <v>102</v>
-      </c>
-      <c r="B43" t="s" s="18">
-        <v>21</v>
       </c>
       <c r="C43" t="s" s="18">
         <v>103</v>
       </c>
-      <c r="D43" t="n" s="136">
-        <v>-0.007756</v>
-      </c>
-      <c r="E43" t="n" s="137">
-        <v>-141919.45</v>
-      </c>
-      <c r="F43" t="s" s="18">
-        <v>21</v>
+      <c r="D43" t="n" s="135">
+        <v>-0.042945</v>
+      </c>
+      <c r="E43" t="n" s="136">
+        <v>3.3713341295E8</v>
+      </c>
+      <c r="F43" t="n" s="137">
+        <v>3.3713341295E8</v>
       </c>
       <c r="G43" t="n" s="138">
-        <v>-2.2418306E7</v>
+        <v>2.474E8</v>
       </c>
     </row>
     <row r="44">
@@ -2353,16 +2353,16 @@
         <v>106</v>
       </c>
       <c r="D44" t="n" s="139">
-        <v>-0.135936</v>
+        <v>-0.068388</v>
       </c>
       <c r="E44" t="n" s="140">
-        <v>1.1920494267E8</v>
+        <v>1.7369543453E8</v>
       </c>
       <c r="F44" t="n" s="141">
-        <v>1.1920494267E8</v>
+        <v>1.7369543453E8</v>
       </c>
       <c r="G44" t="n" s="142">
-        <v>1.056E8</v>
+        <v>24880.0</v>
       </c>
     </row>
     <row r="45">
@@ -2376,16 +2376,16 @@
         <v>109</v>
       </c>
       <c r="D45" t="n" s="143">
-        <v>-0.18935</v>
+        <v>-0.120381</v>
       </c>
       <c r="E45" t="n" s="144">
-        <v>1.7181775551E8</v>
+        <v>1.1945634207E8</v>
       </c>
       <c r="F45" t="n" s="145">
-        <v>1.7181775551E8</v>
+        <v>1.1945634207E8</v>
       </c>
       <c r="G45" t="n" s="146">
-        <v>24880.0</v>
+        <v>1.056E8</v>
       </c>
     </row>
     <row r="46">
@@ -2399,13 +2399,13 @@
         <v>112</v>
       </c>
       <c r="D46" t="n" s="147">
-        <v>-0.351194</v>
+        <v>-0.361084</v>
       </c>
       <c r="E46" t="n" s="148">
-        <v>2.08398125E8</v>
+        <v>2.0821315625E8</v>
       </c>
       <c r="F46" t="n" s="149">
-        <v>2.08398125E8</v>
+        <v>2.0821315625E8</v>
       </c>
       <c r="G46" t="n" s="150">
         <v>1.973E8</v>
@@ -2422,13 +2422,13 @@
         <v>115</v>
       </c>
       <c r="D47" t="n" s="151">
-        <v>-0.496091</v>
+        <v>-0.478616</v>
       </c>
       <c r="E47" t="n" s="152">
-        <v>1.760605E8</v>
+        <v>1.76375E8</v>
       </c>
       <c r="F47" t="n" s="153">
-        <v>1.760605E8</v>
+        <v>1.76375E8</v>
       </c>
       <c r="G47" t="n" s="154">
         <v>42500.0</v>
@@ -2445,13 +2445,13 @@
         <v>118</v>
       </c>
       <c r="D48" t="n" s="155">
-        <v>-0.620179</v>
+        <v>-0.666477</v>
       </c>
       <c r="E48" t="n" s="156">
-        <v>4.430496875E8</v>
+        <v>4.4219514063E8</v>
       </c>
       <c r="F48" t="n" s="157">
-        <v>4.430496875E8</v>
+        <v>4.4219514063E8</v>
       </c>
       <c r="G48" t="n" s="158">
         <v>4.207E8</v>

</xml_diff>

<commit_message>
Update ALLW XLSX 2026-10-23
</commit_message>
<xml_diff>
--- a/latest/allw-latest.xlsx
+++ b/latest/allw-latest.xlsx
@@ -192,7 +192,7 @@
     <t>ALLW</t>
   </si>
   <si>
-    <t>As of 21-Oct-2026</t>
+    <t>As of 22-Oct-2026</t>
   </si>
   <si>
     <t>Name</t>
@@ -252,6 +252,12 @@
     <t>999USDZ92</t>
   </si>
   <si>
+    <t>TSY INFL IX N/B 01/36 1.875</t>
+  </si>
+  <si>
+    <t>91282CPU9</t>
+  </si>
+  <si>
     <t>STATE STREET SPDR PORTFOLIO EM</t>
   </si>
   <si>
@@ -261,12 +267,6 @@
     <t>78463X509</t>
   </si>
   <si>
-    <t>TSY INFL IX N/B 01/36 1.875</t>
-  </si>
-  <si>
-    <t>91282CPU9</t>
-  </si>
-  <si>
     <t>TSY INFL IX N/B 01/35 2.125</t>
   </si>
   <si>
@@ -354,18 +354,18 @@
     <t>912810RW0</t>
   </si>
   <si>
+    <t>TSY INFL IX N/B 02/52 0.125</t>
+  </si>
+  <si>
+    <t>912810TE8</t>
+  </si>
+  <si>
     <t>TSY INFL IX N/B 02/46 1</t>
   </si>
   <si>
     <t>912810RR1</t>
   </si>
   <si>
-    <t>TSY INFL IX N/B 02/52 0.125</t>
-  </si>
-  <si>
-    <t>912810TE8</t>
-  </si>
-  <si>
     <t>TSY INFL IX N/B 02/50 0.25</t>
   </si>
   <si>
@@ -414,6 +414,15 @@
     <t>ADI3BDHZ1</t>
   </si>
   <si>
+    <t>EURO-BUND FUTURE  DEC26</t>
+  </si>
+  <si>
+    <t>RXZ6</t>
+  </si>
+  <si>
+    <t>ADI39K4N9</t>
+  </si>
+  <si>
     <t>SPI 200 FUTURES   DEC26</t>
   </si>
   <si>
@@ -423,6 +432,33 @@
     <t>ADI391SG0</t>
   </si>
   <si>
+    <t>CANADIAN DOLLAR</t>
+  </si>
+  <si>
+    <t>999CADZ91</t>
+  </si>
+  <si>
+    <t>AUSTRALIAN DOLLAR</t>
+  </si>
+  <si>
+    <t>999AUDZ93</t>
+  </si>
+  <si>
+    <t>FTSE 100 IDX FUT  DEC26</t>
+  </si>
+  <si>
+    <t>Z Z6</t>
+  </si>
+  <si>
+    <t>ADI38QPG9</t>
+  </si>
+  <si>
+    <t>JAPANESE YEN</t>
+  </si>
+  <si>
+    <t>999JPYZ94</t>
+  </si>
+  <si>
     <t>TOPIX INDX FUTR   DEC26</t>
   </si>
   <si>
@@ -432,40 +468,22 @@
     <t>ADI3917X6</t>
   </si>
   <si>
-    <t>FTSE 100 IDX FUT  DEC26</t>
-  </si>
-  <si>
-    <t>Z Z6</t>
-  </si>
-  <si>
-    <t>ADI38QPG9</t>
-  </si>
-  <si>
-    <t>CANADIAN DOLLAR</t>
-  </si>
-  <si>
-    <t>999CADZ91</t>
-  </si>
-  <si>
-    <t>AUSTRALIAN DOLLAR</t>
-  </si>
-  <si>
-    <t>999AUDZ93</t>
-  </si>
-  <si>
-    <t>JAPANESE YEN</t>
-  </si>
-  <si>
-    <t>999JPYZ94</t>
-  </si>
-  <si>
-    <t>EURO-BUND FUTURE  DEC26</t>
-  </si>
-  <si>
-    <t>RXZ6</t>
-  </si>
-  <si>
-    <t>ADI39K4N9</t>
+    <t>LONG GILT FUTURE  DEC26</t>
+  </si>
+  <si>
+    <t>G Z6</t>
+  </si>
+  <si>
+    <t>ADI3BKVP1</t>
+  </si>
+  <si>
+    <t>US LONG BOND(CBT) DEC26</t>
+  </si>
+  <si>
+    <t>USZ6</t>
+  </si>
+  <si>
+    <t>ADI39KYC0</t>
   </si>
   <si>
     <t>EURO STOXX 50     DEC26</t>
@@ -477,22 +495,13 @@
     <t>ADI2VHXS0</t>
   </si>
   <si>
-    <t>LONG GILT FUTURE  DEC26</t>
-  </si>
-  <si>
-    <t>G Z6</t>
-  </si>
-  <si>
-    <t>ADI3BKVP1</t>
-  </si>
-  <si>
-    <t>US LONG BOND(CBT) DEC26</t>
-  </si>
-  <si>
-    <t>USZ6</t>
-  </si>
-  <si>
-    <t>ADI39KYC0</t>
+    <t>US 10YR NOTE (CBT)DEC26</t>
+  </si>
+  <si>
+    <t>TYZ6</t>
+  </si>
+  <si>
+    <t>ADI39DKR8</t>
   </si>
   <si>
     <t>GOLD 100 OZ FUTR  DEC26</t>
@@ -502,15 +511,6 @@
   </si>
   <si>
     <t>ADI2XJBP4</t>
-  </si>
-  <si>
-    <t>US 10YR NOTE (CBT)DEC26</t>
-  </si>
-  <si>
-    <t>TYZ6</t>
-  </si>
-  <si>
-    <t>ADI39DKR8</t>
   </si>
 </sst>
 </file>
@@ -984,22 +984,22 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
@@ -1479,16 +1479,16 @@
         <v>22</v>
       </c>
       <c r="D6" t="n" s="19">
-        <v>34.220157</v>
+        <v>34.098448</v>
       </c>
       <c r="E6" t="n" s="20">
-        <v>6.2657007632E8</v>
+        <v>6.2787208547E8</v>
       </c>
       <c r="F6" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G6" t="n" s="21">
-        <v>6.2657007632E8</v>
+        <v>6.2787208547E8</v>
       </c>
     </row>
     <row r="7">
@@ -1502,10 +1502,10 @@
         <v>25</v>
       </c>
       <c r="D7" t="n" s="22">
-        <v>13.565821</v>
+        <v>13.332392</v>
       </c>
       <c r="E7" t="n" s="23">
-        <v>2.4838977942E8</v>
+        <v>2.4549612994E8</v>
       </c>
       <c r="F7" t="s" s="18">
         <v>21</v>
@@ -1525,10 +1525,10 @@
         <v>27</v>
       </c>
       <c r="D8" t="n" s="25">
-        <v>4.940418</v>
+        <v>4.91362</v>
       </c>
       <c r="E8" t="n" s="26">
-        <v>9.045890836E7</v>
+        <v>9.047699527E7</v>
       </c>
       <c r="F8" t="s" s="18">
         <v>21</v>
@@ -1548,16 +1548,16 @@
         <v>29</v>
       </c>
       <c r="D9" t="n" s="28">
-        <v>4.279961</v>
+        <v>4.298224</v>
       </c>
       <c r="E9" t="n" s="29">
-        <v>7.836596287E7</v>
+        <v>7.9145395E7</v>
       </c>
       <c r="F9" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G9" t="n" s="30">
-        <v>8.3686251E7</v>
+        <v>8.3711947E7</v>
       </c>
     </row>
     <row r="10">
@@ -1571,16 +1571,16 @@
         <v>31</v>
       </c>
       <c r="D10" t="n" s="31">
-        <v>4.265861</v>
+        <v>4.236269</v>
       </c>
       <c r="E10" t="n" s="32">
-        <v>7.810779793E7</v>
+        <v>7.800457963E7</v>
       </c>
       <c r="F10" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G10" t="n" s="33">
-        <v>7.810779793E7</v>
+        <v>7.800457963E7</v>
       </c>
     </row>
     <row r="11">
@@ -1588,45 +1588,45 @@
         <v>32</v>
       </c>
       <c r="B11" t="s" s="18">
+        <v>21</v>
+      </c>
+      <c r="C11" t="s" s="18">
         <v>33</v>
       </c>
-      <c r="C11" t="s" s="18">
-        <v>34</v>
-      </c>
       <c r="D11" t="n" s="34">
-        <v>4.201033</v>
+        <v>4.208441</v>
       </c>
       <c r="E11" t="n" s="35">
-        <v>7.6920795E7</v>
+        <v>7.749215993E7</v>
       </c>
       <c r="F11" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G11" t="n" s="36">
-        <v>1512700.0</v>
+        <v>8.2620436E7</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s" s="18">
+        <v>34</v>
+      </c>
+      <c r="B12" t="s" s="18">
         <v>35</v>
-      </c>
-      <c r="B12" t="s" s="18">
-        <v>21</v>
       </c>
       <c r="C12" t="s" s="18">
         <v>36</v>
       </c>
       <c r="D12" t="n" s="37">
-        <v>4.188898</v>
+        <v>4.07965</v>
       </c>
       <c r="E12" t="n" s="38">
-        <v>7.669860214E7</v>
+        <v>7.5120682E7</v>
       </c>
       <c r="F12" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G12" t="n" s="39">
-        <v>8.2594772E7</v>
+        <v>1512700.0</v>
       </c>
     </row>
     <row r="13">
@@ -1640,16 +1640,16 @@
         <v>38</v>
       </c>
       <c r="D13" t="n" s="40">
-        <v>4.000619</v>
+        <v>4.016152</v>
       </c>
       <c r="E13" t="n" s="41">
-        <v>7.325122115E7</v>
+        <v>7.395145201E7</v>
       </c>
       <c r="F13" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G13" t="n" s="42">
-        <v>7.6452677E7</v>
+        <v>7.6475749E7</v>
       </c>
     </row>
     <row r="14">
@@ -1663,16 +1663,16 @@
         <v>40</v>
       </c>
       <c r="D14" t="n" s="43">
-        <v>3.689842</v>
+        <v>3.702971</v>
       </c>
       <c r="E14" t="n" s="44">
-        <v>6.756090423E7</v>
+        <v>6.818469674E7</v>
       </c>
       <c r="F14" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G14" t="n" s="45">
-        <v>7.12661895E7</v>
+        <v>7.128824175E7</v>
       </c>
     </row>
     <row r="15">
@@ -1686,16 +1686,16 @@
         <v>42</v>
       </c>
       <c r="D15" t="n" s="46">
-        <v>3.514587</v>
+        <v>3.525603</v>
       </c>
       <c r="E15" t="n" s="47">
-        <v>6.435198017E7</v>
+        <v>6.491872744E7</v>
       </c>
       <c r="F15" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G15" t="n" s="48">
-        <v>6.83176032E7</v>
+        <v>6.833831235E7</v>
       </c>
     </row>
     <row r="16">
@@ -1709,16 +1709,16 @@
         <v>45</v>
       </c>
       <c r="D16" t="n" s="49">
-        <v>3.182175</v>
+        <v>3.187357</v>
       </c>
       <c r="E16" t="n" s="50">
-        <v>5.826553621E7</v>
+        <v>5.869042822E7</v>
       </c>
       <c r="F16" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G16" t="n" s="51">
-        <v>702079.0</v>
+        <v>723323.0</v>
       </c>
     </row>
     <row r="17">
@@ -1732,16 +1732,16 @@
         <v>47</v>
       </c>
       <c r="D17" t="n" s="52">
-        <v>2.532595</v>
+        <v>2.545406</v>
       </c>
       <c r="E17" t="n" s="53">
-        <v>4.637173395E7</v>
+        <v>4.686986361E7</v>
       </c>
       <c r="F17" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G17" t="n" s="54">
-        <v>4.78956E7</v>
+        <v>4.7910418E7</v>
       </c>
     </row>
     <row r="18">
@@ -1755,16 +1755,16 @@
         <v>49</v>
       </c>
       <c r="D18" t="n" s="55">
-        <v>1.495737</v>
+        <v>1.50963</v>
       </c>
       <c r="E18" t="n" s="56">
-        <v>2.73869098E7</v>
+        <v>2.779758093E7</v>
       </c>
       <c r="F18" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G18" t="n" s="57">
-        <v>3.56234385E7</v>
+        <v>3.56343549E7</v>
       </c>
     </row>
     <row r="19">
@@ -1778,16 +1778,16 @@
         <v>51</v>
       </c>
       <c r="D19" t="n" s="58">
-        <v>1.325698</v>
+        <v>1.340319</v>
       </c>
       <c r="E19" t="n" s="59">
-        <v>2.427349561E7</v>
+        <v>2.467997972E7</v>
       </c>
       <c r="F19" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G19" t="n" s="60">
-        <v>3.62872778E7</v>
+        <v>3.629825785E7</v>
       </c>
     </row>
     <row r="20">
@@ -1801,16 +1801,16 @@
         <v>53</v>
       </c>
       <c r="D20" t="n" s="61">
-        <v>1.249254</v>
+        <v>1.266187</v>
       </c>
       <c r="E20" t="n" s="62">
-        <v>2.287380291E7</v>
+        <v>2.33149433E7</v>
       </c>
       <c r="F20" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G20" t="n" s="63">
-        <v>2.68622117E7</v>
+        <v>2.68705706E7</v>
       </c>
     </row>
     <row r="21">
@@ -1824,16 +1824,16 @@
         <v>55</v>
       </c>
       <c r="D21" t="n" s="64">
-        <v>1.175579</v>
+        <v>1.191533</v>
       </c>
       <c r="E21" t="n" s="65">
-        <v>2.152481804E7</v>
+        <v>2.194030341E7</v>
       </c>
       <c r="F21" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G21" t="n" s="66">
-        <v>2.663228725E7</v>
+        <v>2.66403475E7</v>
       </c>
     </row>
     <row r="22">
@@ -1847,16 +1847,16 @@
         <v>57</v>
       </c>
       <c r="D22" t="n" s="67">
-        <v>1.151972</v>
+        <v>1.168226</v>
       </c>
       <c r="E22" t="n" s="68">
-        <v>2.109257637E7</v>
+        <v>2.151113167E7</v>
       </c>
       <c r="F22" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G22" t="n" s="69">
-        <v>2.47812E7</v>
+        <v>2.478888E7</v>
       </c>
     </row>
     <row r="23">
@@ -1870,16 +1870,16 @@
         <v>59</v>
       </c>
       <c r="D23" t="n" s="70">
-        <v>1.110795</v>
+        <v>1.121082</v>
       </c>
       <c r="E23" t="n" s="71">
-        <v>2.033862809E7</v>
+        <v>2.064305597E7</v>
       </c>
       <c r="F23" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G23" t="n" s="72">
-        <v>2.8256526E7</v>
+        <v>2.82653028E7</v>
       </c>
     </row>
     <row r="24">
@@ -1893,16 +1893,16 @@
         <v>61</v>
       </c>
       <c r="D24" t="n" s="73">
-        <v>0.963211</v>
+        <v>0.977111</v>
       </c>
       <c r="E24" t="n" s="74">
-        <v>1.763636501E7</v>
+        <v>1.799204633E7</v>
       </c>
       <c r="F24" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G24" t="n" s="75">
-        <v>2.5104448E7</v>
+        <v>2.5112253E7</v>
       </c>
     </row>
     <row r="25">
@@ -1916,16 +1916,16 @@
         <v>63</v>
       </c>
       <c r="D25" t="n" s="76">
-        <v>0.938601</v>
+        <v>0.94808</v>
       </c>
       <c r="E25" t="n" s="77">
-        <v>1.718576148E7</v>
+        <v>1.745748559E7</v>
       </c>
       <c r="F25" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G25" t="n" s="78">
-        <v>2.50202169E7</v>
+        <v>2.50279524E7</v>
       </c>
     </row>
     <row r="26">
@@ -1939,16 +1939,16 @@
         <v>65</v>
       </c>
       <c r="D26" t="n" s="79">
-        <v>0.895816</v>
+        <v>0.90658</v>
       </c>
       <c r="E26" t="n" s="80">
-        <v>1.640236081E7</v>
+        <v>1.66933111E7</v>
       </c>
       <c r="F26" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G26" t="n" s="81">
-        <v>2.4883726E7</v>
+        <v>2.48914445E7</v>
       </c>
     </row>
     <row r="27">
@@ -1962,16 +1962,16 @@
         <v>67</v>
       </c>
       <c r="D27" t="n" s="82">
-        <v>0.739595</v>
+        <v>0.749249</v>
       </c>
       <c r="E27" t="n" s="83">
-        <v>1.354195987E7</v>
+        <v>1.379630192E7</v>
       </c>
       <c r="F27" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G27" t="n" s="84">
-        <v>1.9602724E7</v>
+        <v>2.8498776E7</v>
       </c>
     </row>
     <row r="28">
@@ -1985,16 +1985,16 @@
         <v>69</v>
       </c>
       <c r="D28" t="n" s="85">
-        <v>0.735992</v>
+        <v>0.747604</v>
       </c>
       <c r="E28" t="n" s="86">
-        <v>1.347599582E7</v>
+        <v>1.376601228E7</v>
       </c>
       <c r="F28" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G28" t="n" s="87">
-        <v>2.8490007E7</v>
+        <v>1.96088312E7</v>
       </c>
     </row>
     <row r="29">
@@ -2008,16 +2008,16 @@
         <v>71</v>
       </c>
       <c r="D29" t="n" s="88">
-        <v>0.726059</v>
+        <v>0.737666</v>
       </c>
       <c r="E29" t="n" s="89">
-        <v>1.329411335E7</v>
+        <v>1.358301757E7</v>
       </c>
       <c r="F29" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G29" t="n" s="90">
-        <v>2.553108015E7</v>
+        <v>2.553892615E7</v>
       </c>
     </row>
     <row r="30">
@@ -2031,16 +2031,16 @@
         <v>73</v>
       </c>
       <c r="D30" t="n" s="91">
-        <v>0.614323</v>
+        <v>0.624754</v>
       </c>
       <c r="E30" t="n" s="92">
-        <v>1.124824372E7</v>
+        <v>1.150390972E7</v>
       </c>
       <c r="F30" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G30" t="n" s="93">
-        <v>2.30973801E7</v>
+        <v>2.31043884E7</v>
       </c>
     </row>
     <row r="31">
@@ -2054,16 +2054,16 @@
         <v>75</v>
       </c>
       <c r="D31" t="n" s="94">
-        <v>0.57715</v>
+        <v>0.584341</v>
       </c>
       <c r="E31" t="n" s="95">
-        <v>1.056759716E7</v>
+        <v>1.075977734E7</v>
       </c>
       <c r="F31" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G31" t="n" s="96">
-        <v>1.5877134E7</v>
+        <v>1.5882048E7</v>
       </c>
     </row>
     <row r="32">
@@ -2077,16 +2077,16 @@
         <v>77</v>
       </c>
       <c r="D32" t="n" s="97">
-        <v>0.565042</v>
+        <v>0.572493</v>
       </c>
       <c r="E32" t="n" s="98">
-        <v>1.034589861E7</v>
+        <v>1.054161226E7</v>
       </c>
       <c r="F32" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G32" t="n" s="99">
-        <v>1.579196875E7</v>
+        <v>1.57968375E7</v>
       </c>
     </row>
     <row r="33">
@@ -2100,10 +2100,10 @@
         <v>79</v>
       </c>
       <c r="D33" t="n" s="100">
-        <v>0.266484</v>
+        <v>0.26436</v>
       </c>
       <c r="E33" t="n" s="101">
-        <v>4879312.98</v>
+        <v>4867795.68</v>
       </c>
       <c r="F33" t="s" s="18">
         <v>21</v>
@@ -2123,10 +2123,10 @@
         <v>21</v>
       </c>
       <c r="D34" t="n" s="103">
-        <v>0.199538</v>
+        <v>0.195958</v>
       </c>
       <c r="E34" t="n" s="104">
-        <v>3653531.14</v>
+        <v>3608272.55</v>
       </c>
       <c r="F34" t="n" s="105">
         <v>4.1426456199E8</v>
@@ -2146,10 +2146,10 @@
         <v>82</v>
       </c>
       <c r="D35" t="n" s="107">
-        <v>0.148631</v>
+        <v>0.14758</v>
       </c>
       <c r="E35" t="n" s="108">
-        <v>2721429.18</v>
+        <v>2717464.79</v>
       </c>
       <c r="F35" t="s" s="18">
         <v>21</v>
@@ -2169,13 +2169,13 @@
         <v>85</v>
       </c>
       <c r="D36" t="n" s="110">
-        <v>0.076665</v>
+        <v>0.097236</v>
       </c>
       <c r="E36" t="n" s="111">
-        <v>1.7268858458E8</v>
+        <v>1.7268536641E8</v>
       </c>
       <c r="F36" t="n" s="112">
-        <v>1.7268858458E8</v>
+        <v>1.7268536641E8</v>
       </c>
       <c r="G36" t="n" s="113">
         <v>2.331E8</v>
@@ -2192,16 +2192,16 @@
         <v>88</v>
       </c>
       <c r="D37" t="n" s="114">
-        <v>0.044932</v>
+        <v>0.077755</v>
       </c>
       <c r="E37" t="n" s="115">
-        <v>6.856045513E7</v>
+        <v>3.3855384209E8</v>
       </c>
       <c r="F37" t="n" s="116">
-        <v>6.856045513E7</v>
+        <v>3.3855384209E8</v>
       </c>
       <c r="G37" t="n" s="117">
-        <v>11025.0</v>
+        <v>2.474E8</v>
       </c>
     </row>
     <row r="38">
@@ -2215,16 +2215,16 @@
         <v>91</v>
       </c>
       <c r="D38" t="n" s="118">
-        <v>0.029882</v>
+        <v>0.026946</v>
       </c>
       <c r="E38" t="n" s="119">
-        <v>8.662445843E7</v>
+        <v>6.807970044E7</v>
       </c>
       <c r="F38" t="n" s="120">
-        <v>8.662445843E7</v>
+        <v>6.807970044E7</v>
       </c>
       <c r="G38" t="n" s="121">
-        <v>3380000.0</v>
+        <v>11025.0</v>
       </c>
     </row>
     <row r="39">
@@ -2232,68 +2232,68 @@
         <v>92</v>
       </c>
       <c r="B39" t="s" s="18">
+        <v>21</v>
+      </c>
+      <c r="C39" t="s" s="18">
         <v>93</v>
       </c>
-      <c r="C39" t="s" s="18">
-        <v>94</v>
-      </c>
       <c r="D39" t="n" s="122">
-        <v>0.00358</v>
+        <v>0.0</v>
       </c>
       <c r="E39" t="n" s="123">
-        <v>7.305620877E7</v>
-      </c>
-      <c r="F39" t="n" s="124">
-        <v>7.305620877E7</v>
-      </c>
-      <c r="G39" t="n" s="125">
-        <v>5060.0</v>
+        <v>7.54</v>
+      </c>
+      <c r="F39" t="s" s="18">
+        <v>21</v>
+      </c>
+      <c r="G39" t="n" s="124">
+        <v>10.58</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s" s="18">
+        <v>94</v>
+      </c>
+      <c r="B40" t="s" s="18">
+        <v>21</v>
+      </c>
+      <c r="C40" t="s" s="18">
         <v>95</v>
       </c>
-      <c r="B40" t="s" s="18">
-        <v>21</v>
-      </c>
-      <c r="C40" t="s" s="18">
-        <v>96</v>
-      </c>
-      <c r="D40" t="n" s="126">
-        <v>0.0</v>
-      </c>
-      <c r="E40" t="n" s="127">
-        <v>7.52</v>
+      <c r="D40" t="n" s="125">
+        <v>-0.006777</v>
+      </c>
+      <c r="E40" t="n" s="126">
+        <v>-124788.06</v>
       </c>
       <c r="F40" t="s" s="18">
         <v>21</v>
       </c>
-      <c r="G40" t="n" s="128">
-        <v>10.58</v>
+      <c r="G40" t="n" s="127">
+        <v>-177976.22</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s" s="18">
+        <v>96</v>
+      </c>
+      <c r="B41" t="s" s="18">
         <v>97</v>
-      </c>
-      <c r="B41" t="s" s="18">
-        <v>21</v>
       </c>
       <c r="C41" t="s" s="18">
         <v>98</v>
       </c>
-      <c r="D41" t="n" s="129">
-        <v>-0.006831</v>
-      </c>
-      <c r="E41" t="n" s="130">
-        <v>-125072.8</v>
-      </c>
-      <c r="F41" t="s" s="18">
-        <v>21</v>
+      <c r="D41" t="n" s="128">
+        <v>-0.00728</v>
+      </c>
+      <c r="E41" t="n" s="129">
+        <v>7.275029368E7</v>
+      </c>
+      <c r="F41" t="n" s="130">
+        <v>7.275029368E7</v>
       </c>
       <c r="G41" t="n" s="131">
-        <v>-177976.22</v>
+        <v>5060.0</v>
       </c>
     </row>
     <row r="42">
@@ -2307,16 +2307,16 @@
         <v>100</v>
       </c>
       <c r="D42" t="n" s="132">
-        <v>-0.007744</v>
+        <v>-0.007745</v>
       </c>
       <c r="E42" t="n" s="133">
-        <v>-141793.78</v>
+        <v>-142611.75</v>
       </c>
       <c r="F42" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G42" t="n" s="134">
-        <v>-2.2418306E7</v>
+        <v>-2.2420706E7</v>
       </c>
     </row>
     <row r="43">
@@ -2330,16 +2330,16 @@
         <v>103</v>
       </c>
       <c r="D43" t="n" s="135">
-        <v>-0.042945</v>
+        <v>-0.014945</v>
       </c>
       <c r="E43" t="n" s="136">
-        <v>3.3713341295E8</v>
+        <v>8.730827211E7</v>
       </c>
       <c r="F43" t="n" s="137">
-        <v>3.3713341295E8</v>
+        <v>8.730827211E7</v>
       </c>
       <c r="G43" t="n" s="138">
-        <v>2.474E8</v>
+        <v>3420000.0</v>
       </c>
     </row>
     <row r="44">
@@ -2353,16 +2353,16 @@
         <v>106</v>
       </c>
       <c r="D44" t="n" s="139">
-        <v>-0.068388</v>
+        <v>-0.076609</v>
       </c>
       <c r="E44" t="n" s="140">
-        <v>1.7369543453E8</v>
+        <v>1.2007264942E8</v>
       </c>
       <c r="F44" t="n" s="141">
-        <v>1.7369543453E8</v>
+        <v>1.2007264942E8</v>
       </c>
       <c r="G44" t="n" s="142">
-        <v>24880.0</v>
+        <v>1.056E8</v>
       </c>
     </row>
     <row r="45">
@@ -2376,16 +2376,16 @@
         <v>109</v>
       </c>
       <c r="D45" t="n" s="143">
-        <v>-0.120381</v>
+        <v>-0.121316</v>
       </c>
       <c r="E45" t="n" s="144">
-        <v>1.1945634207E8</v>
+        <v>2.1259075E8</v>
       </c>
       <c r="F45" t="n" s="145">
-        <v>1.1945634207E8</v>
+        <v>2.1259075E8</v>
       </c>
       <c r="G45" t="n" s="146">
-        <v>1.056E8</v>
+        <v>1.973E8</v>
       </c>
     </row>
     <row r="46">
@@ -2399,16 +2399,16 @@
         <v>112</v>
       </c>
       <c r="D46" t="n" s="147">
-        <v>-0.361084</v>
+        <v>-0.243349</v>
       </c>
       <c r="E46" t="n" s="148">
-        <v>2.0821315625E8</v>
+        <v>1.7005374803E8</v>
       </c>
       <c r="F46" t="n" s="149">
-        <v>2.0821315625E8</v>
+        <v>1.7005374803E8</v>
       </c>
       <c r="G46" t="n" s="150">
-        <v>1.973E8</v>
+        <v>24880.0</v>
       </c>
     </row>
     <row r="47">
@@ -2422,16 +2422,16 @@
         <v>115</v>
       </c>
       <c r="D47" t="n" s="151">
-        <v>-0.478616</v>
+        <v>-0.366428</v>
       </c>
       <c r="E47" t="n" s="152">
-        <v>1.76375E8</v>
+        <v>4.4765109375E8</v>
       </c>
       <c r="F47" t="n" s="153">
-        <v>1.76375E8</v>
+        <v>4.4765109375E8</v>
       </c>
       <c r="G47" t="n" s="154">
-        <v>42500.0</v>
+        <v>4.207E8</v>
       </c>
     </row>
     <row r="48">
@@ -2445,16 +2445,16 @@
         <v>118</v>
       </c>
       <c r="D48" t="n" s="155">
-        <v>-0.666477</v>
+        <v>-0.68273</v>
       </c>
       <c r="E48" t="n" s="156">
-        <v>4.4219514063E8</v>
+        <v>1.745972E8</v>
       </c>
       <c r="F48" t="n" s="157">
-        <v>4.4219514063E8</v>
+        <v>1.745972E8</v>
       </c>
       <c r="G48" t="n" s="158">
-        <v>4.207E8</v>
+        <v>43000.0</v>
       </c>
     </row>
     <row r="49"/>

</xml_diff>

<commit_message>
Update ALLW XLSX 2026-10-26
</commit_message>
<xml_diff>
--- a/latest/allw-latest.xlsx
+++ b/latest/allw-latest.xlsx
@@ -192,7 +192,7 @@
     <t>ALLW</t>
   </si>
   <si>
-    <t>As of 22-Oct-2026</t>
+    <t>As of 23-Oct-2026</t>
   </si>
   <si>
     <t>Name</t>
@@ -240,39 +240,39 @@
     <t>912797TV9</t>
   </si>
   <si>
+    <t>STATE STREET SPDR PORTFOLIO EM</t>
+  </si>
+  <si>
+    <t>SPEM</t>
+  </si>
+  <si>
+    <t>78463X509</t>
+  </si>
+  <si>
     <t>TSY INFL IX N/B 07/35 1.875</t>
   </si>
   <si>
     <t>91282CNS6</t>
   </si>
   <si>
+    <t>TSY INFL IX N/B 01/36 1.875</t>
+  </si>
+  <si>
+    <t>91282CPU9</t>
+  </si>
+  <si>
+    <t>TSY INFL IX N/B 01/35 2.125</t>
+  </si>
+  <si>
+    <t>91282CML2</t>
+  </si>
+  <si>
     <t>US DOLLAR</t>
   </si>
   <si>
     <t>999USDZ92</t>
   </si>
   <si>
-    <t>TSY INFL IX N/B 01/36 1.875</t>
-  </si>
-  <si>
-    <t>91282CPU9</t>
-  </si>
-  <si>
-    <t>STATE STREET SPDR PORTFOLIO EM</t>
-  </si>
-  <si>
-    <t>SPEM</t>
-  </si>
-  <si>
-    <t>78463X509</t>
-  </si>
-  <si>
-    <t>TSY INFL IX N/B 01/35 2.125</t>
-  </si>
-  <si>
-    <t>91282CML2</t>
-  </si>
-  <si>
     <t>TSY INFL IX N/B 07/34 1.875</t>
   </si>
   <si>
@@ -354,18 +354,18 @@
     <t>912810RW0</t>
   </si>
   <si>
+    <t>TSY INFL IX N/B 02/46 1</t>
+  </si>
+  <si>
+    <t>912810RR1</t>
+  </si>
+  <si>
     <t>TSY INFL IX N/B 02/52 0.125</t>
   </si>
   <si>
     <t>912810TE8</t>
   </si>
   <si>
-    <t>TSY INFL IX N/B 02/46 1</t>
-  </si>
-  <si>
-    <t>912810RR1</t>
-  </si>
-  <si>
     <t>TSY INFL IX N/B 02/50 0.25</t>
   </si>
   <si>
@@ -390,13 +390,22 @@
     <t>912810SG4</t>
   </si>
   <si>
+    <t>TRS USD BCOMTR</t>
+  </si>
+  <si>
     <t>EURO CURRENCY</t>
   </si>
   <si>
     <t>999EURZ94</t>
   </si>
   <si>
-    <t>TRS USD BCOMTR</t>
+    <t>AUST 10Y BOND FUT DEC26</t>
+  </si>
+  <si>
+    <t>XMZ6</t>
+  </si>
+  <si>
+    <t>ADI3BDHZ1</t>
   </si>
   <si>
     <t>POUND STERLING</t>
@@ -405,15 +414,6 @@
     <t>999GBPZ94</t>
   </si>
   <si>
-    <t>AUST 10Y BOND FUT DEC26</t>
-  </si>
-  <si>
-    <t>XMZ6</t>
-  </si>
-  <si>
-    <t>ADI3BDHZ1</t>
-  </si>
-  <si>
     <t>EURO-BUND FUTURE  DEC26</t>
   </si>
   <si>
@@ -444,6 +444,12 @@
     <t>999AUDZ93</t>
   </si>
   <si>
+    <t>JAPANESE YEN</t>
+  </si>
+  <si>
+    <t>999JPYZ94</t>
+  </si>
+  <si>
     <t>FTSE 100 IDX FUT  DEC26</t>
   </si>
   <si>
@@ -451,12 +457,6 @@
   </si>
   <si>
     <t>ADI38QPG9</t>
-  </si>
-  <si>
-    <t>JAPANESE YEN</t>
-  </si>
-  <si>
-    <t>999JPYZ94</t>
   </si>
   <si>
     <t>TOPIX INDX FUTR   DEC26</t>
@@ -918,97 +918,97 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
@@ -1479,16 +1479,16 @@
         <v>22</v>
       </c>
       <c r="D6" t="n" s="19">
-        <v>34.098448</v>
+        <v>34.443316</v>
       </c>
       <c r="E6" t="n" s="20">
-        <v>6.2787208547E8</v>
+        <v>6.3221996043E8</v>
       </c>
       <c r="F6" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G6" t="n" s="21">
-        <v>6.2787208547E8</v>
+        <v>6.3221996043E8</v>
       </c>
     </row>
     <row r="7">
@@ -1502,10 +1502,10 @@
         <v>25</v>
       </c>
       <c r="D7" t="n" s="22">
-        <v>13.332392</v>
+        <v>13.303232</v>
       </c>
       <c r="E7" t="n" s="23">
-        <v>2.4549612994E8</v>
+        <v>2.441857981E8</v>
       </c>
       <c r="F7" t="s" s="18">
         <v>21</v>
@@ -1525,10 +1525,10 @@
         <v>27</v>
       </c>
       <c r="D8" t="n" s="25">
-        <v>4.91362</v>
+        <v>4.930857</v>
       </c>
       <c r="E8" t="n" s="26">
-        <v>9.047699527E7</v>
+        <v>9.05077276E7</v>
       </c>
       <c r="F8" t="s" s="18">
         <v>21</v>
@@ -1542,91 +1542,91 @@
         <v>28</v>
       </c>
       <c r="B9" t="s" s="18">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="C9" t="s" s="18">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D9" t="n" s="28">
-        <v>4.298224</v>
+        <v>4.310243</v>
       </c>
       <c r="E9" t="n" s="29">
-        <v>7.9145395E7</v>
+        <v>7.911611445E7</v>
       </c>
       <c r="F9" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G9" t="n" s="30">
-        <v>8.3711947E7</v>
+        <v>1592835.0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="18">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B10" t="s" s="18">
         <v>21</v>
       </c>
       <c r="C10" t="s" s="18">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D10" t="n" s="31">
-        <v>4.236269</v>
+        <v>4.307619</v>
       </c>
       <c r="E10" t="n" s="32">
-        <v>7.800457963E7</v>
+        <v>7.906795843E7</v>
       </c>
       <c r="F10" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G10" t="n" s="33">
-        <v>7.800457963E7</v>
+        <v>8.3719977E7</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="18">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B11" t="s" s="18">
         <v>21</v>
       </c>
       <c r="C11" t="s" s="18">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D11" t="n" s="34">
-        <v>4.208441</v>
+        <v>4.216113</v>
       </c>
       <c r="E11" t="n" s="35">
-        <v>7.749215993E7</v>
+        <v>7.738832706E7</v>
       </c>
       <c r="F11" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G11" t="n" s="36">
-        <v>8.2620436E7</v>
+        <v>8.2628456E7</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s" s="18">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B12" t="s" s="18">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="C12" t="s" s="18">
         <v>36</v>
       </c>
       <c r="D12" t="n" s="37">
-        <v>4.07965</v>
+        <v>4.02457</v>
       </c>
       <c r="E12" t="n" s="38">
-        <v>7.5120682E7</v>
+        <v>7.387247974E7</v>
       </c>
       <c r="F12" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G12" t="n" s="39">
-        <v>1512700.0</v>
+        <v>7.648368E7</v>
       </c>
     </row>
     <row r="13">
@@ -1640,16 +1640,16 @@
         <v>38</v>
       </c>
       <c r="D13" t="n" s="40">
-        <v>4.016152</v>
+        <v>3.72198</v>
       </c>
       <c r="E13" t="n" s="41">
-        <v>7.395145201E7</v>
+        <v>6.831833076E7</v>
       </c>
       <c r="F13" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G13" t="n" s="42">
-        <v>7.6475749E7</v>
+        <v>6.831833076E7</v>
       </c>
     </row>
     <row r="14">
@@ -1663,16 +1663,16 @@
         <v>40</v>
       </c>
       <c r="D14" t="n" s="43">
-        <v>3.702971</v>
+        <v>3.711062</v>
       </c>
       <c r="E14" t="n" s="44">
-        <v>6.818469674E7</v>
+        <v>6.811792584E7</v>
       </c>
       <c r="F14" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G14" t="n" s="45">
-        <v>7.128824175E7</v>
+        <v>7.12955925E7</v>
       </c>
     </row>
     <row r="15">
@@ -1686,16 +1686,16 @@
         <v>42</v>
       </c>
       <c r="D15" t="n" s="46">
-        <v>3.525603</v>
+        <v>3.532618</v>
       </c>
       <c r="E15" t="n" s="47">
-        <v>6.491872744E7</v>
+        <v>6.484252311E7</v>
       </c>
       <c r="F15" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G15" t="n" s="48">
-        <v>6.833831235E7</v>
+        <v>6.83452154E7</v>
       </c>
     </row>
     <row r="16">
@@ -1709,16 +1709,16 @@
         <v>45</v>
       </c>
       <c r="D16" t="n" s="49">
-        <v>3.187357</v>
+        <v>3.274203</v>
       </c>
       <c r="E16" t="n" s="50">
-        <v>5.869042822E7</v>
+        <v>6.009921687E7</v>
       </c>
       <c r="F16" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G16" t="n" s="51">
-        <v>723323.0</v>
+        <v>740047.0</v>
       </c>
     </row>
     <row r="17">
@@ -1732,16 +1732,16 @@
         <v>47</v>
       </c>
       <c r="D17" t="n" s="52">
-        <v>2.545406</v>
+        <v>2.549746</v>
       </c>
       <c r="E17" t="n" s="53">
-        <v>4.686986361E7</v>
+        <v>4.680154386E7</v>
       </c>
       <c r="F17" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G17" t="n" s="54">
-        <v>4.7910418E7</v>
+        <v>4.7915198E7</v>
       </c>
     </row>
     <row r="18">
@@ -1755,16 +1755,16 @@
         <v>49</v>
       </c>
       <c r="D18" t="n" s="55">
-        <v>1.50963</v>
+        <v>1.507705</v>
       </c>
       <c r="E18" t="n" s="56">
-        <v>2.779758093E7</v>
+        <v>2.767449769E7</v>
       </c>
       <c r="F18" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G18" t="n" s="57">
-        <v>3.56343549E7</v>
+        <v>3.56380764E7</v>
       </c>
     </row>
     <row r="19">
@@ -1778,16 +1778,16 @@
         <v>51</v>
       </c>
       <c r="D19" t="n" s="58">
-        <v>1.340319</v>
+        <v>1.337521</v>
       </c>
       <c r="E19" t="n" s="59">
-        <v>2.467997972E7</v>
+        <v>2.455070504E7</v>
       </c>
       <c r="F19" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G19" t="n" s="60">
-        <v>3.629825785E7</v>
+        <v>3.63020881E7</v>
       </c>
     </row>
     <row r="20">
@@ -1801,16 +1801,16 @@
         <v>53</v>
       </c>
       <c r="D20" t="n" s="61">
-        <v>1.266187</v>
+        <v>1.261865</v>
       </c>
       <c r="E20" t="n" s="62">
-        <v>2.33149433E7</v>
+        <v>2.316199931E7</v>
       </c>
       <c r="F20" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G20" t="n" s="63">
-        <v>2.68705706E7</v>
+        <v>2.68733569E7</v>
       </c>
     </row>
     <row r="21">
@@ -1824,16 +1824,16 @@
         <v>55</v>
       </c>
       <c r="D21" t="n" s="64">
-        <v>1.191533</v>
+        <v>1.187461</v>
       </c>
       <c r="E21" t="n" s="65">
-        <v>2.194030341E7</v>
+        <v>2.179629172E7</v>
       </c>
       <c r="F21" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G21" t="n" s="66">
-        <v>2.66403475E7</v>
+        <v>2.664303425E7</v>
       </c>
     </row>
     <row r="22">
@@ -1847,16 +1847,16 @@
         <v>57</v>
       </c>
       <c r="D22" t="n" s="67">
-        <v>1.168226</v>
+        <v>1.164099</v>
       </c>
       <c r="E22" t="n" s="68">
-        <v>2.151113167E7</v>
+        <v>2.136746862E7</v>
       </c>
       <c r="F22" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G22" t="n" s="69">
-        <v>2.478888E7</v>
+        <v>2.479128E7</v>
       </c>
     </row>
     <row r="23">
@@ -1870,16 +1870,16 @@
         <v>59</v>
       </c>
       <c r="D23" t="n" s="70">
-        <v>1.121082</v>
+        <v>1.120115</v>
       </c>
       <c r="E23" t="n" s="71">
-        <v>2.064305597E7</v>
+        <v>2.056012091E7</v>
       </c>
       <c r="F23" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G23" t="n" s="72">
-        <v>2.82653028E7</v>
+        <v>2.82681648E7</v>
       </c>
     </row>
     <row r="24">
@@ -1893,16 +1893,16 @@
         <v>61</v>
       </c>
       <c r="D24" t="n" s="73">
-        <v>0.977111</v>
+        <v>0.97322</v>
       </c>
       <c r="E24" t="n" s="74">
-        <v>1.799204633E7</v>
+        <v>1.786381562E7</v>
       </c>
       <c r="F24" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G24" t="n" s="75">
-        <v>2.5112253E7</v>
+        <v>2.5114706E7</v>
       </c>
     </row>
     <row r="25">
@@ -1916,16 +1916,16 @@
         <v>63</v>
       </c>
       <c r="D25" t="n" s="76">
-        <v>0.94808</v>
+        <v>0.946913</v>
       </c>
       <c r="E25" t="n" s="77">
-        <v>1.745748559E7</v>
+        <v>1.738094437E7</v>
       </c>
       <c r="F25" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G25" t="n" s="78">
-        <v>2.50279524E7</v>
+        <v>2.5030359E7</v>
       </c>
     </row>
     <row r="26">
@@ -1939,16 +1939,16 @@
         <v>65</v>
       </c>
       <c r="D26" t="n" s="79">
-        <v>0.90658</v>
+        <v>0.904351</v>
       </c>
       <c r="E26" t="n" s="80">
-        <v>1.66933111E7</v>
+        <v>1.659969937E7</v>
       </c>
       <c r="F26" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G26" t="n" s="81">
-        <v>2.48914445E7</v>
+        <v>2.48939575E7</v>
       </c>
     </row>
     <row r="27">
@@ -1962,16 +1962,16 @@
         <v>67</v>
       </c>
       <c r="D27" t="n" s="82">
-        <v>0.749249</v>
+        <v>0.746081</v>
       </c>
       <c r="E27" t="n" s="83">
-        <v>1.379630192E7</v>
+        <v>1.369460206E7</v>
       </c>
       <c r="F27" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G27" t="n" s="84">
-        <v>2.8498776E7</v>
+        <v>1.96107744E7</v>
       </c>
     </row>
     <row r="28">
@@ -1985,16 +1985,16 @@
         <v>69</v>
       </c>
       <c r="D28" t="n" s="85">
-        <v>0.747604</v>
+        <v>0.745571</v>
       </c>
       <c r="E28" t="n" s="86">
-        <v>1.376601228E7</v>
+        <v>1.368523098E7</v>
       </c>
       <c r="F28" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G28" t="n" s="87">
-        <v>1.96088312E7</v>
+        <v>2.850162E7</v>
       </c>
     </row>
     <row r="29">
@@ -2008,16 +2008,16 @@
         <v>71</v>
       </c>
       <c r="D29" t="n" s="88">
-        <v>0.737666</v>
+        <v>0.734559</v>
       </c>
       <c r="E29" t="n" s="89">
-        <v>1.358301757E7</v>
+        <v>1.348310591E7</v>
       </c>
       <c r="F29" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G29" t="n" s="90">
-        <v>2.553892615E7</v>
+        <v>2.55414761E7</v>
       </c>
     </row>
     <row r="30">
@@ -2031,16 +2031,16 @@
         <v>73</v>
       </c>
       <c r="D30" t="n" s="91">
-        <v>0.624754</v>
+        <v>0.622252</v>
       </c>
       <c r="E30" t="n" s="92">
-        <v>1.150390972E7</v>
+        <v>1.142167065E7</v>
       </c>
       <c r="F30" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G30" t="n" s="93">
-        <v>2.31043884E7</v>
+        <v>2.31069042E7</v>
       </c>
     </row>
     <row r="31">
@@ -2054,16 +2054,16 @@
         <v>75</v>
       </c>
       <c r="D31" t="n" s="94">
-        <v>0.584341</v>
+        <v>0.582839</v>
       </c>
       <c r="E31" t="n" s="95">
-        <v>1.075977734E7</v>
+        <v>1.069822099E7</v>
       </c>
       <c r="F31" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G31" t="n" s="96">
-        <v>1.5882048E7</v>
+        <v>1.5883686E7</v>
       </c>
     </row>
     <row r="32">
@@ -2077,16 +2077,16 @@
         <v>77</v>
       </c>
       <c r="D32" t="n" s="97">
-        <v>0.572493</v>
+        <v>0.570866</v>
       </c>
       <c r="E32" t="n" s="98">
-        <v>1.054161226E7</v>
+        <v>1.047846152E7</v>
       </c>
       <c r="F32" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G32" t="n" s="99">
-        <v>1.57968375E7</v>
+        <v>1.579838125E7</v>
       </c>
     </row>
     <row r="33">
@@ -2097,42 +2097,42 @@
         <v>21</v>
       </c>
       <c r="C33" t="s" s="18">
-        <v>79</v>
+        <v>21</v>
       </c>
       <c r="D33" t="n" s="100">
-        <v>0.26436</v>
+        <v>0.360298</v>
       </c>
       <c r="E33" t="n" s="101">
-        <v>4867795.68</v>
-      </c>
-      <c r="F33" t="s" s="18">
-        <v>21</v>
-      </c>
-      <c r="G33" t="n" s="102">
-        <v>4347214.14</v>
+        <v>6613398.11</v>
+      </c>
+      <c r="F33" t="n" s="102">
+        <v>4.1779656199E8</v>
+      </c>
+      <c r="G33" t="n" s="103">
+        <v>1138114.82</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s" s="18">
+        <v>79</v>
+      </c>
+      <c r="B34" t="s" s="18">
+        <v>21</v>
+      </c>
+      <c r="C34" t="s" s="18">
         <v>80</v>
       </c>
-      <c r="B34" t="s" s="18">
-        <v>21</v>
-      </c>
-      <c r="C34" t="s" s="18">
-        <v>21</v>
-      </c>
-      <c r="D34" t="n" s="103">
-        <v>0.195958</v>
-      </c>
-      <c r="E34" t="n" s="104">
-        <v>3608272.55</v>
-      </c>
-      <c r="F34" t="n" s="105">
-        <v>4.1426456199E8</v>
+      <c r="D34" t="n" s="104">
+        <v>0.265348</v>
+      </c>
+      <c r="E34" t="n" s="105">
+        <v>4870563.31</v>
+      </c>
+      <c r="F34" t="s" s="18">
+        <v>21</v>
       </c>
       <c r="G34" t="n" s="106">
-        <v>1128643.27</v>
+        <v>4347162.84</v>
       </c>
     </row>
     <row r="35">
@@ -2140,45 +2140,45 @@
         <v>81</v>
       </c>
       <c r="B35" t="s" s="18">
-        <v>21</v>
+        <v>82</v>
       </c>
       <c r="C35" t="s" s="18">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D35" t="n" s="107">
-        <v>0.14758</v>
+        <v>0.16208</v>
       </c>
       <c r="E35" t="n" s="108">
-        <v>2717464.79</v>
-      </c>
-      <c r="F35" t="s" s="18">
-        <v>21</v>
-      </c>
-      <c r="G35" t="n" s="109">
-        <v>2033345.75</v>
+        <v>1.7434516348E8</v>
+      </c>
+      <c r="F35" t="n" s="109">
+        <v>1.7434516348E8</v>
+      </c>
+      <c r="G35" t="n" s="110">
+        <v>2.331E8</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s" s="18">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B36" t="s" s="18">
-        <v>84</v>
+        <v>21</v>
       </c>
       <c r="C36" t="s" s="18">
         <v>85</v>
       </c>
-      <c r="D36" t="n" s="110">
-        <v>0.097236</v>
-      </c>
-      <c r="E36" t="n" s="111">
-        <v>1.7268536641E8</v>
-      </c>
-      <c r="F36" t="n" s="112">
-        <v>1.7268536641E8</v>
+      <c r="D36" t="n" s="111">
+        <v>0.14828</v>
+      </c>
+      <c r="E36" t="n" s="112">
+        <v>2721735.18</v>
+      </c>
+      <c r="F36" t="s" s="18">
+        <v>21</v>
       </c>
       <c r="G36" t="n" s="113">
-        <v>2.331E8</v>
+        <v>2033345.75</v>
       </c>
     </row>
     <row r="37">
@@ -2192,13 +2192,13 @@
         <v>88</v>
       </c>
       <c r="D37" t="n" s="114">
-        <v>0.077755</v>
+        <v>0.072006</v>
       </c>
       <c r="E37" t="n" s="115">
-        <v>3.3855384209E8</v>
+        <v>3.3863945289E8</v>
       </c>
       <c r="F37" t="n" s="116">
-        <v>3.3855384209E8</v>
+        <v>3.3863945289E8</v>
       </c>
       <c r="G37" t="n" s="117">
         <v>2.474E8</v>
@@ -2215,13 +2215,13 @@
         <v>91</v>
       </c>
       <c r="D38" t="n" s="118">
-        <v>0.026946</v>
+        <v>0.03133</v>
       </c>
       <c r="E38" t="n" s="119">
-        <v>6.807970044E7</v>
+        <v>6.834653052E7</v>
       </c>
       <c r="F38" t="n" s="120">
-        <v>6.807970044E7</v>
+        <v>6.834653052E7</v>
       </c>
       <c r="G38" t="n" s="121">
         <v>11025.0</v>
@@ -2241,7 +2241,7 @@
         <v>0.0</v>
       </c>
       <c r="E39" t="n" s="123">
-        <v>7.54</v>
+        <v>7.57</v>
       </c>
       <c r="F39" t="s" s="18">
         <v>21</v>
@@ -2261,10 +2261,10 @@
         <v>95</v>
       </c>
       <c r="D40" t="n" s="125">
-        <v>-0.006777</v>
+        <v>-0.006817</v>
       </c>
       <c r="E40" t="n" s="126">
-        <v>-124788.06</v>
+        <v>-125135.06</v>
       </c>
       <c r="F40" t="s" s="18">
         <v>21</v>
@@ -2278,45 +2278,45 @@
         <v>96</v>
       </c>
       <c r="B41" t="s" s="18">
+        <v>21</v>
+      </c>
+      <c r="C41" t="s" s="18">
         <v>97</v>
       </c>
-      <c r="C41" t="s" s="18">
-        <v>98</v>
-      </c>
       <c r="D41" t="n" s="128">
-        <v>-0.00728</v>
+        <v>-0.007792</v>
       </c>
       <c r="E41" t="n" s="129">
-        <v>7.275029368E7</v>
-      </c>
-      <c r="F41" t="n" s="130">
-        <v>7.275029368E7</v>
-      </c>
-      <c r="G41" t="n" s="131">
-        <v>5060.0</v>
+        <v>-143025.63</v>
+      </c>
+      <c r="F41" t="s" s="18">
+        <v>21</v>
+      </c>
+      <c r="G41" t="n" s="130">
+        <v>-2.2420698E7</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s" s="18">
+        <v>98</v>
+      </c>
+      <c r="B42" t="s" s="18">
         <v>99</v>
-      </c>
-      <c r="B42" t="s" s="18">
-        <v>21</v>
       </c>
       <c r="C42" t="s" s="18">
         <v>100</v>
       </c>
-      <c r="D42" t="n" s="132">
-        <v>-0.007745</v>
-      </c>
-      <c r="E42" t="n" s="133">
-        <v>-142611.75</v>
-      </c>
-      <c r="F42" t="s" s="18">
-        <v>21</v>
+      <c r="D42" t="n" s="131">
+        <v>-0.028347</v>
+      </c>
+      <c r="E42" t="n" s="132">
+        <v>7.247855308E7</v>
+      </c>
+      <c r="F42" t="n" s="133">
+        <v>7.247855308E7</v>
       </c>
       <c r="G42" t="n" s="134">
-        <v>-2.2420706E7</v>
+        <v>5060.0</v>
       </c>
     </row>
     <row r="43">
@@ -2330,13 +2330,13 @@
         <v>103</v>
       </c>
       <c r="D43" t="n" s="135">
-        <v>-0.014945</v>
+        <v>-0.066739</v>
       </c>
       <c r="E43" t="n" s="136">
-        <v>8.730827211E7</v>
+        <v>8.661265629E7</v>
       </c>
       <c r="F43" t="n" s="137">
-        <v>8.730827211E7</v>
+        <v>8.661265629E7</v>
       </c>
       <c r="G43" t="n" s="138">
         <v>3420000.0</v>
@@ -2353,13 +2353,13 @@
         <v>106</v>
       </c>
       <c r="D44" t="n" s="139">
-        <v>-0.076609</v>
+        <v>-0.100075</v>
       </c>
       <c r="E44" t="n" s="140">
-        <v>1.2007264942E8</v>
+        <v>1.1983728585E8</v>
       </c>
       <c r="F44" t="n" s="141">
-        <v>1.2007264942E8</v>
+        <v>1.1983728585E8</v>
       </c>
       <c r="G44" t="n" s="142">
         <v>1.056E8</v>
@@ -2376,13 +2376,13 @@
         <v>109</v>
       </c>
       <c r="D45" t="n" s="143">
-        <v>-0.121316</v>
+        <v>-0.175445</v>
       </c>
       <c r="E45" t="n" s="144">
-        <v>2.1259075E8</v>
+        <v>2.1160425E8</v>
       </c>
       <c r="F45" t="n" s="145">
-        <v>2.1259075E8</v>
+        <v>2.1160425E8</v>
       </c>
       <c r="G45" t="n" s="146">
         <v>1.973E8</v>
@@ -2399,16 +2399,16 @@
         <v>112</v>
       </c>
       <c r="D46" t="n" s="147">
-        <v>-0.243349</v>
+        <v>-0.291363</v>
       </c>
       <c r="E46" t="n" s="148">
-        <v>1.7005374803E8</v>
+        <v>1.718738922E8</v>
       </c>
       <c r="F46" t="n" s="149">
-        <v>1.7005374803E8</v>
+        <v>1.718738922E8</v>
       </c>
       <c r="G46" t="n" s="150">
-        <v>24880.0</v>
+        <v>25260.0</v>
       </c>
     </row>
     <row r="47">
@@ -2422,13 +2422,13 @@
         <v>115</v>
       </c>
       <c r="D47" t="n" s="151">
-        <v>-0.366428</v>
+        <v>-0.424888</v>
       </c>
       <c r="E47" t="n" s="152">
-        <v>4.4765109375E8</v>
+        <v>4.4659934375E8</v>
       </c>
       <c r="F47" t="n" s="153">
-        <v>4.4765109375E8</v>
+        <v>4.4659934375E8</v>
       </c>
       <c r="G47" t="n" s="154">
         <v>4.207E8</v>
@@ -2445,16 +2445,16 @@
         <v>118</v>
       </c>
       <c r="D48" t="n" s="155">
-        <v>-0.68273</v>
+        <v>-0.807884</v>
       </c>
       <c r="E48" t="n" s="156">
-        <v>1.745972E8</v>
+        <v>1.7674839E8</v>
       </c>
       <c r="F48" t="n" s="157">
-        <v>1.745972E8</v>
+        <v>1.7674839E8</v>
       </c>
       <c r="G48" t="n" s="158">
-        <v>43000.0</v>
+        <v>44100.0</v>
       </c>
     </row>
     <row r="49"/>

</xml_diff>

<commit_message>
Update ALLW XLSX 2026-10-27
</commit_message>
<xml_diff>
--- a/latest/allw-latest.xlsx
+++ b/latest/allw-latest.xlsx
@@ -192,7 +192,7 @@
     <t>ALLW</t>
   </si>
   <si>
-    <t>As of 23-Oct-2026</t>
+    <t>As of 26-Oct-2026</t>
   </si>
   <si>
     <t>Name</t>
@@ -240,6 +240,12 @@
     <t>912797TV9</t>
   </si>
   <si>
+    <t>TSY INFL IX N/B 07/35 1.875</t>
+  </si>
+  <si>
+    <t>91282CNS6</t>
+  </si>
+  <si>
     <t>STATE STREET SPDR PORTFOLIO EM</t>
   </si>
   <si>
@@ -249,10 +255,10 @@
     <t>78463X509</t>
   </si>
   <si>
-    <t>TSY INFL IX N/B 07/35 1.875</t>
-  </si>
-  <si>
-    <t>91282CNS6</t>
+    <t>US DOLLAR</t>
+  </si>
+  <si>
+    <t>999USDZ92</t>
   </si>
   <si>
     <t>TSY INFL IX N/B 01/36 1.875</t>
@@ -267,12 +273,6 @@
     <t>91282CML2</t>
   </si>
   <si>
-    <t>US DOLLAR</t>
-  </si>
-  <si>
-    <t>999USDZ92</t>
-  </si>
-  <si>
     <t>TSY INFL IX N/B 07/34 1.875</t>
   </si>
   <si>
@@ -354,18 +354,18 @@
     <t>912810RW0</t>
   </si>
   <si>
+    <t>TSY INFL IX N/B 02/52 0.125</t>
+  </si>
+  <si>
+    <t>912810TE8</t>
+  </si>
+  <si>
     <t>TSY INFL IX N/B 02/46 1</t>
   </si>
   <si>
     <t>912810RR1</t>
   </si>
   <si>
-    <t>TSY INFL IX N/B 02/52 0.125</t>
-  </si>
-  <si>
-    <t>912810TE8</t>
-  </si>
-  <si>
     <t>TSY INFL IX N/B 02/50 0.25</t>
   </si>
   <si>
@@ -390,15 +390,15 @@
     <t>912810SG4</t>
   </si>
   <si>
+    <t>EURO CURRENCY</t>
+  </si>
+  <si>
+    <t>999EURZ94</t>
+  </si>
+  <si>
     <t>TRS USD BCOMTR</t>
   </si>
   <si>
-    <t>EURO CURRENCY</t>
-  </si>
-  <si>
-    <t>999EURZ94</t>
-  </si>
-  <si>
     <t>AUST 10Y BOND FUT DEC26</t>
   </si>
   <si>
@@ -432,6 +432,15 @@
     <t>ADI391SG0</t>
   </si>
   <si>
+    <t>FTSE 100 IDX FUT  DEC26</t>
+  </si>
+  <si>
+    <t>Z Z6</t>
+  </si>
+  <si>
+    <t>ADI38QPG9</t>
+  </si>
+  <si>
     <t>CANADIAN DOLLAR</t>
   </si>
   <si>
@@ -448,15 +457,6 @@
   </si>
   <si>
     <t>999JPYZ94</t>
-  </si>
-  <si>
-    <t>FTSE 100 IDX FUT  DEC26</t>
-  </si>
-  <si>
-    <t>Z Z6</t>
-  </si>
-  <si>
-    <t>ADI38QPG9</t>
   </si>
   <si>
     <t>TOPIX INDX FUTR   DEC26</t>
@@ -918,97 +918,97 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
@@ -1479,16 +1479,16 @@
         <v>22</v>
       </c>
       <c r="D6" t="n" s="19">
-        <v>34.443316</v>
+        <v>33.843897</v>
       </c>
       <c r="E6" t="n" s="20">
-        <v>6.3221996043E8</v>
+        <v>6.2289851787E8</v>
       </c>
       <c r="F6" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G6" t="n" s="21">
-        <v>6.3221996043E8</v>
+        <v>6.2289851787E8</v>
       </c>
     </row>
     <row r="7">
@@ -1502,10 +1502,10 @@
         <v>25</v>
       </c>
       <c r="D7" t="n" s="22">
-        <v>13.303232</v>
+        <v>13.357804</v>
       </c>
       <c r="E7" t="n" s="23">
-        <v>2.441857981E8</v>
+        <v>2.4585101148E8</v>
       </c>
       <c r="F7" t="s" s="18">
         <v>21</v>
@@ -1525,10 +1525,10 @@
         <v>27</v>
       </c>
       <c r="D8" t="n" s="25">
-        <v>4.930857</v>
+        <v>4.917914</v>
       </c>
       <c r="E8" t="n" s="26">
-        <v>9.05077276E7</v>
+        <v>9.051443821E7</v>
       </c>
       <c r="F8" t="s" s="18">
         <v>21</v>
@@ -1542,45 +1542,45 @@
         <v>28</v>
       </c>
       <c r="B9" t="s" s="18">
+        <v>21</v>
+      </c>
+      <c r="C9" t="s" s="18">
         <v>29</v>
       </c>
-      <c r="C9" t="s" s="18">
-        <v>30</v>
-      </c>
       <c r="D9" t="n" s="28">
-        <v>4.310243</v>
+        <v>4.299201</v>
       </c>
       <c r="E9" t="n" s="29">
-        <v>7.911611445E7</v>
+        <v>7.91269959E7</v>
       </c>
       <c r="F9" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G9" t="n" s="30">
-        <v>1592835.0</v>
+        <v>8.372881E7</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="18">
+        <v>30</v>
+      </c>
+      <c r="B10" t="s" s="18">
         <v>31</v>
-      </c>
-      <c r="B10" t="s" s="18">
-        <v>21</v>
       </c>
       <c r="C10" t="s" s="18">
         <v>32</v>
       </c>
       <c r="D10" t="n" s="31">
-        <v>4.307619</v>
+        <v>4.271781</v>
       </c>
       <c r="E10" t="n" s="32">
-        <v>7.906795843E7</v>
+        <v>7.86223356E7</v>
       </c>
       <c r="F10" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G10" t="n" s="33">
-        <v>8.3719977E7</v>
+        <v>1592835.0</v>
       </c>
     </row>
     <row r="11">
@@ -1594,16 +1594,16 @@
         <v>34</v>
       </c>
       <c r="D11" t="n" s="34">
-        <v>4.216113</v>
+        <v>4.218395</v>
       </c>
       <c r="E11" t="n" s="35">
-        <v>7.738832706E7</v>
+        <v>7.763976667E7</v>
       </c>
       <c r="F11" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G11" t="n" s="36">
-        <v>8.2628456E7</v>
+        <v>7.763976667E7</v>
       </c>
     </row>
     <row r="12">
@@ -1617,16 +1617,16 @@
         <v>36</v>
       </c>
       <c r="D12" t="n" s="37">
-        <v>4.02457</v>
+        <v>4.208866</v>
       </c>
       <c r="E12" t="n" s="38">
-        <v>7.387247974E7</v>
+        <v>7.746437777E7</v>
       </c>
       <c r="F12" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G12" t="n" s="39">
-        <v>7.648368E7</v>
+        <v>8.2637278E7</v>
       </c>
     </row>
     <row r="13">
@@ -1640,16 +1640,16 @@
         <v>38</v>
       </c>
       <c r="D13" t="n" s="40">
-        <v>3.72198</v>
+        <v>4.01591</v>
       </c>
       <c r="E13" t="n" s="41">
-        <v>6.831833076E7</v>
+        <v>7.391300689E7</v>
       </c>
       <c r="F13" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G13" t="n" s="42">
-        <v>6.831833076E7</v>
+        <v>7.6491611E7</v>
       </c>
     </row>
     <row r="14">
@@ -1663,16 +1663,16 @@
         <v>40</v>
       </c>
       <c r="D14" t="n" s="43">
-        <v>3.711062</v>
+        <v>3.702411</v>
       </c>
       <c r="E14" t="n" s="44">
-        <v>6.811792584E7</v>
+        <v>6.814305278E7</v>
       </c>
       <c r="F14" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G14" t="n" s="45">
-        <v>7.12955925E7</v>
+        <v>7.130294325E7</v>
       </c>
     </row>
     <row r="15">
@@ -1686,16 +1686,16 @@
         <v>42</v>
       </c>
       <c r="D15" t="n" s="46">
-        <v>3.532618</v>
+        <v>3.524165</v>
       </c>
       <c r="E15" t="n" s="47">
-        <v>6.484252311E7</v>
+        <v>6.486242223E7</v>
       </c>
       <c r="F15" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G15" t="n" s="48">
-        <v>6.83452154E7</v>
+        <v>6.835211845E7</v>
       </c>
     </row>
     <row r="16">
@@ -1709,10 +1709,10 @@
         <v>45</v>
       </c>
       <c r="D16" t="n" s="49">
-        <v>3.274203</v>
+        <v>3.274594</v>
       </c>
       <c r="E16" t="n" s="50">
-        <v>6.009921687E7</v>
+        <v>6.026905766E7</v>
       </c>
       <c r="F16" t="s" s="18">
         <v>21</v>
@@ -1732,16 +1732,16 @@
         <v>47</v>
       </c>
       <c r="D17" t="n" s="52">
-        <v>2.549746</v>
+        <v>2.545407</v>
       </c>
       <c r="E17" t="n" s="53">
-        <v>4.680154386E7</v>
+        <v>4.684833011E7</v>
       </c>
       <c r="F17" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G17" t="n" s="54">
-        <v>4.7915198E7</v>
+        <v>4.7919978E7</v>
       </c>
     </row>
     <row r="18">
@@ -1755,16 +1755,16 @@
         <v>49</v>
       </c>
       <c r="D18" t="n" s="55">
-        <v>1.507705</v>
+        <v>1.508246</v>
       </c>
       <c r="E18" t="n" s="56">
-        <v>2.767449769E7</v>
+        <v>2.775933766E7</v>
       </c>
       <c r="F18" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G18" t="n" s="57">
-        <v>3.56380764E7</v>
+        <v>3.56415498E7</v>
       </c>
     </row>
     <row r="19">
@@ -1778,16 +1778,16 @@
         <v>51</v>
       </c>
       <c r="D19" t="n" s="58">
-        <v>1.337521</v>
+        <v>1.338589</v>
       </c>
       <c r="E19" t="n" s="59">
-        <v>2.455070504E7</v>
+        <v>2.4636796E7</v>
       </c>
       <c r="F19" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G19" t="n" s="60">
-        <v>3.63020881E7</v>
+        <v>3.6305663E7</v>
       </c>
     </row>
     <row r="20">
@@ -1801,16 +1801,16 @@
         <v>53</v>
       </c>
       <c r="D20" t="n" s="61">
-        <v>1.261865</v>
+        <v>1.265064</v>
       </c>
       <c r="E20" t="n" s="62">
-        <v>2.316199931E7</v>
+        <v>2.328355888E7</v>
       </c>
       <c r="F20" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G20" t="n" s="63">
-        <v>2.68733569E7</v>
+        <v>2.68761432E7</v>
       </c>
     </row>
     <row r="21">
@@ -1824,16 +1824,16 @@
         <v>55</v>
       </c>
       <c r="D21" t="n" s="64">
-        <v>1.187461</v>
+        <v>1.190681</v>
       </c>
       <c r="E21" t="n" s="65">
-        <v>2.179629172E7</v>
+        <v>2.191454435E7</v>
       </c>
       <c r="F21" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G21" t="n" s="66">
-        <v>2.664303425E7</v>
+        <v>2.6645721E7</v>
       </c>
     </row>
     <row r="22">
@@ -1847,16 +1847,16 @@
         <v>57</v>
       </c>
       <c r="D22" t="n" s="67">
-        <v>1.164099</v>
+        <v>1.167658</v>
       </c>
       <c r="E22" t="n" s="68">
-        <v>2.136746862E7</v>
+        <v>2.149080803E7</v>
       </c>
       <c r="F22" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G22" t="n" s="69">
-        <v>2.479128E7</v>
+        <v>2.479392E7</v>
       </c>
     </row>
     <row r="23">
@@ -1870,16 +1870,16 @@
         <v>59</v>
       </c>
       <c r="D23" t="n" s="70">
-        <v>1.120115</v>
+        <v>1.120475</v>
       </c>
       <c r="E23" t="n" s="71">
-        <v>2.056012091E7</v>
+        <v>2.062238899E7</v>
       </c>
       <c r="F23" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G23" t="n" s="72">
-        <v>2.82681648E7</v>
+        <v>2.82710268E7</v>
       </c>
     </row>
     <row r="24">
@@ -1893,16 +1893,16 @@
         <v>61</v>
       </c>
       <c r="D24" t="n" s="73">
-        <v>0.97322</v>
+        <v>0.975948</v>
       </c>
       <c r="E24" t="n" s="74">
-        <v>1.786381562E7</v>
+        <v>1.796236218E7</v>
       </c>
       <c r="F24" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G24" t="n" s="75">
-        <v>2.5114706E7</v>
+        <v>2.5117382E7</v>
       </c>
     </row>
     <row r="25">
@@ -1916,16 +1916,16 @@
         <v>63</v>
       </c>
       <c r="D25" t="n" s="76">
-        <v>0.946913</v>
+        <v>0.94735</v>
       </c>
       <c r="E25" t="n" s="77">
-        <v>1.738094437E7</v>
+        <v>1.743602774E7</v>
       </c>
       <c r="F25" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G25" t="n" s="78">
-        <v>2.5030359E7</v>
+        <v>2.50329375E7</v>
       </c>
     </row>
     <row r="26">
@@ -1939,16 +1939,16 @@
         <v>65</v>
       </c>
       <c r="D26" t="n" s="79">
-        <v>0.904351</v>
+        <v>0.905515</v>
       </c>
       <c r="E26" t="n" s="80">
-        <v>1.659969937E7</v>
+        <v>1.66660474E7</v>
       </c>
       <c r="F26" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G26" t="n" s="81">
-        <v>2.48939575E7</v>
+        <v>2.48964705E7</v>
       </c>
     </row>
     <row r="27">
@@ -1962,16 +1962,16 @@
         <v>67</v>
       </c>
       <c r="D27" t="n" s="82">
-        <v>0.746081</v>
+        <v>0.748539</v>
       </c>
       <c r="E27" t="n" s="83">
-        <v>1.369460206E7</v>
+        <v>1.377690092E7</v>
       </c>
       <c r="F27" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G27" t="n" s="84">
-        <v>1.96107744E7</v>
+        <v>2.8504701E7</v>
       </c>
     </row>
     <row r="28">
@@ -1985,16 +1985,16 @@
         <v>69</v>
       </c>
       <c r="D28" t="n" s="85">
-        <v>0.745571</v>
+        <v>0.746957</v>
       </c>
       <c r="E28" t="n" s="86">
-        <v>1.368523098E7</v>
+        <v>1.374776957E7</v>
       </c>
       <c r="F28" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G28" t="n" s="87">
-        <v>2.850162E7</v>
+        <v>1.96128564E7</v>
       </c>
     </row>
     <row r="29">
@@ -2008,16 +2008,16 @@
         <v>71</v>
       </c>
       <c r="D29" t="n" s="88">
-        <v>0.734559</v>
+        <v>0.736559</v>
       </c>
       <c r="E29" t="n" s="89">
-        <v>1.348310591E7</v>
+        <v>1.355639867E7</v>
       </c>
       <c r="F29" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G29" t="n" s="90">
-        <v>2.55414761E7</v>
+        <v>2.55442222E7</v>
       </c>
     </row>
     <row r="30">
@@ -2031,16 +2031,16 @@
         <v>73</v>
       </c>
       <c r="D30" t="n" s="91">
-        <v>0.622252</v>
+        <v>0.624216</v>
       </c>
       <c r="E30" t="n" s="92">
-        <v>1.142167065E7</v>
+        <v>1.148872276E7</v>
       </c>
       <c r="F30" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G30" t="n" s="93">
-        <v>2.31069042E7</v>
+        <v>2.31092403E7</v>
       </c>
     </row>
     <row r="31">
@@ -2054,16 +2054,16 @@
         <v>75</v>
       </c>
       <c r="D31" t="n" s="94">
-        <v>0.582839</v>
+        <v>0.583804</v>
       </c>
       <c r="E31" t="n" s="95">
-        <v>1.069822099E7</v>
+        <v>1.074493244E7</v>
       </c>
       <c r="F31" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G31" t="n" s="96">
-        <v>1.5883686E7</v>
+        <v>1.5885324E7</v>
       </c>
     </row>
     <row r="32">
@@ -2077,16 +2077,16 @@
         <v>77</v>
       </c>
       <c r="D32" t="n" s="97">
-        <v>0.570866</v>
+        <v>0.57185</v>
       </c>
       <c r="E32" t="n" s="98">
-        <v>1.047846152E7</v>
+        <v>1.052492754E7</v>
       </c>
       <c r="F32" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G32" t="n" s="99">
-        <v>1.579838125E7</v>
+        <v>1.580004375E7</v>
       </c>
     </row>
     <row r="33">
@@ -2097,42 +2097,42 @@
         <v>21</v>
       </c>
       <c r="C33" t="s" s="18">
-        <v>21</v>
+        <v>79</v>
       </c>
       <c r="D33" t="n" s="100">
-        <v>0.360298</v>
+        <v>0.263226</v>
       </c>
       <c r="E33" t="n" s="101">
-        <v>6613398.11</v>
-      </c>
-      <c r="F33" t="n" s="102">
-        <v>4.1779656199E8</v>
-      </c>
-      <c r="G33" t="n" s="103">
-        <v>1138114.82</v>
+        <v>4844693.48</v>
+      </c>
+      <c r="F33" t="s" s="18">
+        <v>21</v>
+      </c>
+      <c r="G33" t="n" s="102">
+        <v>4347162.84</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s" s="18">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B34" t="s" s="18">
         <v>21</v>
       </c>
       <c r="C34" t="s" s="18">
-        <v>80</v>
-      </c>
-      <c r="D34" t="n" s="104">
-        <v>0.265348</v>
-      </c>
-      <c r="E34" t="n" s="105">
-        <v>4870563.31</v>
-      </c>
-      <c r="F34" t="s" s="18">
-        <v>21</v>
+        <v>21</v>
+      </c>
+      <c r="D34" t="n" s="103">
+        <v>0.246881</v>
+      </c>
+      <c r="E34" t="n" s="104">
+        <v>4543848.9</v>
+      </c>
+      <c r="F34" t="n" s="105">
+        <v>4.1779656199E8</v>
       </c>
       <c r="G34" t="n" s="106">
-        <v>4347162.84</v>
+        <v>1138114.82</v>
       </c>
     </row>
     <row r="35">
@@ -2146,13 +2146,13 @@
         <v>83</v>
       </c>
       <c r="D35" t="n" s="107">
-        <v>0.16208</v>
+        <v>0.161735</v>
       </c>
       <c r="E35" t="n" s="108">
-        <v>1.7434516348E8</v>
+        <v>1.7444438881E8</v>
       </c>
       <c r="F35" t="n" s="109">
-        <v>1.7434516348E8</v>
+        <v>1.7444438881E8</v>
       </c>
       <c r="G35" t="n" s="110">
         <v>2.331E8</v>
@@ -2169,10 +2169,10 @@
         <v>85</v>
       </c>
       <c r="D36" t="n" s="111">
-        <v>0.14828</v>
+        <v>0.147079</v>
       </c>
       <c r="E36" t="n" s="112">
-        <v>2721735.18</v>
+        <v>2706994.99</v>
       </c>
       <c r="F36" t="s" s="18">
         <v>21</v>
@@ -2192,13 +2192,13 @@
         <v>88</v>
       </c>
       <c r="D37" t="n" s="114">
-        <v>0.072006</v>
+        <v>0.047462</v>
       </c>
       <c r="E37" t="n" s="115">
-        <v>3.3863945289E8</v>
+        <v>3.3639963714E8</v>
       </c>
       <c r="F37" t="n" s="116">
-        <v>3.3863945289E8</v>
+        <v>3.3639963714E8</v>
       </c>
       <c r="G37" t="n" s="117">
         <v>2.474E8</v>
@@ -2215,13 +2215,13 @@
         <v>91</v>
       </c>
       <c r="D38" t="n" s="118">
-        <v>0.03133</v>
+        <v>0.035477</v>
       </c>
       <c r="E38" t="n" s="119">
-        <v>6.834653052E7</v>
+        <v>6.846298957E7</v>
       </c>
       <c r="F38" t="n" s="120">
-        <v>6.834653052E7</v>
+        <v>6.846298957E7</v>
       </c>
       <c r="G38" t="n" s="121">
         <v>11025.0</v>
@@ -2232,91 +2232,91 @@
         <v>92</v>
       </c>
       <c r="B39" t="s" s="18">
-        <v>21</v>
+        <v>93</v>
       </c>
       <c r="C39" t="s" s="18">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D39" t="n" s="122">
-        <v>0.0</v>
+        <v>0.007934</v>
       </c>
       <c r="E39" t="n" s="123">
-        <v>7.57</v>
-      </c>
-      <c r="F39" t="s" s="18">
-        <v>21</v>
-      </c>
-      <c r="G39" t="n" s="124">
-        <v>10.58</v>
+        <v>7.274956233E7</v>
+      </c>
+      <c r="F39" t="n" s="124">
+        <v>7.274956233E7</v>
+      </c>
+      <c r="G39" t="n" s="125">
+        <v>5060.0</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s" s="18">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B40" t="s" s="18">
         <v>21</v>
       </c>
       <c r="C40" t="s" s="18">
-        <v>95</v>
-      </c>
-      <c r="D40" t="n" s="125">
-        <v>-0.006817</v>
-      </c>
-      <c r="E40" t="n" s="126">
-        <v>-125135.06</v>
+        <v>96</v>
+      </c>
+      <c r="D40" t="n" s="126">
+        <v>0.0</v>
+      </c>
+      <c r="E40" t="n" s="127">
+        <v>7.54</v>
       </c>
       <c r="F40" t="s" s="18">
         <v>21</v>
       </c>
-      <c r="G40" t="n" s="127">
-        <v>-177976.22</v>
+      <c r="G40" t="n" s="128">
+        <v>10.58</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s" s="18">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B41" t="s" s="18">
         <v>21</v>
       </c>
       <c r="C41" t="s" s="18">
-        <v>97</v>
-      </c>
-      <c r="D41" t="n" s="128">
-        <v>-0.007792</v>
-      </c>
-      <c r="E41" t="n" s="129">
-        <v>-143025.63</v>
+        <v>98</v>
+      </c>
+      <c r="D41" t="n" s="129">
+        <v>-0.006803</v>
+      </c>
+      <c r="E41" t="n" s="130">
+        <v>-125206.28</v>
       </c>
       <c r="F41" t="s" s="18">
         <v>21</v>
       </c>
-      <c r="G41" t="n" s="130">
-        <v>-2.2420698E7</v>
+      <c r="G41" t="n" s="131">
+        <v>-177976.22</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s" s="18">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B42" t="s" s="18">
-        <v>99</v>
+        <v>21</v>
       </c>
       <c r="C42" t="s" s="18">
         <v>100</v>
       </c>
-      <c r="D42" t="n" s="131">
-        <v>-0.028347</v>
-      </c>
-      <c r="E42" t="n" s="132">
-        <v>7.247855308E7</v>
-      </c>
-      <c r="F42" t="n" s="133">
-        <v>7.247855308E7</v>
+      <c r="D42" t="n" s="132">
+        <v>-0.007717</v>
+      </c>
+      <c r="E42" t="n" s="133">
+        <v>-142024.5</v>
+      </c>
+      <c r="F42" t="s" s="18">
+        <v>21</v>
       </c>
       <c r="G42" t="n" s="134">
-        <v>5060.0</v>
+        <v>-2.2420698E7</v>
       </c>
     </row>
     <row r="43">
@@ -2330,13 +2330,13 @@
         <v>103</v>
       </c>
       <c r="D43" t="n" s="135">
-        <v>-0.066739</v>
+        <v>-0.053734</v>
       </c>
       <c r="E43" t="n" s="136">
-        <v>8.661265629E7</v>
+        <v>8.623387071E7</v>
       </c>
       <c r="F43" t="n" s="137">
-        <v>8.661265629E7</v>
+        <v>8.623387071E7</v>
       </c>
       <c r="G43" t="n" s="138">
         <v>3420000.0</v>
@@ -2353,13 +2353,13 @@
         <v>106</v>
       </c>
       <c r="D44" t="n" s="139">
-        <v>-0.100075</v>
+        <v>-0.083223</v>
       </c>
       <c r="E44" t="n" s="140">
-        <v>1.1983728585E8</v>
+        <v>1.1948350851E8</v>
       </c>
       <c r="F44" t="n" s="141">
-        <v>1.1983728585E8</v>
+        <v>1.1948350851E8</v>
       </c>
       <c r="G44" t="n" s="142">
         <v>1.056E8</v>
@@ -2376,13 +2376,13 @@
         <v>109</v>
       </c>
       <c r="D45" t="n" s="143">
-        <v>-0.175445</v>
+        <v>-0.148171</v>
       </c>
       <c r="E45" t="n" s="144">
-        <v>2.1160425E8</v>
+        <v>2.120975E8</v>
       </c>
       <c r="F45" t="n" s="145">
-        <v>2.1160425E8</v>
+        <v>2.120975E8</v>
       </c>
       <c r="G45" t="n" s="146">
         <v>1.973E8</v>
@@ -2399,13 +2399,13 @@
         <v>112</v>
       </c>
       <c r="D46" t="n" s="147">
-        <v>-0.291363</v>
+        <v>-0.194203</v>
       </c>
       <c r="E46" t="n" s="148">
-        <v>1.718738922E8</v>
+        <v>1.7270635147E8</v>
       </c>
       <c r="F46" t="n" s="149">
-        <v>1.718738922E8</v>
+        <v>1.7270635147E8</v>
       </c>
       <c r="G46" t="n" s="150">
         <v>25260.0</v>
@@ -2422,13 +2422,13 @@
         <v>115</v>
       </c>
       <c r="D47" t="n" s="151">
-        <v>-0.424888</v>
+        <v>-0.434456</v>
       </c>
       <c r="E47" t="n" s="152">
-        <v>4.4659934375E8</v>
+        <v>4.4640214063E8</v>
       </c>
       <c r="F47" t="n" s="153">
-        <v>4.4659934375E8</v>
+        <v>4.4640214063E8</v>
       </c>
       <c r="G47" t="n" s="154">
         <v>4.207E8</v>
@@ -2445,13 +2445,13 @@
         <v>118</v>
       </c>
       <c r="D48" t="n" s="155">
-        <v>-0.807884</v>
+        <v>-0.732623</v>
       </c>
       <c r="E48" t="n" s="156">
-        <v>1.7674839E8</v>
+        <v>1.7809344E8</v>
       </c>
       <c r="F48" t="n" s="157">
-        <v>1.7674839E8</v>
+        <v>1.7809344E8</v>
       </c>
       <c r="G48" t="n" s="158">
         <v>44100.0</v>

</xml_diff>

<commit_message>
Update ALLW XLSX 2026-10-28
</commit_message>
<xml_diff>
--- a/latest/allw-latest.xlsx
+++ b/latest/allw-latest.xlsx
@@ -192,7 +192,7 @@
     <t>ALLW</t>
   </si>
   <si>
-    <t>As of 26-Oct-2026</t>
+    <t>As of 27-Oct-2026</t>
   </si>
   <si>
     <t>Name</t>
@@ -255,24 +255,24 @@
     <t>78463X509</t>
   </si>
   <si>
+    <t>TSY INFL IX N/B 01/36 1.875</t>
+  </si>
+  <si>
+    <t>91282CPU9</t>
+  </si>
+  <si>
+    <t>TSY INFL IX N/B 01/35 2.125</t>
+  </si>
+  <si>
+    <t>91282CML2</t>
+  </si>
+  <si>
     <t>US DOLLAR</t>
   </si>
   <si>
     <t>999USDZ92</t>
   </si>
   <si>
-    <t>TSY INFL IX N/B 01/36 1.875</t>
-  </si>
-  <si>
-    <t>91282CPU9</t>
-  </si>
-  <si>
-    <t>TSY INFL IX N/B 01/35 2.125</t>
-  </si>
-  <si>
-    <t>91282CML2</t>
-  </si>
-  <si>
     <t>TSY INFL IX N/B 07/34 1.875</t>
   </si>
   <si>
@@ -396,24 +396,24 @@
     <t>999EURZ94</t>
   </si>
   <si>
+    <t>AUST 10Y BOND FUT DEC26</t>
+  </si>
+  <si>
+    <t>XMZ6</t>
+  </si>
+  <si>
+    <t>ADI3BDHZ1</t>
+  </si>
+  <si>
+    <t>POUND STERLING</t>
+  </si>
+  <si>
+    <t>999GBPZ94</t>
+  </si>
+  <si>
     <t>TRS USD BCOMTR</t>
   </si>
   <si>
-    <t>AUST 10Y BOND FUT DEC26</t>
-  </si>
-  <si>
-    <t>XMZ6</t>
-  </si>
-  <si>
-    <t>ADI3BDHZ1</t>
-  </si>
-  <si>
-    <t>POUND STERLING</t>
-  </si>
-  <si>
-    <t>999GBPZ94</t>
-  </si>
-  <si>
     <t>EURO-BUND FUTURE  DEC26</t>
   </si>
   <si>
@@ -432,6 +432,33 @@
     <t>ADI391SG0</t>
   </si>
   <si>
+    <t>CANADIAN DOLLAR</t>
+  </si>
+  <si>
+    <t>999CADZ91</t>
+  </si>
+  <si>
+    <t>AUSTRALIAN DOLLAR</t>
+  </si>
+  <si>
+    <t>999AUDZ93</t>
+  </si>
+  <si>
+    <t>JAPANESE YEN</t>
+  </si>
+  <si>
+    <t>999JPYZ94</t>
+  </si>
+  <si>
+    <t>TOPIX INDX FUTR   DEC26</t>
+  </si>
+  <si>
+    <t>TPZ6</t>
+  </si>
+  <si>
+    <t>ADI3917X6</t>
+  </si>
+  <si>
     <t>FTSE 100 IDX FUT  DEC26</t>
   </si>
   <si>
@@ -441,33 +468,6 @@
     <t>ADI38QPG9</t>
   </si>
   <si>
-    <t>CANADIAN DOLLAR</t>
-  </si>
-  <si>
-    <t>999CADZ91</t>
-  </si>
-  <si>
-    <t>AUSTRALIAN DOLLAR</t>
-  </si>
-  <si>
-    <t>999AUDZ93</t>
-  </si>
-  <si>
-    <t>JAPANESE YEN</t>
-  </si>
-  <si>
-    <t>999JPYZ94</t>
-  </si>
-  <si>
-    <t>TOPIX INDX FUTR   DEC26</t>
-  </si>
-  <si>
-    <t>TPZ6</t>
-  </si>
-  <si>
-    <t>ADI3917X6</t>
-  </si>
-  <si>
     <t>LONG GILT FUTURE  DEC26</t>
   </si>
   <si>
@@ -477,6 +477,15 @@
     <t>ADI3BKVP1</t>
   </si>
   <si>
+    <t>EURO STOXX 50     DEC26</t>
+  </si>
+  <si>
+    <t>VGZ6</t>
+  </si>
+  <si>
+    <t>ADI2VHXS0</t>
+  </si>
+  <si>
     <t>US LONG BOND(CBT) DEC26</t>
   </si>
   <si>
@@ -484,15 +493,6 @@
   </si>
   <si>
     <t>ADI39KYC0</t>
-  </si>
-  <si>
-    <t>EURO STOXX 50     DEC26</t>
-  </si>
-  <si>
-    <t>VGZ6</t>
-  </si>
-  <si>
-    <t>ADI2VHXS0</t>
   </si>
   <si>
     <t>US 10YR NOTE (CBT)DEC26</t>
@@ -939,76 +939,76 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
@@ -1479,16 +1479,16 @@
         <v>22</v>
       </c>
       <c r="D6" t="n" s="19">
-        <v>33.843897</v>
+        <v>34.029566</v>
       </c>
       <c r="E6" t="n" s="20">
-        <v>6.2289851787E8</v>
+        <v>6.2709983373E8</v>
       </c>
       <c r="F6" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G6" t="n" s="21">
-        <v>6.2289851787E8</v>
+        <v>6.2709983373E8</v>
       </c>
     </row>
     <row r="7">
@@ -1502,10 +1502,10 @@
         <v>25</v>
       </c>
       <c r="D7" t="n" s="22">
-        <v>13.357804</v>
+        <v>13.421096</v>
       </c>
       <c r="E7" t="n" s="23">
-        <v>2.4585101148E8</v>
+        <v>2.473251348E8</v>
       </c>
       <c r="F7" t="s" s="18">
         <v>21</v>
@@ -1525,10 +1525,10 @@
         <v>27</v>
       </c>
       <c r="D8" t="n" s="25">
-        <v>4.917914</v>
+        <v>4.912305</v>
       </c>
       <c r="E8" t="n" s="26">
-        <v>9.051443821E7</v>
+        <v>9.052438766E7</v>
       </c>
       <c r="F8" t="s" s="18">
         <v>21</v>
@@ -1548,16 +1548,16 @@
         <v>29</v>
       </c>
       <c r="D9" t="n" s="28">
-        <v>4.299201</v>
+        <v>4.294811</v>
       </c>
       <c r="E9" t="n" s="29">
-        <v>7.91269959E7</v>
+        <v>7.914515664E7</v>
       </c>
       <c r="F9" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G9" t="n" s="30">
-        <v>8.372881E7</v>
+        <v>8.3737643E7</v>
       </c>
     </row>
     <row r="10">
@@ -1571,10 +1571,10 @@
         <v>32</v>
       </c>
       <c r="D10" t="n" s="31">
-        <v>4.271781</v>
+        <v>4.288913</v>
       </c>
       <c r="E10" t="n" s="32">
-        <v>7.86223356E7</v>
+        <v>7.90364727E7</v>
       </c>
       <c r="F10" t="s" s="18">
         <v>21</v>
@@ -1594,16 +1594,16 @@
         <v>34</v>
       </c>
       <c r="D11" t="n" s="34">
-        <v>4.218395</v>
+        <v>4.204712</v>
       </c>
       <c r="E11" t="n" s="35">
-        <v>7.763976667E7</v>
+        <v>7.748480906E7</v>
       </c>
       <c r="F11" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G11" t="n" s="36">
-        <v>7.763976667E7</v>
+        <v>8.2645298E7</v>
       </c>
     </row>
     <row r="12">
@@ -1617,16 +1617,16 @@
         <v>36</v>
       </c>
       <c r="D12" t="n" s="37">
-        <v>4.208866</v>
+        <v>4.011467</v>
       </c>
       <c r="E12" t="n" s="38">
-        <v>7.746437777E7</v>
+        <v>7.392365937E7</v>
       </c>
       <c r="F12" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G12" t="n" s="39">
-        <v>8.2637278E7</v>
+        <v>7.6499542E7</v>
       </c>
     </row>
     <row r="13">
@@ -1640,16 +1640,16 @@
         <v>38</v>
       </c>
       <c r="D13" t="n" s="40">
-        <v>4.01591</v>
+        <v>3.985137</v>
       </c>
       <c r="E13" t="n" s="41">
-        <v>7.391300689E7</v>
+        <v>7.343845081E7</v>
       </c>
       <c r="F13" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G13" t="n" s="42">
-        <v>7.6491611E7</v>
+        <v>7.343845081E7</v>
       </c>
     </row>
     <row r="14">
@@ -1663,16 +1663,16 @@
         <v>40</v>
       </c>
       <c r="D14" t="n" s="43">
-        <v>3.702411</v>
+        <v>3.698012</v>
       </c>
       <c r="E14" t="n" s="44">
-        <v>6.814305278E7</v>
+        <v>6.814729239E7</v>
       </c>
       <c r="F14" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G14" t="n" s="45">
-        <v>7.130294325E7</v>
+        <v>7.1310294E7</v>
       </c>
     </row>
     <row r="15">
@@ -1686,16 +1686,16 @@
         <v>42</v>
       </c>
       <c r="D15" t="n" s="46">
-        <v>3.524165</v>
+        <v>3.520581</v>
       </c>
       <c r="E15" t="n" s="47">
-        <v>6.486242223E7</v>
+        <v>6.487757943E7</v>
       </c>
       <c r="F15" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G15" t="n" s="48">
-        <v>6.835211845E7</v>
+        <v>6.835964905E7</v>
       </c>
     </row>
     <row r="16">
@@ -1709,10 +1709,10 @@
         <v>45</v>
       </c>
       <c r="D16" t="n" s="49">
-        <v>3.274594</v>
+        <v>3.258071</v>
       </c>
       <c r="E16" t="n" s="50">
-        <v>6.026905766E7</v>
+        <v>6.004001311E7</v>
       </c>
       <c r="F16" t="s" s="18">
         <v>21</v>
@@ -1732,16 +1732,16 @@
         <v>47</v>
       </c>
       <c r="D17" t="n" s="52">
-        <v>2.545407</v>
+        <v>2.542935</v>
       </c>
       <c r="E17" t="n" s="53">
-        <v>4.684833011E7</v>
+        <v>4.686142743E7</v>
       </c>
       <c r="F17" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G17" t="n" s="54">
-        <v>4.7919978E7</v>
+        <v>4.7924758E7</v>
       </c>
     </row>
     <row r="18">
@@ -1755,16 +1755,16 @@
         <v>49</v>
       </c>
       <c r="D18" t="n" s="55">
-        <v>1.508246</v>
+        <v>1.507197</v>
       </c>
       <c r="E18" t="n" s="56">
-        <v>2.775933766E7</v>
+        <v>2.777476759E7</v>
       </c>
       <c r="F18" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G18" t="n" s="57">
-        <v>3.56415498E7</v>
+        <v>3.56452713E7</v>
       </c>
     </row>
     <row r="19">
@@ -1778,16 +1778,16 @@
         <v>51</v>
       </c>
       <c r="D19" t="n" s="58">
-        <v>1.338589</v>
+        <v>1.338019</v>
       </c>
       <c r="E19" t="n" s="59">
-        <v>2.4636796E7</v>
+        <v>2.465712438E7</v>
       </c>
       <c r="F19" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G19" t="n" s="60">
-        <v>3.6305663E7</v>
+        <v>3.630949325E7</v>
       </c>
     </row>
     <row r="20">
@@ -1801,16 +1801,16 @@
         <v>53</v>
       </c>
       <c r="D20" t="n" s="61">
-        <v>1.265064</v>
+        <v>1.264085</v>
       </c>
       <c r="E20" t="n" s="62">
-        <v>2.328355888E7</v>
+        <v>2.329467782E7</v>
       </c>
       <c r="F20" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G20" t="n" s="63">
-        <v>2.68761432E7</v>
+        <v>2.68786762E7</v>
       </c>
     </row>
     <row r="21">
@@ -1824,16 +1824,16 @@
         <v>55</v>
       </c>
       <c r="D21" t="n" s="64">
-        <v>1.190681</v>
+        <v>1.189832</v>
       </c>
       <c r="E21" t="n" s="65">
-        <v>2.191454435E7</v>
+        <v>2.192632353E7</v>
       </c>
       <c r="F21" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G21" t="n" s="66">
-        <v>2.6645721E7</v>
+        <v>2.6648652E7</v>
       </c>
     </row>
     <row r="22">
@@ -1847,16 +1847,16 @@
         <v>57</v>
       </c>
       <c r="D22" t="n" s="67">
-        <v>1.167658</v>
+        <v>1.166848</v>
       </c>
       <c r="E22" t="n" s="68">
-        <v>2.149080803E7</v>
+        <v>2.15027826E7</v>
       </c>
       <c r="F22" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G22" t="n" s="69">
-        <v>2.479392E7</v>
+        <v>2.479656E7</v>
       </c>
     </row>
     <row r="23">
@@ -1870,16 +1870,16 @@
         <v>59</v>
       </c>
       <c r="D23" t="n" s="70">
-        <v>1.120475</v>
+        <v>1.119726</v>
       </c>
       <c r="E23" t="n" s="71">
-        <v>2.062238899E7</v>
+        <v>2.063441665E7</v>
       </c>
       <c r="F23" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G23" t="n" s="72">
-        <v>2.82710268E7</v>
+        <v>2.82738888E7</v>
       </c>
     </row>
     <row r="24">
@@ -1893,16 +1893,16 @@
         <v>61</v>
       </c>
       <c r="D24" t="n" s="73">
-        <v>0.975948</v>
+        <v>0.975142</v>
       </c>
       <c r="E24" t="n" s="74">
-        <v>1.796236218E7</v>
+        <v>1.797000374E7</v>
       </c>
       <c r="F24" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G24" t="n" s="75">
-        <v>2.5117382E7</v>
+        <v>2.5119835E7</v>
       </c>
     </row>
     <row r="25">
@@ -1916,16 +1916,16 @@
         <v>63</v>
       </c>
       <c r="D25" t="n" s="76">
-        <v>0.94735</v>
+        <v>0.946741</v>
       </c>
       <c r="E25" t="n" s="77">
-        <v>1.743602774E7</v>
+        <v>1.744662521E7</v>
       </c>
       <c r="F25" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G25" t="n" s="78">
-        <v>2.50329375E7</v>
+        <v>2.5035516E7</v>
       </c>
     </row>
     <row r="26">
@@ -1939,16 +1939,16 @@
         <v>65</v>
       </c>
       <c r="D26" t="n" s="79">
-        <v>0.905515</v>
+        <v>0.905002</v>
       </c>
       <c r="E26" t="n" s="80">
-        <v>1.66660474E7</v>
+        <v>1.667745592E7</v>
       </c>
       <c r="F26" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G26" t="n" s="81">
-        <v>2.48964705E7</v>
+        <v>2.48989835E7</v>
       </c>
     </row>
     <row r="27">
@@ -1962,16 +1962,16 @@
         <v>67</v>
       </c>
       <c r="D27" t="n" s="82">
-        <v>0.748539</v>
+        <v>0.748494</v>
       </c>
       <c r="E27" t="n" s="83">
-        <v>1.377690092E7</v>
+        <v>1.379330894E7</v>
       </c>
       <c r="F27" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G27" t="n" s="84">
-        <v>2.8504701E7</v>
+        <v>2.8507545E7</v>
       </c>
     </row>
     <row r="28">
@@ -1985,16 +1985,16 @@
         <v>69</v>
       </c>
       <c r="D28" t="n" s="85">
-        <v>0.746957</v>
+        <v>0.746491</v>
       </c>
       <c r="E28" t="n" s="86">
-        <v>1.374776957E7</v>
+        <v>1.375641072E7</v>
       </c>
       <c r="F28" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G28" t="n" s="87">
-        <v>1.96128564E7</v>
+        <v>1.96147996E7</v>
       </c>
     </row>
     <row r="29">
@@ -2008,16 +2008,16 @@
         <v>71</v>
       </c>
       <c r="D29" t="n" s="88">
-        <v>0.736559</v>
+        <v>0.736253</v>
       </c>
       <c r="E29" t="n" s="89">
-        <v>1.355639867E7</v>
+        <v>1.356773102E7</v>
       </c>
       <c r="F29" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G29" t="n" s="90">
-        <v>2.55442222E7</v>
+        <v>2.554677215E7</v>
       </c>
     </row>
     <row r="30">
@@ -2031,16 +2031,16 @@
         <v>73</v>
       </c>
       <c r="D30" t="n" s="91">
-        <v>0.624216</v>
+        <v>0.624086</v>
       </c>
       <c r="E30" t="n" s="92">
-        <v>1.148872276E7</v>
+        <v>1.15007177E7</v>
       </c>
       <c r="F30" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G30" t="n" s="93">
-        <v>2.31092403E7</v>
+        <v>2.31115764E7</v>
       </c>
     </row>
     <row r="31">
@@ -2054,16 +2054,16 @@
         <v>75</v>
       </c>
       <c r="D31" t="n" s="94">
-        <v>0.583804</v>
+        <v>0.583487</v>
       </c>
       <c r="E31" t="n" s="95">
-        <v>1.074493244E7</v>
+        <v>1.075255659E7</v>
       </c>
       <c r="F31" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G31" t="n" s="96">
-        <v>1.5885324E7</v>
+        <v>1.5886962E7</v>
       </c>
     </row>
     <row r="32">
@@ -2077,16 +2077,16 @@
         <v>77</v>
       </c>
       <c r="D32" t="n" s="97">
-        <v>0.57185</v>
+        <v>0.571597</v>
       </c>
       <c r="E32" t="n" s="98">
-        <v>1.052492754E7</v>
+        <v>1.053344204E7</v>
       </c>
       <c r="F32" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G32" t="n" s="99">
-        <v>1.580004375E7</v>
+        <v>1.580170625E7</v>
       </c>
     </row>
     <row r="33">
@@ -2100,7 +2100,7 @@
         <v>79</v>
       </c>
       <c r="D33" t="n" s="100">
-        <v>0.263226</v>
+        <v>0.262897</v>
       </c>
       <c r="E33" t="n" s="101">
         <v>4844693.48</v>
@@ -2117,68 +2117,68 @@
         <v>80</v>
       </c>
       <c r="B34" t="s" s="18">
-        <v>21</v>
+        <v>81</v>
       </c>
       <c r="C34" t="s" s="18">
-        <v>21</v>
+        <v>82</v>
       </c>
       <c r="D34" t="n" s="103">
-        <v>0.246881</v>
+        <v>0.168682</v>
       </c>
       <c r="E34" t="n" s="104">
-        <v>4543848.9</v>
+        <v>1.7457613506E8</v>
       </c>
       <c r="F34" t="n" s="105">
-        <v>4.1779656199E8</v>
+        <v>1.7457613506E8</v>
       </c>
       <c r="G34" t="n" s="106">
-        <v>1138114.82</v>
+        <v>2.331E8</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s" s="18">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B35" t="s" s="18">
-        <v>82</v>
+        <v>21</v>
       </c>
       <c r="C35" t="s" s="18">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D35" t="n" s="107">
-        <v>0.161735</v>
+        <v>0.146895</v>
       </c>
       <c r="E35" t="n" s="108">
-        <v>1.7444438881E8</v>
-      </c>
-      <c r="F35" t="n" s="109">
-        <v>1.7444438881E8</v>
-      </c>
-      <c r="G35" t="n" s="110">
-        <v>2.331E8</v>
+        <v>2706994.99</v>
+      </c>
+      <c r="F35" t="s" s="18">
+        <v>21</v>
+      </c>
+      <c r="G35" t="n" s="109">
+        <v>2033345.75</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s" s="18">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B36" t="s" s="18">
         <v>21</v>
       </c>
       <c r="C36" t="s" s="18">
-        <v>85</v>
-      </c>
-      <c r="D36" t="n" s="111">
-        <v>0.147079</v>
-      </c>
-      <c r="E36" t="n" s="112">
-        <v>2706994.99</v>
-      </c>
-      <c r="F36" t="s" s="18">
-        <v>21</v>
+        <v>21</v>
+      </c>
+      <c r="D36" t="n" s="110">
+        <v>0.083421</v>
+      </c>
+      <c r="E36" t="n" s="111">
+        <v>1537290.97</v>
+      </c>
+      <c r="F36" t="n" s="112">
+        <v>4.1779656199E8</v>
       </c>
       <c r="G36" t="n" s="113">
-        <v>2033345.75</v>
+        <v>1138114.82</v>
       </c>
     </row>
     <row r="37">
@@ -2192,13 +2192,13 @@
         <v>88</v>
       </c>
       <c r="D37" t="n" s="114">
-        <v>0.047462</v>
+        <v>0.059372</v>
       </c>
       <c r="E37" t="n" s="115">
-        <v>3.3639963714E8</v>
+        <v>3.3662020898E8</v>
       </c>
       <c r="F37" t="n" s="116">
-        <v>3.3639963714E8</v>
+        <v>3.3662020898E8</v>
       </c>
       <c r="G37" t="n" s="117">
         <v>2.474E8</v>
@@ -2215,13 +2215,13 @@
         <v>91</v>
       </c>
       <c r="D38" t="n" s="118">
-        <v>0.035477</v>
+        <v>0.051847</v>
       </c>
       <c r="E38" t="n" s="119">
-        <v>6.846298957E7</v>
+        <v>6.8765477E7</v>
       </c>
       <c r="F38" t="n" s="120">
-        <v>6.846298957E7</v>
+        <v>6.8765477E7</v>
       </c>
       <c r="G38" t="n" s="121">
         <v>11025.0</v>
@@ -2232,91 +2232,91 @@
         <v>92</v>
       </c>
       <c r="B39" t="s" s="18">
+        <v>21</v>
+      </c>
+      <c r="C39" t="s" s="18">
         <v>93</v>
       </c>
-      <c r="C39" t="s" s="18">
-        <v>94</v>
-      </c>
       <c r="D39" t="n" s="122">
-        <v>0.007934</v>
+        <v>0.0</v>
       </c>
       <c r="E39" t="n" s="123">
-        <v>7.274956233E7</v>
-      </c>
-      <c r="F39" t="n" s="124">
-        <v>7.274956233E7</v>
-      </c>
-      <c r="G39" t="n" s="125">
-        <v>5060.0</v>
+        <v>7.54</v>
+      </c>
+      <c r="F39" t="s" s="18">
+        <v>21</v>
+      </c>
+      <c r="G39" t="n" s="124">
+        <v>10.58</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s" s="18">
+        <v>94</v>
+      </c>
+      <c r="B40" t="s" s="18">
+        <v>21</v>
+      </c>
+      <c r="C40" t="s" s="18">
         <v>95</v>
       </c>
-      <c r="B40" t="s" s="18">
-        <v>21</v>
-      </c>
-      <c r="C40" t="s" s="18">
-        <v>96</v>
-      </c>
-      <c r="D40" t="n" s="126">
-        <v>0.0</v>
-      </c>
-      <c r="E40" t="n" s="127">
-        <v>7.54</v>
+      <c r="D40" t="n" s="125">
+        <v>-0.006794</v>
+      </c>
+      <c r="E40" t="n" s="126">
+        <v>-125206.28</v>
       </c>
       <c r="F40" t="s" s="18">
         <v>21</v>
       </c>
-      <c r="G40" t="n" s="128">
-        <v>10.58</v>
+      <c r="G40" t="n" s="127">
+        <v>-177976.22</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s" s="18">
+        <v>96</v>
+      </c>
+      <c r="B41" t="s" s="18">
+        <v>21</v>
+      </c>
+      <c r="C41" t="s" s="18">
         <v>97</v>
       </c>
-      <c r="B41" t="s" s="18">
-        <v>21</v>
-      </c>
-      <c r="C41" t="s" s="18">
-        <v>98</v>
-      </c>
-      <c r="D41" t="n" s="129">
-        <v>-0.006803</v>
-      </c>
-      <c r="E41" t="n" s="130">
-        <v>-125206.28</v>
+      <c r="D41" t="n" s="128">
+        <v>-0.007707</v>
+      </c>
+      <c r="E41" t="n" s="129">
+        <v>-142024.5</v>
       </c>
       <c r="F41" t="s" s="18">
         <v>21</v>
       </c>
-      <c r="G41" t="n" s="131">
-        <v>-177976.22</v>
+      <c r="G41" t="n" s="130">
+        <v>-2.2420698E7</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s" s="18">
+        <v>98</v>
+      </c>
+      <c r="B42" t="s" s="18">
         <v>99</v>
-      </c>
-      <c r="B42" t="s" s="18">
-        <v>21</v>
       </c>
       <c r="C42" t="s" s="18">
         <v>100</v>
       </c>
-      <c r="D42" t="n" s="132">
-        <v>-0.007717</v>
-      </c>
-      <c r="E42" t="n" s="133">
-        <v>-142024.5</v>
-      </c>
-      <c r="F42" t="s" s="18">
-        <v>21</v>
+      <c r="D42" t="n" s="131">
+        <v>-0.018399</v>
+      </c>
+      <c r="E42" t="n" s="132">
+        <v>8.688379311E7</v>
+      </c>
+      <c r="F42" t="n" s="133">
+        <v>8.688379311E7</v>
       </c>
       <c r="G42" t="n" s="134">
-        <v>-2.2420698E7</v>
+        <v>3420000.0</v>
       </c>
     </row>
     <row r="43">
@@ -2330,16 +2330,16 @@
         <v>103</v>
       </c>
       <c r="D43" t="n" s="135">
-        <v>-0.053734</v>
+        <v>-0.022416</v>
       </c>
       <c r="E43" t="n" s="136">
-        <v>8.623387071E7</v>
+        <v>7.219044259E7</v>
       </c>
       <c r="F43" t="n" s="137">
-        <v>8.623387071E7</v>
+        <v>7.219044259E7</v>
       </c>
       <c r="G43" t="n" s="138">
-        <v>3420000.0</v>
+        <v>5060.0</v>
       </c>
     </row>
     <row r="44">
@@ -2353,13 +2353,13 @@
         <v>106</v>
       </c>
       <c r="D44" t="n" s="139">
-        <v>-0.083223</v>
+        <v>-0.080068</v>
       </c>
       <c r="E44" t="n" s="140">
-        <v>1.1948350851E8</v>
+        <v>1.1953974266E8</v>
       </c>
       <c r="F44" t="n" s="141">
-        <v>1.1948350851E8</v>
+        <v>1.1953974266E8</v>
       </c>
       <c r="G44" t="n" s="142">
         <v>1.056E8</v>
@@ -2376,16 +2376,16 @@
         <v>109</v>
       </c>
       <c r="D45" t="n" s="143">
-        <v>-0.148171</v>
+        <v>-0.12369</v>
       </c>
       <c r="E45" t="n" s="144">
-        <v>2.120975E8</v>
+        <v>1.7400129722E8</v>
       </c>
       <c r="F45" t="n" s="145">
-        <v>2.120975E8</v>
+        <v>1.7400129722E8</v>
       </c>
       <c r="G45" t="n" s="146">
-        <v>1.973E8</v>
+        <v>25260.0</v>
       </c>
     </row>
     <row r="46">
@@ -2399,16 +2399,16 @@
         <v>112</v>
       </c>
       <c r="D46" t="n" s="147">
-        <v>-0.194203</v>
+        <v>-0.151332</v>
       </c>
       <c r="E46" t="n" s="148">
-        <v>1.7270635147E8</v>
+        <v>2.1203584375E8</v>
       </c>
       <c r="F46" t="n" s="149">
-        <v>1.7270635147E8</v>
+        <v>2.1203584375E8</v>
       </c>
       <c r="G46" t="n" s="150">
-        <v>25260.0</v>
+        <v>1.973E8</v>
       </c>
     </row>
     <row r="47">
@@ -2422,13 +2422,13 @@
         <v>115</v>
       </c>
       <c r="D47" t="n" s="151">
-        <v>-0.434456</v>
+        <v>-0.448181</v>
       </c>
       <c r="E47" t="n" s="152">
-        <v>4.4640214063E8</v>
+        <v>4.4613920313E8</v>
       </c>
       <c r="F47" t="n" s="153">
-        <v>4.4640214063E8</v>
+        <v>4.4613920313E8</v>
       </c>
       <c r="G47" t="n" s="154">
         <v>4.207E8</v>
@@ -2445,13 +2445,13 @@
         <v>118</v>
       </c>
       <c r="D48" t="n" s="155">
-        <v>-0.732623</v>
+        <v>-0.645077</v>
       </c>
       <c r="E48" t="n" s="156">
-        <v>1.7809344E8</v>
+        <v>1.7968986E8</v>
       </c>
       <c r="F48" t="n" s="157">
-        <v>1.7809344E8</v>
+        <v>1.7968986E8</v>
       </c>
       <c r="G48" t="n" s="158">
         <v>44100.0</v>

</xml_diff>

<commit_message>
Update ALLW XLSX 2026-10-29
</commit_message>
<xml_diff>
--- a/latest/allw-latest.xlsx
+++ b/latest/allw-latest.xlsx
@@ -192,7 +192,7 @@
     <t>ALLW</t>
   </si>
   <si>
-    <t>As of 27-Oct-2026</t>
+    <t>As of 28-Oct-2026</t>
   </si>
   <si>
     <t>Name</t>
@@ -240,21 +240,21 @@
     <t>912797TV9</t>
   </si>
   <si>
+    <t>STATE STREET SPDR PORTFOLIO EM</t>
+  </si>
+  <si>
+    <t>SPEM</t>
+  </si>
+  <si>
+    <t>78463X509</t>
+  </si>
+  <si>
     <t>TSY INFL IX N/B 07/35 1.875</t>
   </si>
   <si>
     <t>91282CNS6</t>
   </si>
   <si>
-    <t>STATE STREET SPDR PORTFOLIO EM</t>
-  </si>
-  <si>
-    <t>SPEM</t>
-  </si>
-  <si>
-    <t>78463X509</t>
-  </si>
-  <si>
     <t>TSY INFL IX N/B 01/36 1.875</t>
   </si>
   <si>
@@ -267,18 +267,18 @@
     <t>91282CML2</t>
   </si>
   <si>
+    <t>TSY INFL IX N/B 07/34 1.875</t>
+  </si>
+  <si>
+    <t>91282CLE9</t>
+  </si>
+  <si>
     <t>US DOLLAR</t>
   </si>
   <si>
     <t>999USDZ92</t>
   </si>
   <si>
-    <t>TSY INFL IX N/B 07/34 1.875</t>
-  </si>
-  <si>
-    <t>91282CLE9</t>
-  </si>
-  <si>
     <t>TSY INFL IX N/B 01/34 1.75</t>
   </si>
   <si>
@@ -396,6 +396,15 @@
     <t>999EURZ94</t>
   </si>
   <si>
+    <t>TRS USD BCOMTR</t>
+  </si>
+  <si>
+    <t>POUND STERLING</t>
+  </si>
+  <si>
+    <t>999GBPZ94</t>
+  </si>
+  <si>
     <t>AUST 10Y BOND FUT DEC26</t>
   </si>
   <si>
@@ -405,13 +414,13 @@
     <t>ADI3BDHZ1</t>
   </si>
   <si>
-    <t>POUND STERLING</t>
-  </si>
-  <si>
-    <t>999GBPZ94</t>
-  </si>
-  <si>
-    <t>TRS USD BCOMTR</t>
+    <t>SPI 200 FUTURES   DEC26</t>
+  </si>
+  <si>
+    <t>XPZ6</t>
+  </si>
+  <si>
+    <t>ADI391SG0</t>
   </si>
   <si>
     <t>EURO-BUND FUTURE  DEC26</t>
@@ -423,15 +432,6 @@
     <t>ADI39K4N9</t>
   </si>
   <si>
-    <t>SPI 200 FUTURES   DEC26</t>
-  </si>
-  <si>
-    <t>XPZ6</t>
-  </si>
-  <si>
-    <t>ADI391SG0</t>
-  </si>
-  <si>
     <t>CANADIAN DOLLAR</t>
   </si>
   <si>
@@ -450,6 +450,15 @@
     <t>999JPYZ94</t>
   </si>
   <si>
+    <t>FTSE 100 IDX FUT  DEC26</t>
+  </si>
+  <si>
+    <t>Z Z6</t>
+  </si>
+  <si>
+    <t>ADI38QPG9</t>
+  </si>
+  <si>
     <t>TOPIX INDX FUTR   DEC26</t>
   </si>
   <si>
@@ -457,15 +466,6 @@
   </si>
   <si>
     <t>ADI3917X6</t>
-  </si>
-  <si>
-    <t>FTSE 100 IDX FUT  DEC26</t>
-  </si>
-  <si>
-    <t>Z Z6</t>
-  </si>
-  <si>
-    <t>ADI38QPG9</t>
   </si>
   <si>
     <t>LONG GILT FUTURE  DEC26</t>
@@ -1479,16 +1479,16 @@
         <v>22</v>
       </c>
       <c r="D6" t="n" s="19">
-        <v>34.029566</v>
+        <v>34.374392</v>
       </c>
       <c r="E6" t="n" s="20">
-        <v>6.2709983373E8</v>
+        <v>6.3047819153E8</v>
       </c>
       <c r="F6" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G6" t="n" s="21">
-        <v>6.2709983373E8</v>
+        <v>6.3047819153E8</v>
       </c>
     </row>
     <row r="7">
@@ -1502,10 +1502,10 @@
         <v>25</v>
       </c>
       <c r="D7" t="n" s="22">
-        <v>13.421096</v>
+        <v>13.5291</v>
       </c>
       <c r="E7" t="n" s="23">
-        <v>2.473251348E8</v>
+        <v>2.481440922E8</v>
       </c>
       <c r="F7" t="s" s="18">
         <v>21</v>
@@ -1525,10 +1525,10 @@
         <v>27</v>
       </c>
       <c r="D8" t="n" s="25">
-        <v>4.912305</v>
+        <v>4.936453</v>
       </c>
       <c r="E8" t="n" s="26">
-        <v>9.052438766E7</v>
+        <v>9.054199314E7</v>
       </c>
       <c r="F8" t="s" s="18">
         <v>21</v>
@@ -1542,45 +1542,45 @@
         <v>28</v>
       </c>
       <c r="B9" t="s" s="18">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="C9" t="s" s="18">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D9" t="n" s="28">
-        <v>4.294811</v>
+        <v>4.325659</v>
       </c>
       <c r="E9" t="n" s="29">
-        <v>7.914515664E7</v>
+        <v>7.933911135E7</v>
       </c>
       <c r="F9" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G9" t="n" s="30">
-        <v>8.3737643E7</v>
+        <v>1592835.0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="18">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B10" t="s" s="18">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="C10" t="s" s="18">
         <v>32</v>
       </c>
       <c r="D10" t="n" s="31">
-        <v>4.288913</v>
+        <v>4.313358</v>
       </c>
       <c r="E10" t="n" s="32">
-        <v>7.90364727E7</v>
+        <v>7.911349046E7</v>
       </c>
       <c r="F10" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G10" t="n" s="33">
-        <v>1592835.0</v>
+        <v>8.3745673E7</v>
       </c>
     </row>
     <row r="11">
@@ -1594,16 +1594,16 @@
         <v>34</v>
       </c>
       <c r="D11" t="n" s="34">
-        <v>4.204712</v>
+        <v>4.221755</v>
       </c>
       <c r="E11" t="n" s="35">
-        <v>7.748480906E7</v>
+        <v>7.743335021E7</v>
       </c>
       <c r="F11" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G11" t="n" s="36">
-        <v>8.2645298E7</v>
+        <v>8.265412E7</v>
       </c>
     </row>
     <row r="12">
@@ -1617,16 +1617,16 @@
         <v>36</v>
       </c>
       <c r="D12" t="n" s="37">
-        <v>4.011467</v>
+        <v>4.02968</v>
       </c>
       <c r="E12" t="n" s="38">
-        <v>7.392365937E7</v>
+        <v>7.391040311E7</v>
       </c>
       <c r="F12" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G12" t="n" s="39">
-        <v>7.6499542E7</v>
+        <v>7.6507473E7</v>
       </c>
     </row>
     <row r="13">
@@ -1640,16 +1640,16 @@
         <v>38</v>
       </c>
       <c r="D13" t="n" s="40">
-        <v>3.985137</v>
+        <v>3.71612</v>
       </c>
       <c r="E13" t="n" s="41">
-        <v>7.343845081E7</v>
+        <v>6.815925048E7</v>
       </c>
       <c r="F13" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G13" t="n" s="42">
-        <v>7.343845081E7</v>
+        <v>7.13169765E7</v>
       </c>
     </row>
     <row r="14">
@@ -1663,16 +1663,16 @@
         <v>40</v>
       </c>
       <c r="D14" t="n" s="43">
-        <v>3.698012</v>
+        <v>3.58178</v>
       </c>
       <c r="E14" t="n" s="44">
-        <v>6.814729239E7</v>
+        <v>6.569525077E7</v>
       </c>
       <c r="F14" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G14" t="n" s="45">
-        <v>7.1310294E7</v>
+        <v>6.569525077E7</v>
       </c>
     </row>
     <row r="15">
@@ -1686,16 +1686,16 @@
         <v>42</v>
       </c>
       <c r="D15" t="n" s="46">
-        <v>3.520581</v>
+        <v>3.537848</v>
       </c>
       <c r="E15" t="n" s="47">
-        <v>6.487757943E7</v>
+        <v>6.488947233E7</v>
       </c>
       <c r="F15" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G15" t="n" s="48">
-        <v>6.835964905E7</v>
+        <v>6.83665521E7</v>
       </c>
     </row>
     <row r="16">
@@ -1709,10 +1709,10 @@
         <v>45</v>
       </c>
       <c r="D16" t="n" s="49">
-        <v>3.258071</v>
+        <v>3.272643</v>
       </c>
       <c r="E16" t="n" s="50">
-        <v>6.004001311E7</v>
+        <v>6.002521217E7</v>
       </c>
       <c r="F16" t="s" s="18">
         <v>21</v>
@@ -1732,16 +1732,16 @@
         <v>47</v>
       </c>
       <c r="D17" t="n" s="52">
-        <v>2.542935</v>
+        <v>2.553075</v>
       </c>
       <c r="E17" t="n" s="53">
-        <v>4.686142743E7</v>
+        <v>4.68272513E7</v>
       </c>
       <c r="F17" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G17" t="n" s="54">
-        <v>4.7924758E7</v>
+        <v>4.7930016E7</v>
       </c>
     </row>
     <row r="18">
@@ -1755,16 +1755,16 @@
         <v>49</v>
       </c>
       <c r="D18" t="n" s="55">
-        <v>1.507197</v>
+        <v>1.508055</v>
       </c>
       <c r="E18" t="n" s="56">
-        <v>2.777476759E7</v>
+        <v>2.76599979E7</v>
       </c>
       <c r="F18" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G18" t="n" s="57">
-        <v>3.56452713E7</v>
+        <v>3.56489928E7</v>
       </c>
     </row>
     <row r="19">
@@ -1778,16 +1778,16 @@
         <v>51</v>
       </c>
       <c r="D19" t="n" s="58">
-        <v>1.338019</v>
+        <v>1.337632</v>
       </c>
       <c r="E19" t="n" s="59">
-        <v>2.465712438E7</v>
+        <v>2.453418919E7</v>
       </c>
       <c r="F19" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G19" t="n" s="60">
-        <v>3.630949325E7</v>
+        <v>3.63133235E7</v>
       </c>
     </row>
     <row r="20">
@@ -1801,16 +1801,16 @@
         <v>53</v>
       </c>
       <c r="D20" t="n" s="61">
-        <v>1.264085</v>
+        <v>1.262799</v>
       </c>
       <c r="E20" t="n" s="62">
-        <v>2.329467782E7</v>
+        <v>2.316163502E7</v>
       </c>
       <c r="F20" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G20" t="n" s="63">
-        <v>2.68786762E7</v>
+        <v>2.68814625E7</v>
       </c>
     </row>
     <row r="21">
@@ -1824,16 +1824,16 @@
         <v>55</v>
       </c>
       <c r="D21" t="n" s="64">
-        <v>1.189832</v>
+        <v>1.18907</v>
       </c>
       <c r="E21" t="n" s="65">
-        <v>2.192632353E7</v>
+        <v>2.180933179E7</v>
       </c>
       <c r="F21" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G21" t="n" s="66">
-        <v>2.6648652E7</v>
+        <v>2.665133875E7</v>
       </c>
     </row>
     <row r="22">
@@ -1847,16 +1847,16 @@
         <v>57</v>
       </c>
       <c r="D22" t="n" s="67">
-        <v>1.166848</v>
+        <v>1.165736</v>
       </c>
       <c r="E22" t="n" s="68">
-        <v>2.15027826E7</v>
+        <v>2.138135333E7</v>
       </c>
       <c r="F22" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G22" t="n" s="69">
-        <v>2.479656E7</v>
+        <v>2.479896E7</v>
       </c>
     </row>
     <row r="23">
@@ -1870,16 +1870,16 @@
         <v>59</v>
       </c>
       <c r="D23" t="n" s="70">
-        <v>1.119726</v>
+        <v>1.120948</v>
       </c>
       <c r="E23" t="n" s="71">
-        <v>2.063441665E7</v>
+        <v>2.055987694E7</v>
       </c>
       <c r="F23" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G23" t="n" s="72">
-        <v>2.82738888E7</v>
+        <v>2.82769416E7</v>
       </c>
     </row>
     <row r="24">
@@ -1893,16 +1893,16 @@
         <v>61</v>
       </c>
       <c r="D24" t="n" s="73">
-        <v>0.975142</v>
+        <v>0.973937</v>
       </c>
       <c r="E24" t="n" s="74">
-        <v>1.797000374E7</v>
+        <v>1.786347927E7</v>
       </c>
       <c r="F24" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G24" t="n" s="75">
-        <v>2.5119835E7</v>
+        <v>2.5122511E7</v>
       </c>
     </row>
     <row r="25">
@@ -1916,16 +1916,16 @@
         <v>63</v>
       </c>
       <c r="D25" t="n" s="76">
-        <v>0.946741</v>
+        <v>0.947442</v>
       </c>
       <c r="E25" t="n" s="77">
-        <v>1.744662521E7</v>
+        <v>1.737751347E7</v>
       </c>
       <c r="F25" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G25" t="n" s="78">
-        <v>2.5035516E7</v>
+        <v>2.50380945E7</v>
       </c>
     </row>
     <row r="26">
@@ -1939,16 +1939,16 @@
         <v>65</v>
       </c>
       <c r="D26" t="n" s="79">
-        <v>0.905002</v>
+        <v>0.904275</v>
       </c>
       <c r="E26" t="n" s="80">
-        <v>1.667745592E7</v>
+        <v>1.658575853E7</v>
       </c>
       <c r="F26" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G26" t="n" s="81">
-        <v>2.48989835E7</v>
+        <v>2.49014965E7</v>
       </c>
     </row>
     <row r="27">
@@ -1962,16 +1962,16 @@
         <v>67</v>
       </c>
       <c r="D27" t="n" s="82">
-        <v>0.748494</v>
+        <v>0.746728</v>
       </c>
       <c r="E27" t="n" s="83">
-        <v>1.379330894E7</v>
+        <v>1.369612373E7</v>
       </c>
       <c r="F27" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G27" t="n" s="84">
-        <v>2.8507545E7</v>
+        <v>2.8510389E7</v>
       </c>
     </row>
     <row r="28">
@@ -1985,16 +1985,16 @@
         <v>69</v>
       </c>
       <c r="D28" t="n" s="85">
-        <v>0.746491</v>
+        <v>0.746021</v>
       </c>
       <c r="E28" t="n" s="86">
-        <v>1.375641072E7</v>
+        <v>1.368315803E7</v>
       </c>
       <c r="F28" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G28" t="n" s="87">
-        <v>1.96147996E7</v>
+        <v>1.96168816E7</v>
       </c>
     </row>
     <row r="29">
@@ -2008,16 +2008,16 @@
         <v>71</v>
       </c>
       <c r="D29" t="n" s="88">
-        <v>0.736253</v>
+        <v>0.734796</v>
       </c>
       <c r="E29" t="n" s="89">
-        <v>1.356773102E7</v>
+        <v>1.347726741E7</v>
       </c>
       <c r="F29" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G29" t="n" s="90">
-        <v>2.554677215E7</v>
+        <v>2.55493221E7</v>
       </c>
     </row>
     <row r="30">
@@ -2031,16 +2031,16 @@
         <v>73</v>
       </c>
       <c r="D30" t="n" s="91">
-        <v>0.624086</v>
+        <v>0.622616</v>
       </c>
       <c r="E30" t="n" s="92">
-        <v>1.15007177E7</v>
+        <v>1.141971739E7</v>
       </c>
       <c r="F30" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G30" t="n" s="93">
-        <v>2.31115764E7</v>
+        <v>2.31139125E7</v>
       </c>
     </row>
     <row r="31">
@@ -2054,16 +2054,16 @@
         <v>75</v>
       </c>
       <c r="D31" t="n" s="94">
-        <v>0.583487</v>
+        <v>0.582851</v>
       </c>
       <c r="E31" t="n" s="95">
-        <v>1.075255659E7</v>
+        <v>1.069035899E7</v>
       </c>
       <c r="F31" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G31" t="n" s="96">
-        <v>1.5886962E7</v>
+        <v>1.58886E7</v>
       </c>
     </row>
     <row r="32">
@@ -2077,16 +2077,16 @@
         <v>77</v>
       </c>
       <c r="D32" t="n" s="97">
-        <v>0.571597</v>
+        <v>0.570885</v>
       </c>
       <c r="E32" t="n" s="98">
-        <v>1.053344204E7</v>
+        <v>1.047088783E7</v>
       </c>
       <c r="F32" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G32" t="n" s="99">
-        <v>1.580170625E7</v>
+        <v>1.580325E7</v>
       </c>
     </row>
     <row r="33">
@@ -2100,10 +2100,10 @@
         <v>79</v>
       </c>
       <c r="D33" t="n" s="100">
-        <v>0.262897</v>
+        <v>0.26402</v>
       </c>
       <c r="E33" t="n" s="101">
-        <v>4844693.48</v>
+        <v>4842523.99</v>
       </c>
       <c r="F33" t="s" s="18">
         <v>21</v>
@@ -2117,39 +2117,39 @@
         <v>80</v>
       </c>
       <c r="B34" t="s" s="18">
-        <v>81</v>
+        <v>21</v>
       </c>
       <c r="C34" t="s" s="18">
-        <v>82</v>
+        <v>21</v>
       </c>
       <c r="D34" t="n" s="103">
-        <v>0.168682</v>
+        <v>0.162273</v>
       </c>
       <c r="E34" t="n" s="104">
-        <v>1.7457613506E8</v>
+        <v>2976323.37</v>
       </c>
       <c r="F34" t="n" s="105">
-        <v>1.7457613506E8</v>
+        <v>4.1779656199E8</v>
       </c>
       <c r="G34" t="n" s="106">
-        <v>2.331E8</v>
+        <v>1138114.82</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s" s="18">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B35" t="s" s="18">
         <v>21</v>
       </c>
       <c r="C35" t="s" s="18">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D35" t="n" s="107">
-        <v>0.146895</v>
+        <v>0.14745</v>
       </c>
       <c r="E35" t="n" s="108">
-        <v>2706994.99</v>
+        <v>2704453.08</v>
       </c>
       <c r="F35" t="s" s="18">
         <v>21</v>
@@ -2160,25 +2160,25 @@
     </row>
     <row r="36">
       <c r="A36" t="s" s="18">
+        <v>83</v>
+      </c>
+      <c r="B36" t="s" s="18">
+        <v>84</v>
+      </c>
+      <c r="C36" t="s" s="18">
         <v>85</v>
       </c>
-      <c r="B36" t="s" s="18">
-        <v>21</v>
-      </c>
-      <c r="C36" t="s" s="18">
-        <v>21</v>
-      </c>
       <c r="D36" t="n" s="110">
-        <v>0.083421</v>
+        <v>0.13008</v>
       </c>
       <c r="E36" t="n" s="111">
-        <v>1537290.97</v>
+        <v>1.738900731E8</v>
       </c>
       <c r="F36" t="n" s="112">
-        <v>4.1779656199E8</v>
+        <v>1.738900731E8</v>
       </c>
       <c r="G36" t="n" s="113">
-        <v>1138114.82</v>
+        <v>2.331E8</v>
       </c>
     </row>
     <row r="37">
@@ -2192,16 +2192,16 @@
         <v>88</v>
       </c>
       <c r="D37" t="n" s="114">
-        <v>0.059372</v>
+        <v>0.049565</v>
       </c>
       <c r="E37" t="n" s="115">
-        <v>3.3662020898E8</v>
+        <v>6.873359176E7</v>
       </c>
       <c r="F37" t="n" s="116">
-        <v>3.3662020898E8</v>
+        <v>6.873359176E7</v>
       </c>
       <c r="G37" t="n" s="117">
-        <v>2.474E8</v>
+        <v>11025.0</v>
       </c>
     </row>
     <row r="38">
@@ -2215,16 +2215,16 @@
         <v>91</v>
       </c>
       <c r="D38" t="n" s="118">
-        <v>0.051847</v>
+        <v>0.016051</v>
       </c>
       <c r="E38" t="n" s="119">
-        <v>6.8765477E7</v>
+        <v>3.3567025284E8</v>
       </c>
       <c r="F38" t="n" s="120">
-        <v>6.8765477E7</v>
+        <v>3.3567025284E8</v>
       </c>
       <c r="G38" t="n" s="121">
-        <v>11025.0</v>
+        <v>2.474E8</v>
       </c>
     </row>
     <row r="39">
@@ -2261,10 +2261,10 @@
         <v>95</v>
       </c>
       <c r="D40" t="n" s="125">
-        <v>-0.006794</v>
+        <v>-0.006828</v>
       </c>
       <c r="E40" t="n" s="126">
-        <v>-125206.28</v>
+        <v>-125232.98</v>
       </c>
       <c r="F40" t="s" s="18">
         <v>21</v>
@@ -2284,10 +2284,10 @@
         <v>97</v>
       </c>
       <c r="D41" t="n" s="128">
-        <v>-0.007707</v>
+        <v>-0.007725</v>
       </c>
       <c r="E41" t="n" s="129">
-        <v>-142024.5</v>
+        <v>-141696.88</v>
       </c>
       <c r="F41" t="s" s="18">
         <v>21</v>
@@ -2307,16 +2307,16 @@
         <v>100</v>
       </c>
       <c r="D42" t="n" s="131">
-        <v>-0.018399</v>
+        <v>-0.022317</v>
       </c>
       <c r="E42" t="n" s="132">
-        <v>8.688379311E7</v>
+        <v>7.212601965E7</v>
       </c>
       <c r="F42" t="n" s="133">
-        <v>8.688379311E7</v>
+        <v>7.212601965E7</v>
       </c>
       <c r="G42" t="n" s="134">
-        <v>3420000.0</v>
+        <v>5060.0</v>
       </c>
     </row>
     <row r="43">
@@ -2330,16 +2330,16 @@
         <v>103</v>
       </c>
       <c r="D43" t="n" s="135">
-        <v>-0.022416</v>
+        <v>-0.036119</v>
       </c>
       <c r="E43" t="n" s="136">
-        <v>7.219044259E7</v>
+        <v>8.635916072E7</v>
       </c>
       <c r="F43" t="n" s="137">
-        <v>7.219044259E7</v>
+        <v>8.635916072E7</v>
       </c>
       <c r="G43" t="n" s="138">
-        <v>5060.0</v>
+        <v>3420000.0</v>
       </c>
     </row>
     <row r="44">
@@ -2353,13 +2353,13 @@
         <v>106</v>
       </c>
       <c r="D44" t="n" s="139">
-        <v>-0.080068</v>
+        <v>-0.08037</v>
       </c>
       <c r="E44" t="n" s="140">
-        <v>1.1953974266E8</v>
+        <v>1.1942749295E8</v>
       </c>
       <c r="F44" t="n" s="141">
-        <v>1.1953974266E8</v>
+        <v>1.1942749295E8</v>
       </c>
       <c r="G44" t="n" s="142">
         <v>1.056E8</v>
@@ -2376,13 +2376,13 @@
         <v>109</v>
       </c>
       <c r="D45" t="n" s="143">
-        <v>-0.12369</v>
+        <v>-0.122684</v>
       </c>
       <c r="E45" t="n" s="144">
-        <v>1.7400129722E8</v>
+        <v>1.7395151642E8</v>
       </c>
       <c r="F45" t="n" s="145">
-        <v>1.7400129722E8</v>
+        <v>1.7395151642E8</v>
       </c>
       <c r="G45" t="n" s="146">
         <v>25260.0</v>
@@ -2399,13 +2399,13 @@
         <v>112</v>
       </c>
       <c r="D46" t="n" s="147">
-        <v>-0.151332</v>
+        <v>-0.229362</v>
       </c>
       <c r="E46" t="n" s="148">
-        <v>2.1203584375E8</v>
+        <v>2.1061775E8</v>
       </c>
       <c r="F46" t="n" s="149">
-        <v>2.1203584375E8</v>
+        <v>2.1061775E8</v>
       </c>
       <c r="G46" t="n" s="150">
         <v>1.973E8</v>
@@ -2422,13 +2422,13 @@
         <v>115</v>
       </c>
       <c r="D47" t="n" s="151">
-        <v>-0.448181</v>
+        <v>-0.507639</v>
       </c>
       <c r="E47" t="n" s="152">
-        <v>4.4613920313E8</v>
+        <v>4.4508745313E8</v>
       </c>
       <c r="F47" t="n" s="153">
-        <v>4.4613920313E8</v>
+        <v>4.4508745313E8</v>
       </c>
       <c r="G47" t="n" s="154">
         <v>4.207E8</v>
@@ -2445,13 +2445,13 @@
         <v>118</v>
       </c>
       <c r="D48" t="n" s="155">
-        <v>-0.645077</v>
+        <v>-0.703423</v>
       </c>
       <c r="E48" t="n" s="156">
-        <v>1.7968986E8</v>
+        <v>1.7867556E8</v>
       </c>
       <c r="F48" t="n" s="157">
-        <v>1.7968986E8</v>
+        <v>1.7867556E8</v>
       </c>
       <c r="G48" t="n" s="158">
         <v>44100.0</v>

</xml_diff>

<commit_message>
Update ALLW XLSX 2026-10-30
</commit_message>
<xml_diff>
--- a/latest/allw-latest.xlsx
+++ b/latest/allw-latest.xlsx
@@ -192,7 +192,7 @@
     <t>ALLW</t>
   </si>
   <si>
-    <t>As of 28-Oct-2026</t>
+    <t>As of 29-Oct-2026</t>
   </si>
   <si>
     <t>Name</t>
@@ -240,6 +240,12 @@
     <t>912797TV9</t>
   </si>
   <si>
+    <t>TSY INFL IX N/B 07/35 1.875</t>
+  </si>
+  <si>
+    <t>91282CNS6</t>
+  </si>
+  <si>
     <t>STATE STREET SPDR PORTFOLIO EM</t>
   </si>
   <si>
@@ -249,18 +255,18 @@
     <t>78463X509</t>
   </si>
   <si>
-    <t>TSY INFL IX N/B 07/35 1.875</t>
-  </si>
-  <si>
-    <t>91282CNS6</t>
-  </si>
-  <si>
     <t>TSY INFL IX N/B 01/36 1.875</t>
   </si>
   <si>
     <t>91282CPU9</t>
   </si>
   <si>
+    <t>US DOLLAR</t>
+  </si>
+  <si>
+    <t>999USDZ92</t>
+  </si>
+  <si>
     <t>TSY INFL IX N/B 01/35 2.125</t>
   </si>
   <si>
@@ -273,12 +279,6 @@
     <t>91282CLE9</t>
   </si>
   <si>
-    <t>US DOLLAR</t>
-  </si>
-  <si>
-    <t>999USDZ92</t>
-  </si>
-  <si>
     <t>TSY INFL IX N/B 01/34 1.75</t>
   </si>
   <si>
@@ -396,48 +396,57 @@
     <t>999EURZ94</t>
   </si>
   <si>
+    <t>AUST 10Y BOND FUT DEC26</t>
+  </si>
+  <si>
+    <t>XMZ6</t>
+  </si>
+  <si>
+    <t>ADI3BDHZ1</t>
+  </si>
+  <si>
+    <t>POUND STERLING</t>
+  </si>
+  <si>
+    <t>999GBPZ94</t>
+  </si>
+  <si>
+    <t>SPI 200 FUTURES   DEC26</t>
+  </si>
+  <si>
+    <t>XPZ6</t>
+  </si>
+  <si>
+    <t>ADI391SG0</t>
+  </si>
+  <si>
+    <t>EURO-BUND FUTURE  DEC26</t>
+  </si>
+  <si>
+    <t>RXZ6</t>
+  </si>
+  <si>
+    <t>ADI39K4N9</t>
+  </si>
+  <si>
+    <t>TOPIX INDX FUTR   DEC26</t>
+  </si>
+  <si>
+    <t>TPZ6</t>
+  </si>
+  <si>
+    <t>ADI3917X6</t>
+  </si>
+  <si>
+    <t>CANADIAN DOLLAR</t>
+  </si>
+  <si>
+    <t>999CADZ91</t>
+  </si>
+  <si>
     <t>TRS USD BCOMTR</t>
   </si>
   <si>
-    <t>POUND STERLING</t>
-  </si>
-  <si>
-    <t>999GBPZ94</t>
-  </si>
-  <si>
-    <t>AUST 10Y BOND FUT DEC26</t>
-  </si>
-  <si>
-    <t>XMZ6</t>
-  </si>
-  <si>
-    <t>ADI3BDHZ1</t>
-  </si>
-  <si>
-    <t>SPI 200 FUTURES   DEC26</t>
-  </si>
-  <si>
-    <t>XPZ6</t>
-  </si>
-  <si>
-    <t>ADI391SG0</t>
-  </si>
-  <si>
-    <t>EURO-BUND FUTURE  DEC26</t>
-  </si>
-  <si>
-    <t>RXZ6</t>
-  </si>
-  <si>
-    <t>ADI39K4N9</t>
-  </si>
-  <si>
-    <t>CANADIAN DOLLAR</t>
-  </si>
-  <si>
-    <t>999CADZ91</t>
-  </si>
-  <si>
     <t>AUSTRALIAN DOLLAR</t>
   </si>
   <si>
@@ -457,15 +466,6 @@
   </si>
   <si>
     <t>ADI38QPG9</t>
-  </si>
-  <si>
-    <t>TOPIX INDX FUTR   DEC26</t>
-  </si>
-  <si>
-    <t>TPZ6</t>
-  </si>
-  <si>
-    <t>ADI3917X6</t>
   </si>
   <si>
     <t>LONG GILT FUTURE  DEC26</t>
@@ -993,22 +993,22 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyNumberFormat="true">
@@ -1479,16 +1479,16 @@
         <v>22</v>
       </c>
       <c r="D6" t="n" s="19">
-        <v>34.374392</v>
+        <v>33.786555</v>
       </c>
       <c r="E6" t="n" s="20">
-        <v>6.3047819153E8</v>
+        <v>6.2083297667E8</v>
       </c>
       <c r="F6" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G6" t="n" s="21">
-        <v>6.3047819153E8</v>
+        <v>6.2083297667E8</v>
       </c>
     </row>
     <row r="7">
@@ -1502,10 +1502,10 @@
         <v>25</v>
       </c>
       <c r="D7" t="n" s="22">
-        <v>13.5291</v>
+        <v>13.458276</v>
       </c>
       <c r="E7" t="n" s="23">
-        <v>2.481440922E8</v>
+        <v>2.4729783622E8</v>
       </c>
       <c r="F7" t="s" s="18">
         <v>21</v>
@@ -1525,10 +1525,10 @@
         <v>27</v>
       </c>
       <c r="D8" t="n" s="25">
-        <v>4.936453</v>
+        <v>4.928369</v>
       </c>
       <c r="E8" t="n" s="26">
-        <v>9.054199314E7</v>
+        <v>9.05595161E7</v>
       </c>
       <c r="F8" t="s" s="18">
         <v>21</v>
@@ -1542,45 +1542,45 @@
         <v>28</v>
       </c>
       <c r="B9" t="s" s="18">
+        <v>21</v>
+      </c>
+      <c r="C9" t="s" s="18">
         <v>29</v>
       </c>
-      <c r="C9" t="s" s="18">
-        <v>30</v>
-      </c>
       <c r="D9" t="n" s="28">
-        <v>4.325659</v>
+        <v>4.315807</v>
       </c>
       <c r="E9" t="n" s="29">
-        <v>7.933911135E7</v>
+        <v>7.930359539E7</v>
       </c>
       <c r="F9" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G9" t="n" s="30">
-        <v>1592835.0</v>
+        <v>8.3763339E7</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="18">
+        <v>30</v>
+      </c>
+      <c r="B10" t="s" s="18">
         <v>31</v>
-      </c>
-      <c r="B10" t="s" s="18">
-        <v>21</v>
       </c>
       <c r="C10" t="s" s="18">
         <v>32</v>
       </c>
       <c r="D10" t="n" s="31">
-        <v>4.313358</v>
+        <v>4.283933</v>
       </c>
       <c r="E10" t="n" s="32">
-        <v>7.911349046E7</v>
+        <v>7.87179057E7</v>
       </c>
       <c r="F10" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G10" t="n" s="33">
-        <v>8.3745673E7</v>
+        <v>1592835.0</v>
       </c>
     </row>
     <row r="11">
@@ -1594,16 +1594,16 @@
         <v>34</v>
       </c>
       <c r="D11" t="n" s="34">
-        <v>4.221755</v>
+        <v>4.22455</v>
       </c>
       <c r="E11" t="n" s="35">
-        <v>7.743335021E7</v>
+        <v>7.7626742E7</v>
       </c>
       <c r="F11" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G11" t="n" s="36">
-        <v>8.265412E7</v>
+        <v>8.2670962E7</v>
       </c>
     </row>
     <row r="12">
@@ -1617,16 +1617,16 @@
         <v>36</v>
       </c>
       <c r="D12" t="n" s="37">
-        <v>4.02968</v>
+        <v>4.100128</v>
       </c>
       <c r="E12" t="n" s="38">
-        <v>7.391040311E7</v>
+        <v>7.534046563E7</v>
       </c>
       <c r="F12" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G12" t="n" s="39">
-        <v>7.6507473E7</v>
+        <v>7.534046563E7</v>
       </c>
     </row>
     <row r="13">
@@ -1640,16 +1640,16 @@
         <v>38</v>
       </c>
       <c r="D13" t="n" s="40">
-        <v>3.71612</v>
+        <v>4.031476</v>
       </c>
       <c r="E13" t="n" s="41">
-        <v>6.815925048E7</v>
+        <v>7.407897222E7</v>
       </c>
       <c r="F13" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G13" t="n" s="42">
-        <v>7.13169765E7</v>
+        <v>7.6522614E7</v>
       </c>
     </row>
     <row r="14">
@@ -1663,16 +1663,16 @@
         <v>40</v>
       </c>
       <c r="D14" t="n" s="43">
-        <v>3.58178</v>
+        <v>3.717815</v>
       </c>
       <c r="E14" t="n" s="44">
-        <v>6.569525077E7</v>
+        <v>6.831540658E7</v>
       </c>
       <c r="F14" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G14" t="n" s="45">
-        <v>6.569525077E7</v>
+        <v>7.1331678E7</v>
       </c>
     </row>
     <row r="15">
@@ -1686,16 +1686,16 @@
         <v>42</v>
       </c>
       <c r="D15" t="n" s="46">
-        <v>3.537848</v>
+        <v>3.539861</v>
       </c>
       <c r="E15" t="n" s="47">
-        <v>6.488947233E7</v>
+        <v>6.504548027E7</v>
       </c>
       <c r="F15" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G15" t="n" s="48">
-        <v>6.83665521E7</v>
+        <v>6.83803582E7</v>
       </c>
     </row>
     <row r="16">
@@ -1709,10 +1709,10 @@
         <v>45</v>
       </c>
       <c r="D16" t="n" s="49">
-        <v>3.272643</v>
+        <v>3.254972</v>
       </c>
       <c r="E16" t="n" s="50">
-        <v>6.002521217E7</v>
+        <v>5.981059854E7</v>
       </c>
       <c r="F16" t="s" s="18">
         <v>21</v>
@@ -1732,16 +1732,16 @@
         <v>47</v>
       </c>
       <c r="D17" t="n" s="52">
-        <v>2.553075</v>
+        <v>2.554922</v>
       </c>
       <c r="E17" t="n" s="53">
-        <v>4.68272513E7</v>
+        <v>4.694707721E7</v>
       </c>
       <c r="F17" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G17" t="n" s="54">
-        <v>4.7930016E7</v>
+        <v>4.7939576E7</v>
       </c>
     </row>
     <row r="18">
@@ -1755,16 +1755,16 @@
         <v>49</v>
       </c>
       <c r="D18" t="n" s="55">
-        <v>1.508055</v>
+        <v>1.50916</v>
       </c>
       <c r="E18" t="n" s="56">
-        <v>2.76599979E7</v>
+        <v>2.773104303E7</v>
       </c>
       <c r="F18" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G18" t="n" s="57">
-        <v>3.56489928E7</v>
+        <v>3.56561877E7</v>
       </c>
     </row>
     <row r="19">
@@ -1778,16 +1778,16 @@
         <v>51</v>
       </c>
       <c r="D19" t="n" s="58">
-        <v>1.337632</v>
+        <v>1.339393</v>
       </c>
       <c r="E19" t="n" s="59">
-        <v>2.453418919E7</v>
+        <v>2.461155009E7</v>
       </c>
       <c r="F19" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G19" t="n" s="60">
-        <v>3.63133235E7</v>
+        <v>3.632072865E7</v>
       </c>
     </row>
     <row r="20">
@@ -1801,16 +1801,16 @@
         <v>53</v>
       </c>
       <c r="D20" t="n" s="61">
-        <v>1.262799</v>
+        <v>1.263835</v>
       </c>
       <c r="E20" t="n" s="62">
-        <v>2.316163502E7</v>
+        <v>2.322315146E7</v>
       </c>
       <c r="F20" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G20" t="n" s="63">
-        <v>2.68814625E7</v>
+        <v>2.68870351E7</v>
       </c>
     </row>
     <row r="21">
@@ -1824,16 +1824,16 @@
         <v>55</v>
       </c>
       <c r="D21" t="n" s="64">
-        <v>1.18907</v>
+        <v>1.189654</v>
       </c>
       <c r="E21" t="n" s="65">
-        <v>2.180933179E7</v>
+        <v>2.186006586E7</v>
       </c>
       <c r="F21" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G21" t="n" s="66">
-        <v>2.665133875E7</v>
+        <v>2.665671225E7</v>
       </c>
     </row>
     <row r="22">
@@ -1847,16 +1847,16 @@
         <v>57</v>
       </c>
       <c r="D22" t="n" s="67">
-        <v>1.165736</v>
+        <v>1.166765</v>
       </c>
       <c r="E22" t="n" s="68">
-        <v>2.138135333E7</v>
+        <v>2.143947308E7</v>
       </c>
       <c r="F22" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G22" t="n" s="69">
-        <v>2.479896E7</v>
+        <v>2.4804E7</v>
       </c>
     </row>
     <row r="23">
@@ -1870,16 +1870,16 @@
         <v>59</v>
       </c>
       <c r="D23" t="n" s="70">
-        <v>1.120948</v>
+        <v>1.122309</v>
       </c>
       <c r="E23" t="n" s="71">
-        <v>2.055987694E7</v>
+        <v>2.062259297E7</v>
       </c>
       <c r="F23" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G23" t="n" s="72">
-        <v>2.82769416E7</v>
+        <v>2.82826656E7</v>
       </c>
     </row>
     <row r="24">
@@ -1893,16 +1893,16 @@
         <v>61</v>
       </c>
       <c r="D24" t="n" s="73">
-        <v>0.973937</v>
+        <v>0.974756</v>
       </c>
       <c r="E24" t="n" s="74">
-        <v>1.786347927E7</v>
+        <v>1.791129589E7</v>
       </c>
       <c r="F24" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G24" t="n" s="75">
-        <v>2.5122511E7</v>
+        <v>2.512764E7</v>
       </c>
     </row>
     <row r="25">
@@ -1916,16 +1916,16 @@
         <v>63</v>
       </c>
       <c r="D25" t="n" s="76">
-        <v>0.947442</v>
+        <v>0.948617</v>
       </c>
       <c r="E25" t="n" s="77">
-        <v>1.737751347E7</v>
+        <v>1.743098356E7</v>
       </c>
       <c r="F25" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G25" t="n" s="78">
-        <v>2.50380945E7</v>
+        <v>2.50432515E7</v>
       </c>
     </row>
     <row r="26">
@@ -1939,16 +1939,16 @@
         <v>65</v>
       </c>
       <c r="D26" t="n" s="79">
-        <v>0.904275</v>
+        <v>0.905534</v>
       </c>
       <c r="E26" t="n" s="80">
-        <v>1.658575853E7</v>
+        <v>1.663933099E7</v>
       </c>
       <c r="F26" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G26" t="n" s="81">
-        <v>2.49014965E7</v>
+        <v>2.4906702E7</v>
       </c>
     </row>
     <row r="27">
@@ -1962,16 +1962,16 @@
         <v>67</v>
       </c>
       <c r="D27" t="n" s="82">
-        <v>0.746728</v>
+        <v>0.74785</v>
       </c>
       <c r="E27" t="n" s="83">
-        <v>1.369612373E7</v>
+        <v>1.374185573E7</v>
       </c>
       <c r="F27" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G27" t="n" s="84">
-        <v>2.8510389E7</v>
+        <v>2.8516314E7</v>
       </c>
     </row>
     <row r="28">
@@ -1985,16 +1985,16 @@
         <v>69</v>
       </c>
       <c r="D28" t="n" s="85">
-        <v>0.746021</v>
+        <v>0.746826</v>
       </c>
       <c r="E28" t="n" s="86">
-        <v>1.368315803E7</v>
+        <v>1.372304101E7</v>
       </c>
       <c r="F28" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G28" t="n" s="87">
-        <v>1.96168816E7</v>
+        <v>1.9620768E7</v>
       </c>
     </row>
     <row r="29">
@@ -2008,16 +2008,16 @@
         <v>71</v>
       </c>
       <c r="D29" t="n" s="88">
-        <v>0.734796</v>
+        <v>0.735912</v>
       </c>
       <c r="E29" t="n" s="89">
-        <v>1.347726741E7</v>
+        <v>1.352248583E7</v>
       </c>
       <c r="F29" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G29" t="n" s="90">
-        <v>2.55493221E7</v>
+        <v>2.555461815E7</v>
       </c>
     </row>
     <row r="30">
@@ -2031,16 +2031,16 @@
         <v>73</v>
       </c>
       <c r="D30" t="n" s="91">
-        <v>0.622616</v>
+        <v>0.623469</v>
       </c>
       <c r="E30" t="n" s="92">
-        <v>1.141971739E7</v>
+        <v>1.145634252E7</v>
       </c>
       <c r="F30" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G30" t="n" s="93">
-        <v>2.31139125E7</v>
+        <v>2.31185847E7</v>
       </c>
     </row>
     <row r="31">
@@ -2054,16 +2054,16 @@
         <v>75</v>
       </c>
       <c r="D31" t="n" s="94">
-        <v>0.582851</v>
+        <v>0.583622</v>
       </c>
       <c r="E31" t="n" s="95">
-        <v>1.069035899E7</v>
+        <v>1.072414387E7</v>
       </c>
       <c r="F31" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G31" t="n" s="96">
-        <v>1.58886E7</v>
+        <v>1.5891759E7</v>
       </c>
     </row>
     <row r="32">
@@ -2077,16 +2077,16 @@
         <v>77</v>
       </c>
       <c r="D32" t="n" s="97">
-        <v>0.570885</v>
+        <v>0.57174</v>
       </c>
       <c r="E32" t="n" s="98">
-        <v>1.047088783E7</v>
+        <v>1.050581542E7</v>
       </c>
       <c r="F32" t="s" s="18">
         <v>21</v>
       </c>
       <c r="G32" t="n" s="99">
-        <v>1.580325E7</v>
+        <v>1.5806575E7</v>
       </c>
     </row>
     <row r="33">
@@ -2100,10 +2100,10 @@
         <v>79</v>
       </c>
       <c r="D33" t="n" s="100">
-        <v>0.26402</v>
+        <v>0.264092</v>
       </c>
       <c r="E33" t="n" s="101">
-        <v>4842523.99</v>
+        <v>4852735.37</v>
       </c>
       <c r="F33" t="s" s="18">
         <v>21</v>
@@ -2117,39 +2117,39 @@
         <v>80</v>
       </c>
       <c r="B34" t="s" s="18">
-        <v>21</v>
+        <v>81</v>
       </c>
       <c r="C34" t="s" s="18">
-        <v>21</v>
+        <v>82</v>
       </c>
       <c r="D34" t="n" s="103">
-        <v>0.162273</v>
+        <v>0.158494</v>
       </c>
       <c r="E34" t="n" s="104">
-        <v>2976323.37</v>
+        <v>1.744653231E8</v>
       </c>
       <c r="F34" t="n" s="105">
-        <v>4.1779656199E8</v>
+        <v>1.744653231E8</v>
       </c>
       <c r="G34" t="n" s="106">
-        <v>1138114.82</v>
+        <v>2.331E8</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s" s="18">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B35" t="s" s="18">
         <v>21</v>
       </c>
       <c r="C35" t="s" s="18">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D35" t="n" s="107">
-        <v>0.14745</v>
+        <v>0.147988</v>
       </c>
       <c r="E35" t="n" s="108">
-        <v>2704453.08</v>
+        <v>2719296.43</v>
       </c>
       <c r="F35" t="s" s="18">
         <v>21</v>
@@ -2160,88 +2160,88 @@
     </row>
     <row r="36">
       <c r="A36" t="s" s="18">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B36" t="s" s="18">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C36" t="s" s="18">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D36" t="n" s="110">
-        <v>0.13008</v>
+        <v>0.068492</v>
       </c>
       <c r="E36" t="n" s="111">
-        <v>1.738900731E8</v>
+        <v>6.910233418E7</v>
       </c>
       <c r="F36" t="n" s="112">
-        <v>1.738900731E8</v>
+        <v>6.910233418E7</v>
       </c>
       <c r="G36" t="n" s="113">
-        <v>2.331E8</v>
+        <v>11025.0</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s" s="18">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B37" t="s" s="18">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C37" t="s" s="18">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D37" t="n" s="114">
-        <v>0.049565</v>
+        <v>0.062648</v>
       </c>
       <c r="E37" t="n" s="115">
-        <v>6.873359176E7</v>
+        <v>3.372342119E8</v>
       </c>
       <c r="F37" t="n" s="116">
-        <v>6.873359176E7</v>
+        <v>3.372342119E8</v>
       </c>
       <c r="G37" t="n" s="117">
-        <v>11025.0</v>
+        <v>2.474E8</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s" s="18">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B38" t="s" s="18">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C38" t="s" s="18">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="D38" t="n" s="118">
-        <v>0.016051</v>
+        <v>0.008667</v>
       </c>
       <c r="E38" t="n" s="119">
-        <v>3.3567025284E8</v>
+        <v>8.740144459E7</v>
       </c>
       <c r="F38" t="n" s="120">
-        <v>3.3567025284E8</v>
+        <v>8.740144459E7</v>
       </c>
       <c r="G38" t="n" s="121">
-        <v>2.474E8</v>
+        <v>3420000.0</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s" s="18">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B39" t="s" s="18">
         <v>21</v>
       </c>
       <c r="C39" t="s" s="18">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D39" t="n" s="122">
         <v>0.0</v>
       </c>
       <c r="E39" t="n" s="123">
-        <v>7.54</v>
+        <v>7.57</v>
       </c>
       <c r="F39" t="s" s="18">
         <v>21</v>
@@ -2252,71 +2252,71 @@
     </row>
     <row r="40">
       <c r="A40" t="s" s="18">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B40" t="s" s="18">
         <v>21</v>
       </c>
       <c r="C40" t="s" s="18">
-        <v>95</v>
+        <v>21</v>
       </c>
       <c r="D40" t="n" s="125">
-        <v>-0.006828</v>
+        <v>-0.002395</v>
       </c>
       <c r="E40" t="n" s="126">
-        <v>-125232.98</v>
-      </c>
-      <c r="F40" t="s" s="18">
-        <v>21</v>
-      </c>
-      <c r="G40" t="n" s="127">
-        <v>-177976.22</v>
+        <v>-44005.76</v>
+      </c>
+      <c r="F40" t="n" s="127">
+        <v>4.1779656199E8</v>
+      </c>
+      <c r="G40" t="n" s="128">
+        <v>1138114.82</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s" s="18">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B41" t="s" s="18">
         <v>21</v>
       </c>
       <c r="C41" t="s" s="18">
-        <v>97</v>
-      </c>
-      <c r="D41" t="n" s="128">
-        <v>-0.007725</v>
-      </c>
-      <c r="E41" t="n" s="129">
-        <v>-141696.88</v>
+        <v>98</v>
+      </c>
+      <c r="D41" t="n" s="129">
+        <v>-0.006817</v>
+      </c>
+      <c r="E41" t="n" s="130">
+        <v>-125268.59</v>
       </c>
       <c r="F41" t="s" s="18">
         <v>21</v>
       </c>
-      <c r="G41" t="n" s="130">
-        <v>-2.2420698E7</v>
+      <c r="G41" t="n" s="131">
+        <v>-177976.22</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s" s="18">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B42" t="s" s="18">
-        <v>99</v>
+        <v>21</v>
       </c>
       <c r="C42" t="s" s="18">
         <v>100</v>
       </c>
-      <c r="D42" t="n" s="131">
-        <v>-0.022317</v>
-      </c>
-      <c r="E42" t="n" s="132">
-        <v>7.212601965E7</v>
-      </c>
-      <c r="F42" t="n" s="133">
-        <v>7.212601965E7</v>
+      <c r="D42" t="n" s="132">
+        <v>-0.007731</v>
+      </c>
+      <c r="E42" t="n" s="133">
+        <v>-142056.0</v>
+      </c>
+      <c r="F42" t="s" s="18">
+        <v>21</v>
       </c>
       <c r="G42" t="n" s="134">
-        <v>5060.0</v>
+        <v>-2.2420698E7</v>
       </c>
     </row>
     <row r="43">
@@ -2330,16 +2330,16 @@
         <v>103</v>
       </c>
       <c r="D43" t="n" s="135">
-        <v>-0.036119</v>
+        <v>-0.009878</v>
       </c>
       <c r="E43" t="n" s="136">
-        <v>8.635916072E7</v>
+        <v>7.275196022E7</v>
       </c>
       <c r="F43" t="n" s="137">
-        <v>8.635916072E7</v>
+        <v>7.275196022E7</v>
       </c>
       <c r="G43" t="n" s="138">
-        <v>3420000.0</v>
+        <v>5060.0</v>
       </c>
     </row>
     <row r="44">
@@ -2353,13 +2353,13 @@
         <v>106</v>
       </c>
       <c r="D44" t="n" s="139">
-        <v>-0.08037</v>
+        <v>-0.045309</v>
       </c>
       <c r="E44" t="n" s="140">
-        <v>1.1942749295E8</v>
+        <v>1.2073260073E8</v>
       </c>
       <c r="F44" t="n" s="141">
-        <v>1.1942749295E8</v>
+        <v>1.2073260073E8</v>
       </c>
       <c r="G44" t="n" s="142">
         <v>1.056E8</v>
@@ -2376,13 +2376,13 @@
         <v>109</v>
       </c>
       <c r="D45" t="n" s="143">
-        <v>-0.122684</v>
+        <v>-0.06287</v>
       </c>
       <c r="E45" t="n" s="144">
-        <v>1.7395151642E8</v>
+        <v>1.7541803739E8</v>
       </c>
       <c r="F45" t="n" s="145">
-        <v>1.7395151642E8</v>
+        <v>1.7541803739E8</v>
       </c>
       <c r="G45" t="n" s="146">
         <v>25260.0</v>
@@ -2399,13 +2399,13 @@
         <v>112</v>
       </c>
       <c r="D46" t="n" s="147">
-        <v>-0.229362</v>
+        <v>-0.1719</v>
       </c>
       <c r="E46" t="n" s="148">
-        <v>2.1061775E8</v>
+        <v>2.1166590625E8</v>
       </c>
       <c r="F46" t="n" s="149">
-        <v>2.1061775E8</v>
+        <v>2.1166590625E8</v>
       </c>
       <c r="G46" t="n" s="150">
         <v>1.973E8</v>
@@ -2422,13 +2422,13 @@
         <v>115</v>
       </c>
       <c r="D47" t="n" s="151">
-        <v>-0.507639</v>
+        <v>-0.417276</v>
       </c>
       <c r="E47" t="n" s="152">
-        <v>4.4508745313E8</v>
+        <v>4.467308125E8</v>
       </c>
       <c r="F47" t="n" s="153">
-        <v>4.4508745313E8</v>
+        <v>4.467308125E8</v>
       </c>
       <c r="G47" t="n" s="154">
         <v>4.207E8</v>
@@ -2445,13 +2445,13 @@
         <v>118</v>
       </c>
       <c r="D48" t="n" s="155">
-        <v>-0.703423</v>
+        <v>-0.750615</v>
       </c>
       <c r="E48" t="n" s="156">
-        <v>1.7867556E8</v>
+        <v>1.7778474E8</v>
       </c>
       <c r="F48" t="n" s="157">
-        <v>1.7867556E8</v>
+        <v>1.7778474E8</v>
       </c>
       <c r="G48" t="n" s="158">
         <v>44100.0</v>

</xml_diff>